<commit_message>
Calculator: cap on available users, treatment share input, months-to-power
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ygiEd3g3fKiFCARJZcKLp
</commit_message>
<xml_diff>
--- a/calculadora-sample-size.xlsx
+++ b/calculadora-sample-size.xlsx
@@ -22,12 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="107">
   <si>
     <t xml:space="preserve">Calculadora de sample size y poder: experimento de crédito por score</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas azules con fondo amarillo = edítalas con tu data. Todo lo demás son fórmulas. Los valores actuales son EJEMPLOS, reemplázalos.</t>
+    <t xml:space="preserve">Celdas azules con fondo amarillo = edítalas con tu data. Todo lo demás son fórmulas. Los valores actuales son EJEMPLOS, reemplázalos. El cálculo nunca usa más usuarios que tu tope.</t>
   </si>
   <si>
     <t xml:space="preserve">PARÁMETROS GENERALES</t>
@@ -45,10 +45,10 @@
     <t xml:space="preserve">Estándar 0.05.</t>
   </si>
   <si>
-    <t xml:space="preserve">Poder estadístico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estándar 0.80 (80% de detectar un efecto real).</t>
+    <t xml:space="preserve">Poder estadístico objetivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estándar 0.80 (80% de probabilidad de detectar un efecto real).</t>
   </si>
   <si>
     <t xml:space="preserve">Número de comparaciones (tiers probados)</t>
@@ -57,10 +57,10 @@
     <t xml:space="preserve">3 si pruebas Excelente, Bueno y Bajo. Pon 1 si pruebas solo uno.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pérdidas / inactivos extra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se suma a n para cubrir quienes no activan o salen. Ej. 5%.</t>
+    <t xml:space="preserve">Pérdidas / inactivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se descuenta de tus usuarios (los que no activan o salen). Ej. 5%.</t>
   </si>
   <si>
     <t xml:space="preserve">Alpha ajustado (Bonferroni)</t>
@@ -72,7 +72,7 @@
     <t xml:space="preserve">z de alpha</t>
   </si>
   <si>
-    <t xml:space="preserve">Valor crítico de la normal para el alpha ajustado (dos colas).</t>
+    <t xml:space="preserve">Valor crítico de la normal (dos colas).</t>
   </si>
   <si>
     <t xml:space="preserve">z de poder</t>
@@ -102,10 +102,16 @@
     <t xml:space="preserve">Lo que recibirá el tier en el experimento. Hoy todos tienen 500.</t>
   </si>
   <si>
-    <t xml:space="preserve">Referidores totales en el tier (pool)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Todos los referidores disponibles del tier. Se divide 50/50 entre tratamiento y control.</t>
+    <t xml:space="preserve">MÁXIMO de referidores disponibles en el tier (tope)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El máximo que de verdad existe. Todo se calcula con este tope, nunca con más.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% del tope que va a tratamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% = mitad tratamiento y mitad control (el más eficiente). El resto queda en control a 500 MXN. Usa entre 10% y 90%.</t>
   </si>
   <si>
     <t xml:space="preserve">Loans nuevos al mes del tier (con 500 MXN)</t>
@@ -117,7 +123,7 @@
     <t xml:space="preserve">Meses de ventana de medición</t>
   </si>
   <si>
-    <t xml:space="preserve">Cuánto tiempo mides a cada usuario. Más meses = tasa más alta = menos usuarios necesarios.</t>
+    <t xml:space="preserve">Cuánto tiempo mides a cada usuario. Más meses = tasa más alta = más poder.</t>
   </si>
   <si>
     <t xml:space="preserve">Lift relativo esperado entre quienes usan el crédito</t>
@@ -132,13 +138,13 @@
     <t xml:space="preserve">% de quienes reciben el crédito que realmente lo usa. Diluye el efecto.</t>
   </si>
   <si>
-    <t xml:space="preserve">RESULTADOS</t>
+    <t xml:space="preserve">RESULTADOS CON TU TOPE</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo leerlo</t>
   </si>
   <si>
-    <t xml:space="preserve">Tasa base mensual (loans / pool)</t>
+    <t xml:space="preserve">Tasa base mensual (loans / tope)</t>
   </si>
   <si>
     <t xml:space="preserve">Aproximación: asume 1 loan por referidor al mes.</t>
@@ -162,37 +168,19 @@
     <t xml:space="preserve">Tasa base ajustada por el lift efectivo.</t>
   </si>
   <si>
-    <t xml:space="preserve">n requerido por brazo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usuarios por brazo (tratamiento o control) para detectar el lift con el poder elegido.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n por brazo con pérdidas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n requerido más el margen de pérdidas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total de usuarios necesarios en el tier (2 brazos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lo que necesitas en el pool del tier.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disponible por brazo (pool / 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lo que tienes si divides el pool 50/50.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿Alcanza?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SÍ = tienes suficientes usuarios para el lift esperado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poder real con lo disponible</t>
+    <t xml:space="preserve">Usuarios efectivos en tratamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tope × % tratamiento, menos pérdidas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usuarios efectivos en control (500 MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tope × % control, menos pérdidas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PODER real con tu tope</t>
   </si>
   <si>
     <t xml:space="preserve">Probabilidad de detectar el lift esperado con tus usuarios. Busca 80% o más.</t>
@@ -201,13 +189,46 @@
     <t xml:space="preserve">Efecto mínimo detectable relativo (todo el grupo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Con lo disponible, solo detectas cambios de este tamaño o mayores en la tasa base.</t>
+    <t xml:space="preserve">Con tu tope solo detectas cambios de este tamaño o mayores en la tasa base.</t>
   </si>
   <si>
     <t xml:space="preserve">Efecto mínimo detectable entre quienes usan el crédito</t>
   </si>
   <si>
-    <t xml:space="preserve">Lo mismo, pero corregido por take-up. Compáralo con el lift que esperas.</t>
+    <t xml:space="preserve">Lo mismo, corregido por take-up. Compáralo con el lift que esperas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Detecta el lift esperado?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SÍ = con tu tope llegas al poder objetivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFERENCIA: lo que necesitarías</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usuarios totales que harían falta (con pérdidas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para detectar el lift esperado con el poder objetivo y tu % de tratamiento. Es solo referencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cabe en tu tope?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compara lo necesario contra el máximo que tienes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meses de ventana para llegar al poder con tu tope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con tu tope y tu lift, cuántos meses mediría cada usuario para llegar a 80% (máx. 12). Asume meses independientes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recomendación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qué hacer con este tier.</t>
   </si>
   <si>
     <t xml:space="preserve">CÁLCULO AUXILIAR (no editar)</t>
@@ -216,16 +237,28 @@
     <t xml:space="preserve">Para qué sirve</t>
   </si>
   <si>
-    <t xml:space="preserve">Referidores por brazo disponibles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para calcular el efecto mínimo detectable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n efectivo por brazo (con pérdidas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disponible por brazo menos pérdidas.</t>
+    <t xml:space="preserve">k = tratamiento / control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Razón entre grupos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n efectivo tratamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tope × % tratamiento × (1 - pérdidas).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n efectivo control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tope × (1 - % tratamiento) × (1 - pérdidas).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasa combinada bajo H0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media ponderada de p1 y p2, para el error estándar.</t>
   </si>
   <si>
     <t xml:space="preserve">Iteración 0 del efecto mínimo (pp)</t>
@@ -237,9 +270,6 @@
     <t xml:space="preserve">Iteración 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Se refina con la varianza real de ambos brazos.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Iteración 2</t>
   </si>
   <si>
@@ -252,13 +282,19 @@
     <t xml:space="preserve">Converge en 4 pasos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Supuestos: prueba de dos proporciones, dos colas, 50/50 entre tratamiento y control, aproximación normal. La tasa base mensual asume 1 loan por referidor; si hay referidores con varios loans, la tasa real es menor. Tasa acumulada = 1-(1-p)^meses asume meses independientes (en la práctica es algo menor).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usuarios necesarios por brazo según tasa base y lift</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usa el alpha, poder y comparaciones de la hoja Calculadora. Edita los valores azules para cambiar la rejilla.</t>
+    <t xml:space="preserve">PODER POR MESES DE VENTANA (auxiliar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poder con tu tope si midieras cada usuario por N meses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuestos: prueba de dos proporciones, dos colas, aproximación normal, con grupos de tamaño distinto si cambias el % de tratamiento. La tasa base mensual asume 1 loan por referidor; si hay referidores con varios loans, la tasa real es menor. Tasa acumulada = 1-(1-p)^meses asume meses independientes (en la práctica es algo menor). Si tu tope de 10K es el TOTAL entre los 3 tiers y no por tier, divídelo entre los tiers en la fila del tope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usuarios necesarios por brazo según tasa base y lift (referencia, 50/50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usa el alpha, poder y comparaciones de la hoja Calculadora. Es solo referencia: compara contra tu tope. Edita los valores azules para cambiar la rejilla.</t>
   </si>
   <si>
     <t xml:space="preserve">Take-up para esta tabla</t>
@@ -282,22 +318,25 @@
     <t xml:space="preserve">2. Parámetros generales: deja alpha 0.05 y poder 0.80 salvo que tengas otra regla. Pon en comparaciones cuántos tiers pruebas (3 si Excelente, Bueno y Bajo).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Por tier: pool de referidores, loans nuevos al mes con 500 MXN, meses de ventana, lift esperado y take-up.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Lee la fila 'n por brazo con pérdidas' (cuántos necesitas) contra 'Disponible por brazo' (cuántos tienes). La fila '¿Alcanza?' lo resume.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Si dice NO, mira 'Efecto mínimo detectable' (lo más chico que sí verías) y prueba: más meses de ventana, menos tiers, o más pool.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. La hoja Tabla_n da una rejilla de referencia: usuarios por brazo para cada tasa base y lift.</t>
+    <t xml:space="preserve">3. Por tier: tu TOPE de referidores (el máximo que existe), el % que va a tratamiento, loans nuevos al mes con 500 MXN, meses de ventana, lift esperado y take-up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Lee primero 'PODER real con tu tope' y '¿Detecta el lift esperado?'. Esos números usan solo tus usuarios disponibles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Si dice NO, mira 'Efecto mínimo detectable' (lo más chico que sí verías con tu tope) y 'Meses de ventana para llegar al poder'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. 'Referencia: lo que necesitarías' es solo para comparar contra tu tope. Si no cabe, no lo persigas: alarga la ventana, prueba menos tiers o espera un lift mayor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. La hoja Tabla_n da una rejilla de referencia: usuarios por brazo para cada tasa base y lift (50/50).</t>
   </si>
   <si>
     <t xml:space="preserve">De dónde sale cada dato:</t>
   </si>
   <si>
-    <t xml:space="preserve">Pool: referidores activos del tier. Loans al mes: referidos con loan del tier en el último mes. Lift: tu hipótesis (qué mejora justificaría pagar más crédito).</t>
+    <t xml:space="preserve">Tope: referidores activos del tier. Loans al mes: referidos con loan del tier en el último mes. Lift: tu hipótesis (qué mejora justificaría pagar más crédito).</t>
   </si>
   <si>
     <t xml:space="preserve">Take-up: de los que reciben el crédito, % que realmente lo usa. Si no lo tienes, prueba 100%, 60% y 40% para ver la sensibilidad.</t>
@@ -395,7 +434,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -412,6 +451,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -464,7 +509,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -482,15 +527,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -514,11 +559,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -526,27 +571,51 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -558,6 +627,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -578,7 +651,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -599,6 +672,32 @@
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -633,7 +732,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9E1F2"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -851,12 +950,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1064,36 +1163,36 @@
       </c>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>1000</v>
+      <c r="B16" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0.5</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>1</v>
+      <c r="B17" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>100</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>31</v>
@@ -1104,14 +1203,14 @@
       <c r="A18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>-0.15</v>
+      <c r="B18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>33</v>
@@ -1123,13 +1222,13 @@
         <v>34</v>
       </c>
       <c r="B19" s="11" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>0.6</v>
+        <v>0.15</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>0.6</v>
+        <v>-0.15</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>35</v>
@@ -1137,48 +1236,45 @@
       <c r="F19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+      <c r="A20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>37</v>
+      </c>
       <c r="F20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="15" t="n">
-        <f aca="false">B16/B15</f>
-        <v>0.1</v>
-      </c>
-      <c r="C22" s="15" t="n">
-        <f aca="false">C16/C15</f>
-        <v>0.1</v>
-      </c>
-      <c r="D22" s="15" t="n">
-        <f aca="false">D16/D15</f>
-        <v>0.1</v>
-      </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="5" t="s">
         <v>39</v>
       </c>
       <c r="F22" s="2"/>
@@ -1188,16 +1284,16 @@
         <v>40</v>
       </c>
       <c r="B23" s="15" t="n">
-        <f aca="false">1-(1-B22)^B17</f>
-        <v>0.1</v>
+        <f aca="false">B17/B15</f>
+        <v>0.05</v>
       </c>
       <c r="C23" s="15" t="n">
-        <f aca="false">1-(1-C22)^C17</f>
-        <v>0.1</v>
+        <f aca="false">C17/C15</f>
+        <v>0.03</v>
       </c>
       <c r="D23" s="15" t="n">
-        <f aca="false">1-(1-D22)^D17</f>
-        <v>0.1</v>
+        <f aca="false">D17/D15</f>
+        <v>0.01</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>41</v>
@@ -1208,17 +1304,17 @@
       <c r="A24" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="16" t="n">
-        <f aca="false">B18*B19</f>
-        <v>0.18</v>
-      </c>
-      <c r="C24" s="16" t="n">
-        <f aca="false">C18*C19</f>
-        <v>0.09</v>
-      </c>
-      <c r="D24" s="16" t="n">
-        <f aca="false">D18*D19</f>
-        <v>-0.09</v>
+      <c r="B24" s="15" t="n">
+        <f aca="false">1-(1-B23)^B18</f>
+        <v>0.05</v>
+      </c>
+      <c r="C24" s="15" t="n">
+        <f aca="false">1-(1-C23)^C18</f>
+        <v>0.03</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <f aca="false">1-(1-D23)^D18</f>
+        <v>0.01</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>43</v>
@@ -1229,17 +1325,17 @@
       <c r="A25" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="15" t="n">
-        <f aca="false">B23*(1+B24)</f>
-        <v>0.118</v>
-      </c>
-      <c r="C25" s="15" t="n">
-        <f aca="false">C23*(1+C24)</f>
-        <v>0.109</v>
-      </c>
-      <c r="D25" s="15" t="n">
-        <f aca="false">D23*(1+D24)</f>
-        <v>0.091</v>
+      <c r="B25" s="16" t="n">
+        <f aca="false">B19*B20</f>
+        <v>0.18</v>
+      </c>
+      <c r="C25" s="16" t="n">
+        <f aca="false">C19*C20</f>
+        <v>0.09</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <f aca="false">D19*D20</f>
+        <v>-0.09</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>45</v>
@@ -1250,17 +1346,17 @@
       <c r="A26" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="17" t="n">
-        <f aca="false">IF(B24=0,"n/a",ROUNDUP((($B$10*SQRT(2*((B23+B25)/2)*(1-(B23+B25)/2))+$B$11*SQRT(B23*(1-B23)+B25*(1-B25)))^2)/(B25-B23)^2,0))</f>
-        <v>6275</v>
-      </c>
-      <c r="C26" s="17" t="n">
-        <f aca="false">IF(C24=0,"n/a",ROUNDUP((($B$10*SQRT(2*((C23+C25)/2)*(1-(C23+C25)/2))+$B$11*SQRT(C23*(1-C23)+C25*(1-C25)))^2)/(C25-C23)^2,0))</f>
-        <v>24189</v>
-      </c>
-      <c r="D26" s="17" t="n">
-        <f aca="false">IF(D24=0,"n/a",ROUNDUP((($B$10*SQRT(2*((D23+D25)/2)*(1-(D23+D25)/2))+$B$11*SQRT(D23*(1-D23)+D25*(1-D25)))^2)/(D25-D23)^2,0))</f>
-        <v>22328</v>
+      <c r="B26" s="15" t="n">
+        <f aca="false">B24*(1+B25)</f>
+        <v>0.0590000000000001</v>
+      </c>
+      <c r="C26" s="15" t="n">
+        <f aca="false">C24*(1+C25)</f>
+        <v>0.0327</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <f aca="false">D24*(1+D25)</f>
+        <v>0.00910000000000001</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>47</v>
@@ -1271,17 +1367,17 @@
       <c r="A27" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B27" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(B26),ROUNDUP(B26/(1-$B$8),0),"n/a")</f>
-        <v>6606</v>
-      </c>
-      <c r="C27" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(C26),ROUNDUP(C26/(1-$B$8),0),"n/a")</f>
-        <v>25463</v>
-      </c>
-      <c r="D27" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(D26),ROUNDUP(D26/(1-$B$8),0),"n/a")</f>
-        <v>23504</v>
+      <c r="B27" s="17" t="n">
+        <f aca="false">B43</f>
+        <v>4750</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <f aca="false">C43</f>
+        <v>4750</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <f aca="false">D43</f>
+        <v>4750</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>49</v>
@@ -1293,16 +1389,16 @@
         <v>50</v>
       </c>
       <c r="B28" s="17" t="n">
-        <f aca="false">IF(ISNUMBER(B27),B27*2,"n/a")</f>
-        <v>13212</v>
+        <f aca="false">B44</f>
+        <v>4750</v>
       </c>
       <c r="C28" s="17" t="n">
-        <f aca="false">IF(ISNUMBER(C27),C27*2,"n/a")</f>
-        <v>50926</v>
+        <f aca="false">C44</f>
+        <v>4750</v>
       </c>
       <c r="D28" s="17" t="n">
-        <f aca="false">IF(ISNUMBER(D27),D27*2,"n/a")</f>
-        <v>47008</v>
+        <f aca="false">D44</f>
+        <v>4750</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>51</v>
@@ -1314,16 +1410,16 @@
         <v>52</v>
       </c>
       <c r="B29" s="18" t="n">
-        <f aca="false">B15/2</f>
-        <v>5000</v>
+        <f aca="false">NORMSDIST((ABS(B26-B24)-$B$10*SQRT(B45*(1-B45)*(1/B44+1/B43)))/SQRT(B24*(1-B24)/B44+B26*(1-B26)/B43))</f>
+        <v>0.322076256263711</v>
       </c>
       <c r="C29" s="18" t="n">
-        <f aca="false">C15/2</f>
-        <v>5000</v>
+        <f aca="false">NORMSDIST((ABS(C26-C24)-$B$10*SQRT(C45*(1-C45)*(1/C44+1/C43)))/SQRT(C24*(1-C24)/C44+C26*(1-C26)/C43))</f>
+        <v>0.0506120133084721</v>
       </c>
       <c r="D29" s="18" t="n">
-        <f aca="false">D15/2</f>
-        <v>5000</v>
+        <f aca="false">NORMSDIST((ABS(D26-D24)-$B$10*SQRT(D45*(1-D45)*(1/D44+1/D43)))/SQRT(D24*(1-D24)/D44+D26*(1-D26)/D43))</f>
+        <v>0.0260067764439741</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>53</v>
@@ -1334,17 +1430,17 @@
       <c r="A30" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="19" t="str">
-        <f aca="false">IF(ISNUMBER(B27),IF(B29&gt;=B27,"SÍ","NO"),"n/a")</f>
-        <v>NO</v>
-      </c>
-      <c r="C30" s="19" t="str">
-        <f aca="false">IF(ISNUMBER(C27),IF(C29&gt;=C27,"SÍ","NO"),"n/a")</f>
-        <v>NO</v>
-      </c>
-      <c r="D30" s="19" t="str">
-        <f aca="false">IF(ISNUMBER(D27),IF(D29&gt;=D27,"SÍ","NO"),"n/a")</f>
-        <v>NO</v>
+      <c r="B30" s="16" t="n">
+        <f aca="false">B50/B24</f>
+        <v>0.309686211710248</v>
+      </c>
+      <c r="C30" s="16" t="n">
+        <f aca="false">C50/C24</f>
+        <v>0.413318181612153</v>
+      </c>
+      <c r="D30" s="16" t="n">
+        <f aca="false">D50/D24</f>
+        <v>0.776701739625666</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>55</v>
@@ -1355,38 +1451,38 @@
       <c r="A31" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="20" t="n">
-        <f aca="false">NORMSDIST((ABS(B25-B23)*SQRT(B38)-$B$10*SQRT(2*((B23+B25)/2)*(1-(B23+B25)/2)))/SQRT(B23*(1-B23)+B25*(1-B25)))</f>
-        <v>0.663131977553076</v>
-      </c>
-      <c r="C31" s="20" t="n">
-        <f aca="false">NORMSDIST((ABS(C25-C23)*SQRT(C38)-$B$10*SQRT(2*((C23+C25)/2)*(1-(C23+C25)/2)))/SQRT(C23*(1-C23)+C25*(1-C25)))</f>
-        <v>0.168451905196954</v>
-      </c>
-      <c r="D31" s="20" t="n">
-        <f aca="false">NORMSDIST((ABS(D25-D23)*SQRT(D38)-$B$10*SQRT(2*((D23+D25)/2)*(1-(D23+D25)/2)))/SQRT(D23*(1-D23)+D25*(1-D25)))</f>
-        <v>0.183596553398769</v>
+      <c r="B31" s="16" t="n">
+        <f aca="false">B30/B20</f>
+        <v>0.516143686183747</v>
+      </c>
+      <c r="C31" s="16" t="n">
+        <f aca="false">C30/C20</f>
+        <v>0.688863636020255</v>
+      </c>
+      <c r="D31" s="16" t="n">
+        <f aca="false">D30/D20</f>
+        <v>1.29450289937611</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>57</v>
       </c>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B32" s="16" t="n">
-        <f aca="false">B43/B23</f>
-        <v>0.20803969230822</v>
-      </c>
-      <c r="C32" s="16" t="n">
-        <f aca="false">C43/C23</f>
-        <v>0.20803969230822</v>
-      </c>
-      <c r="D32" s="16" t="n">
-        <f aca="false">D43/D23</f>
-        <v>0.20803969230822</v>
+      <c r="B32" s="19" t="str">
+        <f aca="false">IF(B29&gt;=$B$6,"SÍ","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="C32" s="19" t="str">
+        <f aca="false">IF(C29&gt;=$B$6,"SÍ","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="D32" s="19" t="str">
+        <f aca="false">IF(D29&gt;=$B$6,"SÍ","NO")</f>
+        <v>NO</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>59</v>
@@ -1394,259 +1490,330 @@
       <c r="F32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="B33" s="16" t="n">
-        <f aca="false">B32/B19</f>
-        <v>0.3467328205137</v>
-      </c>
-      <c r="C33" s="16" t="n">
-        <f aca="false">C32/C19</f>
-        <v>0.3467328205137</v>
-      </c>
-      <c r="D33" s="16" t="n">
-        <f aca="false">D32/D19</f>
-        <v>0.3467328205137</v>
-      </c>
-      <c r="E33" s="8" t="s">
+      <c r="B33" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F33" s="2"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
+      <c r="B34" s="22" t="n">
+        <f aca="false">IF(B25=0,"n/a",ROUNDUP((((($B$10*SQRT(((B24+B42*B26)/(1+B42))*(1-((B24+B42*B26)/(1+B42)))*(1+1/B42))+$B$11*SQRT(B24*(1-B24)+B26*(1-B26)/B42))^2)/(B26-B24)^2)*(1+B42))/(1-$B$8),0))</f>
+        <v>28040</v>
+      </c>
+      <c r="C34" s="22" t="n">
+        <f aca="false">IF(C25=0,"n/a",ROUNDUP((((($B$10*SQRT(((C24+C42*C26)/(1+C42))*(1-((C24+C42*C26)/(1+C42)))*(1+1/C42))+$B$11*SQRT(C24*(1-C24)+C26*(1-C26)/C42))^2)/(C26-C24)^2)*(1+C42))/(1-$B$8),0))</f>
+        <v>183619</v>
+      </c>
+      <c r="D34" s="22" t="n">
+        <f aca="false">IF(D25=0,"n/a",ROUNDUP((((($B$10*SQRT(((D24+D42*D26)/(1+D42))*(1-((D24+D42*D26)/(1+D42)))*(1+1/D42))+$B$11*SQRT(D24*(1-D24)+D26*(1-D26)/D42))^2)/(D26-D24)^2)*(1+D42))/(1-$B$8),0))</f>
+        <v>514749</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="F34" s="2"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
+    <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="23" t="str">
+        <f aca="false">IF(ISNUMBER(B34),IF(B34&lt;=B15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(B34-B15,"#,##0")),"n/a")</f>
+        <v>No cabe: faltan 18,040</v>
+      </c>
+      <c r="C35" s="23" t="str">
+        <f aca="false">IF(ISNUMBER(C34),IF(C34&lt;=C15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(C34-C15,"#,##0")),"n/a")</f>
+        <v>No cabe: faltan 173,619</v>
+      </c>
+      <c r="D35" s="23" t="str">
+        <f aca="false">IF(ISNUMBER(D34),IF(D34&lt;=D15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(D34-D15,"#,##0")),"n/a")</f>
+        <v>No cabe: faltan 504,749</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="F35" s="2"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B36" s="5" t="s">
+    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B36" s="24" t="n">
+        <f aca="false">IF(COUNTIF(B54:B65,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(B54:B65,"&lt;"&amp;$B$6)+1)</f>
+        <v>3</v>
+      </c>
+      <c r="C36" s="24" t="str">
+        <f aca="false">IF(COUNTIF(C54:C65,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(C54:C65,"&lt;"&amp;$B$6)+1)</f>
+        <v>&gt;12</v>
+      </c>
+      <c r="D36" s="24" t="str">
+        <f aca="false">IF(COUNTIF(D54:D65,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(D54:D65,"&lt;"&amp;$B$6)+1)</f>
+        <v>&gt;12</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B37" s="19" t="str">
+        <f aca="false">IF(B32="SÍ","Corre el experimento con tu tope.",IF(ISNUMBER(B36),"Alarga la ventana a "&amp;B36&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
+        <v>Alarga la ventana a 3 meses.</v>
+      </c>
+      <c r="C37" s="19" t="str">
+        <f aca="false">IF(C32="SÍ","Corre el experimento con tu tope.",IF(ISNUMBER(C36),"Alarga la ventana a "&amp;C36&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
+        <v>No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor.</v>
+      </c>
+      <c r="D37" s="19" t="str">
+        <f aca="false">IF(D32="SÍ","Corre el experimento con tu tope.",IF(ISNUMBER(D36),"Alarga la ventana a "&amp;D36&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
+        <v>No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor.</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B41" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C41" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D41" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E36" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F36" s="2"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B37" s="18" t="n">
-        <f aca="false">B29</f>
-        <v>5000</v>
-      </c>
-      <c r="C37" s="18" t="n">
-        <f aca="false">C29</f>
-        <v>5000</v>
-      </c>
-      <c r="D37" s="18" t="n">
-        <f aca="false">D29</f>
-        <v>5000</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B38" s="18" t="n">
-        <f aca="false">B37*(1-$B$8)</f>
-        <v>4750</v>
-      </c>
-      <c r="C38" s="18" t="n">
-        <f aca="false">C37*(1-$B$8)</f>
-        <v>4750</v>
-      </c>
-      <c r="D38" s="18" t="n">
-        <f aca="false">D37*(1-$B$8)</f>
-        <v>4750</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F38" s="2"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B39" s="12" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(2*B23*(1-B23)/B38)</f>
-        <v>0.0199179396974637</v>
-      </c>
-      <c r="C39" s="12" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(2*C23*(1-C23)/C38)</f>
-        <v>0.0199179396974637</v>
-      </c>
-      <c r="D39" s="12" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(2*D23*(1-D23)/D38)</f>
-        <v>0.0199179396974637</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
+      <c r="E41" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B40" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(B23+B39/2)*(1-B23-B39/2))+$B$11*SQRT(B23*(1-B23)+(B23+B39)*(1-B23-B39)))/SQRT(B38)</f>
-        <v>0.020767596860278</v>
-      </c>
-      <c r="C40" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(C23+C39/2)*(1-C23-C39/2))+$B$11*SQRT(C23*(1-C23)+(C23+C39)*(1-C23-C39)))/SQRT(C38)</f>
-        <v>0.020767596860278</v>
-      </c>
-      <c r="D40" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(D23+D39/2)*(1-D23-D39/2))+$B$11*SQRT(D23*(1-D23)+(D23+D39)*(1-D23-D39)))/SQRT(D38)</f>
-        <v>0.020767596860278</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F40" s="2"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B41" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(B23+B40/2)*(1-B23-B40/2))+$B$11*SQRT(B23*(1-B23)+(B23+B40)*(1-B23-B40)))/SQRT(B38)</f>
-        <v>0.0208024806971357</v>
-      </c>
-      <c r="C41" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(C23+C40/2)*(1-C23-C40/2))+$B$11*SQRT(C23*(1-C23)+(C23+C40)*(1-C23-C40)))/SQRT(C38)</f>
-        <v>0.0208024806971357</v>
-      </c>
-      <c r="D41" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(D23+D40/2)*(1-D23-D40/2))+$B$11*SQRT(D23*(1-D23)+(D23+D40)*(1-D23-D40)))/SQRT(D38)</f>
-        <v>0.0208024806971357</v>
-      </c>
-      <c r="E41" s="2"/>
       <c r="F41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B42" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(B23+B41/2)*(1-B23-B41/2))+$B$11*SQRT(B23*(1-B23)+(B23+B41)*(1-B23-B41)))/SQRT(B38)</f>
-        <v>0.020803910620651</v>
-      </c>
-      <c r="C42" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(C23+C41/2)*(1-C23-C41/2))+$B$11*SQRT(C23*(1-C23)+(C23+C41)*(1-C23-C41)))/SQRT(C38)</f>
-        <v>0.020803910620651</v>
-      </c>
-      <c r="D42" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(D23+D41/2)*(1-D23-D41/2))+$B$11*SQRT(D23*(1-D23)+(D23+D41)*(1-D23-D41)))/SQRT(D38)</f>
-        <v>0.020803910620651</v>
-      </c>
-      <c r="E42" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="B42" s="25" t="n">
+        <f aca="false">B16/(1-B16)</f>
+        <v>1</v>
+      </c>
+      <c r="C42" s="25" t="n">
+        <f aca="false">C16/(1-C16)</f>
+        <v>1</v>
+      </c>
+      <c r="D42" s="25" t="n">
+        <f aca="false">D16/(1-D16)</f>
+        <v>1</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>72</v>
+      </c>
       <c r="F42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B43" s="17" t="n">
+        <f aca="false">B15*B16*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="C43" s="17" t="n">
+        <f aca="false">C15*C16*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="D43" s="17" t="n">
+        <f aca="false">D15*D16*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="E43" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B43" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(B23+B42/2)*(1-B23-B42/2))+$B$11*SQRT(B23*(1-B23)+(B23+B42)*(1-B23-B42)))/SQRT(B38)</f>
-        <v>0.020803969230822</v>
-      </c>
-      <c r="C43" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(C23+C42/2)*(1-C23-C42/2))+$B$11*SQRT(C23*(1-C23)+(C23+C42)*(1-C23-C42)))/SQRT(C38)</f>
-        <v>0.020803969230822</v>
-      </c>
-      <c r="D43" s="12" t="n">
-        <f aca="false">($B$10*SQRT(2*(D23+D42/2)*(1-D23-D42/2))+$B$11*SQRT(D23*(1-D23)+(D23+D42)*(1-D23-D42)))/SQRT(D38)</f>
-        <v>0.020803969230822</v>
-      </c>
-      <c r="E43" s="8" t="s">
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="F43" s="2"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
+      <c r="B44" s="17" t="n">
+        <f aca="false">B15*(1-B16)*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="C44" s="17" t="n">
+        <f aca="false">C15*(1-C16)*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="D44" s="17" t="n">
+        <f aca="false">D15*(1-D16)*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="F44" s="2"/>
     </row>
-    <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="B45" s="21"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B45" s="12" t="n">
+        <f aca="false">(B44*B24+B43*B26)/(B44+B43)</f>
+        <v>0.0545000000000001</v>
+      </c>
+      <c r="C45" s="12" t="n">
+        <f aca="false">(C44*C24+C43*C26)/(C44+C43)</f>
+        <v>0.03135</v>
+      </c>
+      <c r="D45" s="12" t="n">
+        <f aca="false">(D44*D24+D43*D26)/(D44+D43)</f>
+        <v>0.00955000000000001</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>78</v>
+      </c>
       <c r="F45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="21"/>
-      <c r="B46" s="21"/>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
+      <c r="A46" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B46" s="12" t="n">
+        <f aca="false">($B$10+$B$11)*SQRT(B24*(1-B24)*(1/B44+1/B43))</f>
+        <v>0.0144700477174636</v>
+      </c>
+      <c r="C46" s="12" t="n">
+        <f aca="false">($B$10+$B$11)*SQRT(C24*(1-C24)*(1/C44+1/C43))</f>
+        <v>0.0113258199429158</v>
+      </c>
+      <c r="D46" s="12" t="n">
+        <f aca="false">($B$10+$B$11)*SQRT(D24*(1-D24)*(1/D44+1/D43))</f>
+        <v>0.00660603325734122</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="F46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
+      <c r="A47" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B47" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B46))/(B44+B43))*(1-((B44*B24+B43*(B24+B46))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B46)*(1-B24-B46)/B43)</f>
+        <v>0.0154205904175831</v>
+      </c>
+      <c r="C47" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C46))/(C44+C43))*(1-((C44*C24+C43*(C24+C46))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C46)*(1-C24-C46)/C43)</f>
+        <v>0.0123109990740818</v>
+      </c>
+      <c r="D47" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D46))/(D44+D43))*(1-((D44*D24+D43*(D24+D46))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D46)*(1-D24-D46)/D43)</f>
+        <v>0.00760576962692852</v>
+      </c>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
+      <c r="A48" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B47))/(B44+B43))*(1-((B44*B24+B43*(B24+B47))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B47)*(1-B24-B47)/B43)</f>
+        <v>0.0154803316438639</v>
+      </c>
+      <c r="C48" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C47))/(C44+C43))*(1-((C44*C24+C43*(C24+C47))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C47)*(1-C24-C47)/C43)</f>
+        <v>0.012392313574853</v>
+      </c>
+      <c r="D48" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D47))/(D44+D43))*(1-((D44*D24+D43*(D24+D47))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D47)*(1-D24-D47)/D43)</f>
+        <v>0.00774515165979732</v>
+      </c>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
+      <c r="A49" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B49" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B48))/(B44+B43))*(1-((B44*B24+B43*(B24+B48))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B48)*(1-B24-B48)/B43)</f>
+        <v>0.015484075950343</v>
+      </c>
+      <c r="C49" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C48))/(C44+C43))*(1-((C44*C24+C43*(C24+C48))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C48)*(1-C24-C48)/C43)</f>
+        <v>0.0123989964120841</v>
+      </c>
+      <c r="D49" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D48))/(D44+D43))*(1-((D44*D24+D43*(D24+D48))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D48)*(1-D24-D48)/D43)</f>
+        <v>0.00776437119734043</v>
+      </c>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
+      <c r="A50" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B50" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B49))/(B44+B43))*(1-((B44*B24+B43*(B24+B49))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B49)*(1-B24-B49)/B43)</f>
+        <v>0.0154843105855124</v>
+      </c>
+      <c r="C50" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C49))/(C44+C43))*(1-((C44*C24+C43*(C24+C49))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C49)*(1-C24-C49)/C43)</f>
+        <v>0.0123995454483646</v>
+      </c>
+      <c r="D50" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D49))/(D44+D43))*(1-((D44*D24+D43*(D24+D49))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D49)*(1-D24-D49)/D43)</f>
+        <v>0.00776701739625667</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>85</v>
+      </c>
       <c r="F50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1658,11 +1825,21 @@
       <c r="F51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
+      <c r="A52" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B52" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D52" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E52" s="21" t="s">
+        <v>87</v>
+      </c>
       <c r="F52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1674,71 +1851,293 @@
       <c r="F53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
+      <c r="A54" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A54)*(1+B$25),0.999)-(1-(1-B$23)^$A54))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A54)+B$43*MIN((1-(1-B$23)^$A54)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A54)+B$43*MIN((1-(1-B$23)^$A54)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A54)*(1-(1-(1-B$23)^$A54))/B$44+MIN((1-(1-B$23)^$A54)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A54)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.322076256263711</v>
+      </c>
+      <c r="C54" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A54)*(1+C$25),0.999)-(1-(1-C$23)^$A54))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A54)+C$43*MIN((1-(1-C$23)^$A54)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A54)+C$43*MIN((1-(1-C$23)^$A54)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A54)*(1-(1-(1-C$23)^$A54))/C$44+MIN((1-(1-C$23)^$A54)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A54)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.0506120133084721</v>
+      </c>
+      <c r="D54" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A54)*(1+D$25),0.999)-(1-(1-D$23)^$A54))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A54)+D$43*MIN((1-(1-D$23)^$A54)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A54)+D$43*MIN((1-(1-D$23)^$A54)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A54)*(1-(1-(1-D$23)^$A54))/D$44+MIN((1-(1-D$23)^$A54)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A54)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.0260067764439741</v>
+      </c>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
+      <c r="A55" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A55)*(1+B$25),0.999)-(1-(1-B$23)^$A55))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A55)+B$43*MIN((1-(1-B$23)^$A55)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A55)+B$43*MIN((1-(1-B$23)^$A55)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A55)*(1-(1-(1-B$23)^$A55))/B$44+MIN((1-(1-B$23)^$A55)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A55)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.648530625309196</v>
+      </c>
+      <c r="C55" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A55)*(1+C$25),0.999)-(1-(1-C$23)^$A55))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A55)+C$43*MIN((1-(1-C$23)^$A55)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A55)+C$43*MIN((1-(1-C$23)^$A55)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A55)*(1-(1-(1-C$23)^$A55))/C$44+MIN((1-(1-C$23)^$A55)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A55)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.0938830966435802</v>
+      </c>
+      <c r="D55" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A55)*(1+D$25),0.999)-(1-(1-D$23)^$A55))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A55)+D$43*MIN((1-(1-D$23)^$A55)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A55)+D$43*MIN((1-(1-D$23)^$A55)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A55)*(1-(1-(1-D$23)^$A55))/D$44+MIN((1-(1-D$23)^$A55)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A55)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.039648899805351</v>
+      </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
+      <c r="A56" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B56" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A56)*(1+B$25),0.999)-(1-(1-B$23)^$A56))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A56)+B$43*MIN((1-(1-B$23)^$A56)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A56)+B$43*MIN((1-(1-B$23)^$A56)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A56)*(1-(1-(1-B$23)^$A56))/B$44+MIN((1-(1-B$23)^$A56)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A56)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.855324473869813</v>
+      </c>
+      <c r="C56" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A56)*(1+C$25),0.999)-(1-(1-C$23)^$A56))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A56)+C$43*MIN((1-(1-C$23)^$A56)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A56)+C$43*MIN((1-(1-C$23)^$A56)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A56)*(1-(1-(1-C$23)^$A56))/C$44+MIN((1-(1-C$23)^$A56)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A56)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.143659104798111</v>
+      </c>
+      <c r="D56" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A56)*(1+D$25),0.999)-(1-(1-D$23)^$A56))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A56)+D$43*MIN((1-(1-D$23)^$A56)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A56)+D$43*MIN((1-(1-D$23)^$A56)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A56)*(1-(1-(1-D$23)^$A56))/D$44+MIN((1-(1-D$23)^$A56)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A56)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.0537724436545908</v>
+      </c>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
+      <c r="A57" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B57" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A57)*(1+B$25),0.999)-(1-(1-B$23)^$A57))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A57)+B$43*MIN((1-(1-B$23)^$A57)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A57)+B$43*MIN((1-(1-B$23)^$A57)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A57)*(1-(1-(1-B$23)^$A57))/B$44+MIN((1-(1-B$23)^$A57)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A57)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.951427708514472</v>
+      </c>
+      <c r="C57" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A57)*(1+C$25),0.999)-(1-(1-C$23)^$A57))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A57)+C$43*MIN((1-(1-C$23)^$A57)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A57)+C$43*MIN((1-(1-C$23)^$A57)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A57)*(1-(1-(1-C$23)^$A57))/C$44+MIN((1-(1-C$23)^$A57)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A57)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.199017743143467</v>
+      </c>
+      <c r="D57" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A57)*(1+D$25),0.999)-(1-(1-D$23)^$A57))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A57)+D$43*MIN((1-(1-D$23)^$A57)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A57)+D$43*MIN((1-(1-D$23)^$A57)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A57)*(1-(1-(1-D$23)^$A57))/D$44+MIN((1-(1-D$23)^$A57)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A57)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.0686574926403583</v>
+      </c>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
+      <c r="A58" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B58" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A58)*(1+B$25),0.999)-(1-(1-B$23)^$A58))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A58)+B$43*MIN((1-(1-B$23)^$A58)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A58)+B$43*MIN((1-(1-B$23)^$A58)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A58)*(1-(1-(1-B$23)^$A58))/B$44+MIN((1-(1-B$23)^$A58)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A58)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.986534104343037</v>
+      </c>
+      <c r="C58" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A58)*(1+C$25),0.999)-(1-(1-C$23)^$A58))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A58)+C$43*MIN((1-(1-C$23)^$A58)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A58)+C$43*MIN((1-(1-C$23)^$A58)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A58)*(1-(1-(1-C$23)^$A58))/C$44+MIN((1-(1-C$23)^$A58)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A58)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.258692789591655</v>
+      </c>
+      <c r="D58" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A58)*(1+D$25),0.999)-(1-(1-D$23)^$A58))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A58)+D$43*MIN((1-(1-D$23)^$A58)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A58)+D$43*MIN((1-(1-D$23)^$A58)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A58)*(1-(1-(1-D$23)^$A58))/D$44+MIN((1-(1-D$23)^$A58)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A58)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.084357351243645</v>
+      </c>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
+      <c r="A59" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B59" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A59)*(1+B$25),0.999)-(1-(1-B$23)^$A59))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A59)+B$43*MIN((1-(1-B$23)^$A59)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A59)+B$43*MIN((1-(1-B$23)^$A59)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A59)*(1-(1-(1-B$23)^$A59))/B$44+MIN((1-(1-B$23)^$A59)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A59)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.996905244060923</v>
+      </c>
+      <c r="C59" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A59)*(1+C$25),0.999)-(1-(1-C$23)^$A59))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A59)+C$43*MIN((1-(1-C$23)^$A59)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A59)+C$43*MIN((1-(1-C$23)^$A59)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A59)*(1-(1-(1-C$23)^$A59))/C$44+MIN((1-(1-C$23)^$A59)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A59)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.321309020930109</v>
+      </c>
+      <c r="D59" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A59)*(1+D$25),0.999)-(1-(1-D$23)^$A59))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A59)+D$43*MIN((1-(1-D$23)^$A59)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A59)+D$43*MIN((1-(1-D$23)^$A59)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A59)*(1-(1-(1-D$23)^$A59))/D$44+MIN((1-(1-D$23)^$A59)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A59)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.10086207082924</v>
+      </c>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
+      <c r="A60" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="B60" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A60)*(1+B$25),0.999)-(1-(1-B$23)^$A60))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A60)+B$43*MIN((1-(1-B$23)^$A60)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A60)+B$43*MIN((1-(1-B$23)^$A60)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A60)*(1-(1-(1-B$23)^$A60))/B$44+MIN((1-(1-B$23)^$A60)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A60)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.999411332147072</v>
+      </c>
+      <c r="C60" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A60)*(1+C$25),0.999)-(1-(1-C$23)^$A60))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A60)+C$43*MIN((1-(1-C$23)^$A60)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A60)+C$43*MIN((1-(1-C$23)^$A60)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A60)*(1-(1-(1-C$23)^$A60))/C$44+MIN((1-(1-C$23)^$A60)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A60)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.385471506279525</v>
+      </c>
+      <c r="D60" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A60)*(1+D$25),0.999)-(1-(1-D$23)^$A60))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A60)+D$43*MIN((1-(1-D$23)^$A60)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A60)+D$43*MIN((1-(1-D$23)^$A60)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A60)*(1-(1-(1-D$23)^$A60))/D$44+MIN((1-(1-D$23)^$A60)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A60)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.118136637139437</v>
+      </c>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
     </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B61" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A61)*(1+B$25),0.999)-(1-(1-B$23)^$A61))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A61)+B$43*MIN((1-(1-B$23)^$A61)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A61)+B$43*MIN((1-(1-B$23)^$A61)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A61)*(1-(1-(1-B$23)^$A61))/B$44+MIN((1-(1-B$23)^$A61)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A61)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.999907837749006</v>
+      </c>
+      <c r="C61" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A61)*(1+C$25),0.999)-(1-(1-C$23)^$A61))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A61)+C$43*MIN((1-(1-C$23)^$A61)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A61)+C$43*MIN((1-(1-C$23)^$A61)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A61)*(1-(1-(1-C$23)^$A61))/C$44+MIN((1-(1-C$23)^$A61)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A61)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.449827485387897</v>
+      </c>
+      <c r="D61" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A61)*(1+D$25),0.999)-(1-(1-D$23)^$A61))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A61)+D$43*MIN((1-(1-D$23)^$A61)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A61)+D$43*MIN((1-(1-D$23)^$A61)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A61)*(1-(1-(1-D$23)^$A61))/D$44+MIN((1-(1-D$23)^$A61)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A61)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.13613395893133</v>
+      </c>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B62" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A62)*(1+B$25),0.999)-(1-(1-B$23)^$A62))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A62)+B$43*MIN((1-(1-B$23)^$A62)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A62)+B$43*MIN((1-(1-B$23)^$A62)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A62)*(1-(1-(1-B$23)^$A62))/B$44+MIN((1-(1-B$23)^$A62)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A62)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.999988227140586</v>
+      </c>
+      <c r="C62" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A62)*(1+C$25),0.999)-(1-(1-C$23)^$A62))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A62)+C$43*MIN((1-(1-C$23)^$A62)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A62)+C$43*MIN((1-(1-C$23)^$A62)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A62)*(1-(1-(1-C$23)^$A62))/C$44+MIN((1-(1-C$23)^$A62)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A62)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.513116896204362</v>
+      </c>
+      <c r="D62" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A62)*(1+D$25),0.999)-(1-(1-D$23)^$A62))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A62)+D$43*MIN((1-(1-D$23)^$A62)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A62)+D$43*MIN((1-(1-D$23)^$A62)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A62)*(1-(1-(1-D$23)^$A62))/D$44+MIN((1-(1-D$23)^$A62)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A62)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.15480036499496</v>
+      </c>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="B63" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A63)*(1+B$25),0.999)-(1-(1-B$23)^$A63))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A63)+B$43*MIN((1-(1-B$23)^$A63)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A63)+B$43*MIN((1-(1-B$23)^$A63)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A63)*(1-(1-(1-B$23)^$A63))/B$44+MIN((1-(1-B$23)^$A63)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A63)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.999998787016377</v>
+      </c>
+      <c r="C63" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A63)*(1+C$25),0.999)-(1-(1-C$23)^$A63))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A63)+C$43*MIN((1-(1-C$23)^$A63)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A63)+C$43*MIN((1-(1-C$23)^$A63)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A63)*(1-(1-(1-C$23)^$A63))/C$44+MIN((1-(1-C$23)^$A63)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A63)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.574213765368228</v>
+      </c>
+      <c r="D63" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A63)*(1+D$25),0.999)-(1-(1-D$23)^$A63))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A63)+D$43*MIN((1-(1-D$23)^$A63)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A63)+D$43*MIN((1-(1-D$23)^$A63)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A63)*(1-(1-(1-D$23)^$A63))/D$44+MIN((1-(1-D$23)^$A63)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A63)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.174078332095706</v>
+      </c>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B64" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A64)*(1+B$25),0.999)-(1-(1-B$23)^$A64))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A64)+B$43*MIN((1-(1-B$23)^$A64)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A64)+B$43*MIN((1-(1-B$23)^$A64)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A64)*(1-(1-(1-B$23)^$A64))/B$44+MIN((1-(1-B$23)^$A64)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A64)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.999999900613897</v>
+      </c>
+      <c r="C64" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A64)*(1+C$25),0.999)-(1-(1-C$23)^$A64))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A64)+C$43*MIN((1-(1-C$23)^$A64)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A64)+C$43*MIN((1-(1-C$23)^$A64)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A64)*(1-(1-(1-C$23)^$A64))/C$44+MIN((1-(1-C$23)^$A64)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A64)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.632158101020602</v>
+      </c>
+      <c r="D64" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A64)*(1+D$25),0.999)-(1-(1-D$23)^$A64))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A64)+D$43*MIN((1-(1-D$23)^$A64)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A64)+D$43*MIN((1-(1-D$23)^$A64)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A64)*(1-(1-(1-D$23)^$A64))/D$44+MIN((1-(1-D$23)^$A64)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A64)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.193908029867781</v>
+      </c>
+      <c r="E64" s="2"/>
+      <c r="F64" s="2"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B65" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A65)*(1+B$25),0.999)-(1-(1-B$23)^$A65))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A65)+B$43*MIN((1-(1-B$23)^$A65)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A65)+B$43*MIN((1-(1-B$23)^$A65)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A65)*(1-(1-(1-B$23)^$A65))/B$44+MIN((1-(1-B$23)^$A65)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A65)*(1+B$25),0.999))/B$43)),0)</f>
+        <v>0.999999993632062</v>
+      </c>
+      <c r="C65" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A65)*(1+C$25),0.999)-(1-(1-C$23)^$A65))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A65)+C$43*MIN((1-(1-C$23)^$A65)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A65)+C$43*MIN((1-(1-C$23)^$A65)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A65)*(1-(1-(1-C$23)^$A65))/C$44+MIN((1-(1-C$23)^$A65)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A65)*(1+C$25),0.999))/C$43)),0)</f>
+        <v>0.686177648758822</v>
+      </c>
+      <c r="D65" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A65)*(1+D$25),0.999)-(1-(1-D$23)^$A65))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A65)+D$43*MIN((1-(1-D$23)^$A65)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A65)+D$43*MIN((1-(1-D$23)^$A65)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A65)*(1-(1-(1-D$23)^$A65))/D$44+MIN((1-(1-D$23)^$A65)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A65)*(1+D$25),0.999))/D$43)),0)</f>
+        <v>0.214228302973138</v>
+      </c>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B67" s="27"/>
+      <c r="C67" s="27"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="27"/>
+      <c r="F67" s="2"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="27"/>
+      <c r="B68" s="27"/>
+      <c r="C68" s="27"/>
+      <c r="D68" s="27"/>
+      <c r="E68" s="27"/>
+      <c r="F68" s="2"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="27"/>
+      <c r="B69" s="27"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="27"/>
+      <c r="F69" s="2"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
+      <c r="D70" s="2"/>
+      <c r="E70" s="2"/>
+      <c r="F70" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A45:E46"/>
+    <mergeCell ref="A67:E69"/>
   </mergeCells>
-  <conditionalFormatting sqref="B30:D30">
+  <conditionalFormatting sqref="B32:D32">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"SÍ"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B35:D35">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>LEFT(B35,2)="Sí"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>LEFT(B35,2)="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1765,248 +2164,248 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="B3" s="11" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="23" t="n">
+      <c r="A5" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="29" t="n">
         <v>0.15</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="29" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="29" t="n">
         <v>0.3</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="29" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="n">
+      <c r="A6" s="29" t="n">
         <v>0.01</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A6+($A6*(1+B$5*$B$3)))/2)*(1-(($A6+($A6*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A6*(1-$A6)+($A6*(1+B$5*$B$3))*(1-($A6*(1+B$5*$B$3)))))^2)/(($A6*(1+B$5*$B$3))-$A6)^2,0)</f>
         <v>217542</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A6+($A6*(1+C$5*$B$3)))/2)*(1-(($A6+($A6*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A6*(1-$A6)+($A6*(1+C$5*$B$3))*(1-($A6*(1+C$5*$B$3)))))^2)/(($A6*(1+C$5*$B$3))-$A6)^2,0)</f>
         <v>98962</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A6+($A6*(1+D$5*$B$3)))/2)*(1-(($A6+($A6*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A6*(1-$A6)+($A6*(1+D$5*$B$3))*(1-($A6*(1+D$5*$B$3)))))^2)/(($A6*(1+D$5*$B$3))-$A6)^2,0)</f>
         <v>56946</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A6+($A6*(1+E$5*$B$3)))/2)*(1-(($A6+($A6*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A6*(1-$A6)+($A6*(1+E$5*$B$3))*(1-($A6*(1+E$5*$B$3)))))^2)/(($A6*(1+E$5*$B$3))-$A6)^2,0)</f>
         <v>26446</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A6+($A6*(1+F$5*$B$3)))/2)*(1-(($A6+($A6*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A6*(1-$A6)+($A6*(1+F$5*$B$3))*(1-($A6*(1+F$5*$B$3)))))^2)/(($A6*(1+F$5*$B$3))-$A6)^2,0)</f>
         <v>10337</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="n">
+      <c r="A7" s="29" t="n">
         <v>0.02</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A7+($A7*(1+B$5*$B$3)))/2)*(1-(($A7+($A7*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A7*(1-$A7)+($A7*(1+B$5*$B$3))*(1-($A7*(1+B$5*$B$3)))))^2)/(($A7*(1+B$5*$B$3))-$A7)^2,0)</f>
         <v>107616</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A7+($A7*(1+C$5*$B$3)))/2)*(1-(($A7+($A7*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A7*(1-$A7)+($A7*(1+C$5*$B$3))*(1-($A7*(1+C$5*$B$3)))))^2)/(($A7*(1+C$5*$B$3))-$A7)^2,0)</f>
         <v>48943</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A7+($A7*(1+D$5*$B$3)))/2)*(1-(($A7+($A7*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A7*(1-$A7)+($A7*(1+D$5*$B$3))*(1-($A7*(1+D$5*$B$3)))))^2)/(($A7*(1+D$5*$B$3))-$A7)^2,0)</f>
         <v>28156</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A7+($A7*(1+E$5*$B$3)))/2)*(1-(($A7+($A7*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A7*(1-$A7)+($A7*(1+E$5*$B$3))*(1-($A7*(1+E$5*$B$3)))))^2)/(($A7*(1+E$5*$B$3))-$A7)^2,0)</f>
         <v>13069</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A7+($A7*(1+F$5*$B$3)))/2)*(1-(($A7+($A7*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A7*(1-$A7)+($A7*(1+F$5*$B$3))*(1-($A7*(1+F$5*$B$3)))))^2)/(($A7*(1+F$5*$B$3))-$A7)^2,0)</f>
         <v>5103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="n">
+      <c r="A8" s="29" t="n">
         <v>0.03</v>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A8+($A8*(1+B$5*$B$3)))/2)*(1-(($A8+($A8*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A8*(1-$A8)+($A8*(1+B$5*$B$3))*(1-($A8*(1+B$5*$B$3)))))^2)/(($A8*(1+B$5*$B$3))-$A8)^2,0)</f>
         <v>70974</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A8+($A8*(1+C$5*$B$3)))/2)*(1-(($A8+($A8*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A8*(1-$A8)+($A8*(1+C$5*$B$3))*(1-($A8*(1+C$5*$B$3)))))^2)/(($A8*(1+C$5*$B$3))-$A8)^2,0)</f>
         <v>32270</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A8+($A8*(1+D$5*$B$3)))/2)*(1-(($A8+($A8*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A8*(1-$A8)+($A8*(1+D$5*$B$3))*(1-($A8*(1+D$5*$B$3)))))^2)/(($A8*(1+D$5*$B$3))-$A8)^2,0)</f>
         <v>18559</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A8+($A8*(1+E$5*$B$3)))/2)*(1-(($A8+($A8*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A8*(1-$A8)+($A8*(1+E$5*$B$3))*(1-($A8*(1+E$5*$B$3)))))^2)/(($A8*(1+E$5*$B$3))-$A8)^2,0)</f>
         <v>8610</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A8+($A8*(1+F$5*$B$3)))/2)*(1-(($A8+($A8*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A8*(1-$A8)+($A8*(1+F$5*$B$3))*(1-($A8*(1+F$5*$B$3)))))^2)/(($A8*(1+F$5*$B$3))-$A8)^2,0)</f>
         <v>3358</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="n">
+      <c r="A9" s="29" t="n">
         <v>0.05</v>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A9+($A9*(1+B$5*$B$3)))/2)*(1-(($A9+($A9*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A9*(1-$A9)+($A9*(1+B$5*$B$3))*(1-($A9*(1+B$5*$B$3)))))^2)/(($A9*(1+B$5*$B$3))-$A9)^2,0)</f>
         <v>41661</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A9+($A9*(1+C$5*$B$3)))/2)*(1-(($A9+($A9*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A9*(1-$A9)+($A9*(1+C$5*$B$3))*(1-($A9*(1+C$5*$B$3)))))^2)/(($A9*(1+C$5*$B$3))-$A9)^2,0)</f>
         <v>18931</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A9+($A9*(1+D$5*$B$3)))/2)*(1-(($A9+($A9*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A9*(1-$A9)+($A9*(1+D$5*$B$3))*(1-($A9*(1+D$5*$B$3)))))^2)/(($A9*(1+D$5*$B$3))-$A9)^2,0)</f>
         <v>10882</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A9+($A9*(1+E$5*$B$3)))/2)*(1-(($A9+($A9*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A9*(1-$A9)+($A9*(1+E$5*$B$3))*(1-($A9*(1+E$5*$B$3)))))^2)/(($A9*(1+E$5*$B$3))-$A9)^2,0)</f>
         <v>5042</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A9+($A9*(1+F$5*$B$3)))/2)*(1-(($A9+($A9*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A9*(1-$A9)+($A9*(1+F$5*$B$3))*(1-($A9*(1+F$5*$B$3)))))^2)/(($A9*(1+F$5*$B$3))-$A9)^2,0)</f>
         <v>1962</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
+      <c r="A10" s="29" t="n">
         <v>0.08</v>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A10+($A10*(1+B$5*$B$3)))/2)*(1-(($A10+($A10*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A10*(1-$A10)+($A10*(1+B$5*$B$3))*(1-($A10*(1+B$5*$B$3)))))^2)/(($A10*(1+B$5*$B$3))-$A10)^2,0)</f>
         <v>25172</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A10+($A10*(1+C$5*$B$3)))/2)*(1-(($A10+($A10*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A10*(1-$A10)+($A10*(1+C$5*$B$3))*(1-($A10*(1+C$5*$B$3)))))^2)/(($A10*(1+C$5*$B$3))-$A10)^2,0)</f>
         <v>11429</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A10+($A10*(1+D$5*$B$3)))/2)*(1-(($A10+($A10*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A10*(1-$A10)+($A10*(1+D$5*$B$3))*(1-($A10*(1+D$5*$B$3)))))^2)/(($A10*(1+D$5*$B$3))-$A10)^2,0)</f>
         <v>6563</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A10+($A10*(1+E$5*$B$3)))/2)*(1-(($A10+($A10*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A10*(1-$A10)+($A10*(1+E$5*$B$3))*(1-($A10*(1+E$5*$B$3)))))^2)/(($A10*(1+E$5*$B$3))-$A10)^2,0)</f>
         <v>3036</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A10+($A10*(1+F$5*$B$3)))/2)*(1-(($A10+($A10*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A10*(1-$A10)+($A10*(1+F$5*$B$3))*(1-($A10*(1+F$5*$B$3)))))^2)/(($A10*(1+F$5*$B$3))-$A10)^2,0)</f>
         <v>1177</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="n">
+      <c r="A11" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A11+($A11*(1+B$5*$B$3)))/2)*(1-(($A11+($A11*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A11*(1-$A11)+($A11*(1+B$5*$B$3))*(1-($A11*(1+B$5*$B$3)))))^2)/(($A11*(1+B$5*$B$3))-$A11)^2,0)</f>
         <v>19676</v>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A11+($A11*(1+C$5*$B$3)))/2)*(1-(($A11+($A11*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A11*(1-$A11)+($A11*(1+C$5*$B$3))*(1-($A11*(1+C$5*$B$3)))))^2)/(($A11*(1+C$5*$B$3))-$A11)^2,0)</f>
         <v>8928</v>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D11" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A11+($A11*(1+D$5*$B$3)))/2)*(1-(($A11+($A11*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A11*(1-$A11)+($A11*(1+D$5*$B$3))*(1-($A11*(1+D$5*$B$3)))))^2)/(($A11*(1+D$5*$B$3))-$A11)^2,0)</f>
         <v>5124</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A11+($A11*(1+E$5*$B$3)))/2)*(1-(($A11+($A11*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A11*(1-$A11)+($A11*(1+E$5*$B$3))*(1-($A11*(1+E$5*$B$3)))))^2)/(($A11*(1+E$5*$B$3))-$A11)^2,0)</f>
         <v>2367</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A11+($A11*(1+F$5*$B$3)))/2)*(1-(($A11+($A11*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A11*(1-$A11)+($A11*(1+F$5*$B$3))*(1-($A11*(1+F$5*$B$3)))))^2)/(($A11*(1+F$5*$B$3))-$A11)^2,0)</f>
         <v>915</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="29" t="n">
         <v>0.15</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A12+($A12*(1+B$5*$B$3)))/2)*(1-(($A12+($A12*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A12*(1-$A12)+($A12*(1+B$5*$B$3))*(1-($A12*(1+B$5*$B$3)))))^2)/(($A12*(1+B$5*$B$3))-$A12)^2,0)</f>
         <v>12347</v>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A12+($A12*(1+C$5*$B$3)))/2)*(1-(($A12+($A12*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A12*(1-$A12)+($A12*(1+C$5*$B$3))*(1-($A12*(1+C$5*$B$3)))))^2)/(($A12*(1+C$5*$B$3))-$A12)^2,0)</f>
         <v>5593</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A12+($A12*(1+D$5*$B$3)))/2)*(1-(($A12+($A12*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A12*(1-$A12)+($A12*(1+D$5*$B$3))*(1-($A12*(1+D$5*$B$3)))))^2)/(($A12*(1+D$5*$B$3))-$A12)^2,0)</f>
         <v>3204</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A12+($A12*(1+E$5*$B$3)))/2)*(1-(($A12+($A12*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A12*(1-$A12)+($A12*(1+E$5*$B$3))*(1-($A12*(1+E$5*$B$3)))))^2)/(($A12*(1+E$5*$B$3))-$A12)^2,0)</f>
         <v>1475</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A12+($A12*(1+F$5*$B$3)))/2)*(1-(($A12+($A12*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A12*(1-$A12)+($A12*(1+F$5*$B$3))*(1-($A12*(1+F$5*$B$3)))))^2)/(($A12*(1+F$5*$B$3))-$A12)^2,0)</f>
         <v>566</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="n">
+      <c r="A13" s="29" t="n">
         <v>0.2</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A13+($A13*(1+B$5*$B$3)))/2)*(1-(($A13+($A13*(1+B$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A13*(1-$A13)+($A13*(1+B$5*$B$3))*(1-($A13*(1+B$5*$B$3)))))^2)/(($A13*(1+B$5*$B$3))-$A13)^2,0)</f>
         <v>8683</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A13+($A13*(1+C$5*$B$3)))/2)*(1-(($A13+($A13*(1+C$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A13*(1-$A13)+($A13*(1+C$5*$B$3))*(1-($A13*(1+C$5*$B$3)))))^2)/(($A13*(1+C$5*$B$3))-$A13)^2,0)</f>
         <v>3926</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A13+($A13*(1+D$5*$B$3)))/2)*(1-(($A13+($A13*(1+D$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A13*(1-$A13)+($A13*(1+D$5*$B$3))*(1-($A13*(1+D$5*$B$3)))))^2)/(($A13*(1+D$5*$B$3))-$A13)^2,0)</f>
         <v>2245</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A13+($A13*(1+E$5*$B$3)))/2)*(1-(($A13+($A13*(1+E$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A13*(1-$A13)+($A13*(1+E$5*$B$3))*(1-($A13*(1+E$5*$B$3)))))^2)/(($A13*(1+E$5*$B$3))-$A13)^2,0)</f>
         <v>1029</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="30" t="n">
         <f aca="false">ROUNDUP(((Calculadora!$B$10*SQRT(2*(($A13+($A13*(1+F$5*$B$3)))/2)*(1-(($A13+($A13*(1+F$5*$B$3)))/2)))+Calculadora!$B$11*SQRT($A13*(1-$A13)+($A13*(1+F$5*$B$3))*(1-($A13*(1+F$5*$B$3)))))^2)/(($A13*(1+F$5*$B$3))-$A13)^2,0)</f>
         <v>392</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2025,71 +2424,76 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="125"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="s">
-        <v>84</v>
+      <c r="A3" s="31" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
-        <v>86</v>
+      <c r="A4" s="31" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="31" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>87</v>
+      <c r="A6" s="31" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
-        <v>89</v>
+      <c r="A7" s="31" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="31" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24"/>
+      <c r="A9" s="31" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>91</v>
+      <c r="A10" s="31"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="32" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>92</v>
+      <c r="A12" s="31" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24"/>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
-        <v>93</v>
+      <c r="A13" s="31" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="31"/>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="31" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calculator: editable treatment and control user counts with cap check
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ygiEd3g3fKiFCARJZcKLp
</commit_message>
<xml_diff>
--- a/calculadora-sample-size.xlsx
+++ b/calculadora-sample-size.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="111">
   <si>
     <t xml:space="preserve">Calculadora de sample size y poder: experimento de crédito por score</t>
   </si>
@@ -105,13 +105,19 @@
     <t xml:space="preserve">MÁXIMO de referidores disponibles en el tier (tope)</t>
   </si>
   <si>
-    <t xml:space="preserve">El máximo que de verdad existe. Todo se calcula con este tope, nunca con más.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% del tope que va a tratamiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50% = mitad tratamiento y mitad control (el más eficiente). El resto queda en control a 500 MXN. Usa entre 10% y 90%.</t>
+    <t xml:space="preserve">El máximo que de verdad existe en el tier. Solo valida que no uses más de lo que hay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usuarios en TRATAMIENTO (nuevo crédito)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuántos referidores recibirán el crédito nuevo. Escríbelo tú. Tratamiento + control no deben pasar del tope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usuarios en CONTROL (se quedan en 500 MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuántos referidores se quedan en 500 MXN para comparar. Lo más eficiente es igual que tratamiento.</t>
   </si>
   <si>
     <t xml:space="preserve">Loans nuevos al mes del tier (con 500 MXN)</t>
@@ -138,7 +144,7 @@
     <t xml:space="preserve">% de quienes reciben el crédito que realmente lo usa. Diluye el efecto.</t>
   </si>
   <si>
-    <t xml:space="preserve">RESULTADOS CON TU TOPE</t>
+    <t xml:space="preserve">RESULTADOS CON TUS USUARIOS</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo leerlo</t>
@@ -171,16 +177,22 @@
     <t xml:space="preserve">Usuarios efectivos en tratamiento</t>
   </si>
   <si>
-    <t xml:space="preserve">Tope × % tratamiento, menos pérdidas.</t>
+    <t xml:space="preserve">Tus usuarios en tratamiento menos pérdidas.</t>
   </si>
   <si>
     <t xml:space="preserve">Usuarios efectivos en control (500 MXN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Tope × % control, menos pérdidas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PODER real con tu tope</t>
+    <t xml:space="preserve">Tus usuarios en control menos pérdidas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Tratamiento + control caben en el tope?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verde = no usas más referidores de los que existen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PODER real con tus usuarios</t>
   </si>
   <si>
     <t xml:space="preserve">Probabilidad de detectar el lift esperado con tus usuarios. Busca 80% o más.</t>
@@ -189,7 +201,7 @@
     <t xml:space="preserve">Efecto mínimo detectable relativo (todo el grupo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Con tu tope solo detectas cambios de este tamaño o mayores en la tasa base.</t>
+    <t xml:space="preserve">Con tus usuarios solo detectas cambios de este tamaño o mayores en la tasa base.</t>
   </si>
   <si>
     <t xml:space="preserve">Efecto mínimo detectable entre quienes usan el crédito</t>
@@ -201,7 +213,7 @@
     <t xml:space="preserve">¿Detecta el lift esperado?</t>
   </si>
   <si>
-    <t xml:space="preserve">SÍ = con tu tope llegas al poder objetivo.</t>
+    <t xml:space="preserve">SÍ = con tus usuarios llegas al poder objetivo.</t>
   </si>
   <si>
     <t xml:space="preserve">REFERENCIA: lo que necesitarías</t>
@@ -210,7 +222,7 @@
     <t xml:space="preserve">Usuarios totales que harían falta (con pérdidas)</t>
   </si>
   <si>
-    <t xml:space="preserve">Para detectar el lift esperado con el poder objetivo y tu % de tratamiento. Es solo referencia.</t>
+    <t xml:space="preserve">Para detectar el lift esperado con el poder objetivo y tu proporción tratamiento/control. Es solo referencia.</t>
   </si>
   <si>
     <t xml:space="preserve">¿Cabe en tu tope?</t>
@@ -219,10 +231,10 @@
     <t xml:space="preserve">Compara lo necesario contra el máximo que tienes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Meses de ventana para llegar al poder con tu tope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con tu tope y tu lift, cuántos meses mediría cada usuario para llegar a 80% (máx. 12). Asume meses independientes.</t>
+    <t xml:space="preserve">Meses de ventana para llegar al poder con tus usuarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con tus usuarios y tu lift, cuántos meses mediría cada usuario para llegar a 80% (máx. 12). Asume meses independientes.</t>
   </si>
   <si>
     <t xml:space="preserve">Recomendación</t>
@@ -231,7 +243,7 @@
     <t xml:space="preserve">Qué hacer con este tier.</t>
   </si>
   <si>
-    <t xml:space="preserve">CÁLCULO AUXILIAR (no editar)</t>
+    <t xml:space="preserve">CÁLCULO AUXILIAR (aquí no se escribe: cambia los datos de arriba)</t>
   </si>
   <si>
     <t xml:space="preserve">Para qué sirve</t>
@@ -246,13 +258,13 @@
     <t xml:space="preserve">n efectivo tratamiento</t>
   </si>
   <si>
-    <t xml:space="preserve">Tope × % tratamiento × (1 - pérdidas).</t>
+    <t xml:space="preserve">Usuarios en tratamiento × (1 - pérdidas).</t>
   </si>
   <si>
     <t xml:space="preserve">n efectivo control</t>
   </si>
   <si>
-    <t xml:space="preserve">Tope × (1 - % tratamiento) × (1 - pérdidas).</t>
+    <t xml:space="preserve">Usuarios en control × (1 - pérdidas).</t>
   </si>
   <si>
     <t xml:space="preserve">Tasa combinada bajo H0</t>
@@ -285,10 +297,10 @@
     <t xml:space="preserve">PODER POR MESES DE VENTANA (auxiliar)</t>
   </si>
   <si>
-    <t xml:space="preserve">Poder con tu tope si midieras cada usuario por N meses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supuestos: prueba de dos proporciones, dos colas, aproximación normal, con grupos de tamaño distinto si cambias el % de tratamiento. La tasa base mensual asume 1 loan por referidor; si hay referidores con varios loans, la tasa real es menor. Tasa acumulada = 1-(1-p)^meses asume meses independientes (en la práctica es algo menor). Si tu tope de 10K es el TOTAL entre los 3 tiers y no por tier, divídelo entre los tiers en la fila del tope.</t>
+    <t xml:space="preserve">Poder con tus usuarios si midieras cada uno por N meses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuestos: prueba de dos proporciones, dos colas, aproximación normal, con grupos de tamaño distinto si tratamiento y control no son iguales. La tasa base mensual asume 1 loan por referidor; si hay referidores con varios loans, la tasa real es menor. Tasa acumulada = 1-(1-p)^meses asume meses independientes (en la práctica es algo menor). Si tu máximo de 10K es el TOTAL entre los 3 tiers y no por tier, repártelo en las filas de tratamiento y control de cada tier.</t>
   </si>
   <si>
     <t xml:space="preserve">Usuarios necesarios por brazo según tasa base y lift (referencia, 50/50)</t>
@@ -318,13 +330,13 @@
     <t xml:space="preserve">2. Parámetros generales: deja alpha 0.05 y poder 0.80 salvo que tengas otra regla. Pon en comparaciones cuántos tiers pruebas (3 si Excelente, Bueno y Bajo).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Por tier: tu TOPE de referidores (el máximo que existe), el % que va a tratamiento, loans nuevos al mes con 500 MXN, meses de ventana, lift esperado y take-up.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Lee primero 'PODER real con tu tope' y '¿Detecta el lift esperado?'. Esos números usan solo tus usuarios disponibles.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Si dice NO, mira 'Efecto mínimo detectable' (lo más chico que sí verías con tu tope) y 'Meses de ventana para llegar al poder'.</t>
+    <t xml:space="preserve">3. Por tier: tu TOPE de referidores (el máximo que existe), cuántos usuarios pones en TRATAMIENTO y cuántos en CONTROL (los escribes tú), loans nuevos al mes con 500 MXN, meses de ventana, lift esperado y take-up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Lee primero 'PODER real con tus usuarios' y '¿Detecta el lift esperado?'. Esos números usan exactamente los usuarios que escribiste. La fila verde/roja te avisa si pasas el tope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Si dice NO, mira 'Efecto mínimo detectable' (lo más chico que sí verías con tus usuarios) y 'Meses de ventana para llegar al poder'.</t>
   </si>
   <si>
     <t xml:space="preserve">6. 'Referencia: lo que necesitarías' es solo para comparar contra tu tope. Si no cabe, no lo persigas: alarga la ventana, prueba menos tiers o espera un lift mayor.</t>
@@ -582,6 +594,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -599,10 +615,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1167,32 +1179,32 @@
       <c r="A16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>0.5</v>
+      <c r="B16" s="14" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>5000</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="C17" s="14" t="n">
-        <v>300</v>
+        <v>5000</v>
       </c>
       <c r="D17" s="14" t="n">
-        <v>100</v>
+        <v>5000</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>31</v>
@@ -1203,14 +1215,14 @@
       <c r="A18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>1</v>
+      <c r="B18" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>100</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>33</v>
@@ -1221,14 +1233,14 @@
       <c r="A19" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C19" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>-0.15</v>
+      <c r="B19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>35</v>
@@ -1240,13 +1252,13 @@
         <v>36</v>
       </c>
       <c r="B20" s="11" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>0.6</v>
+        <v>0.15</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>0.6</v>
+        <v>-0.15</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>37</v>
@@ -1254,48 +1266,45 @@
       <c r="F20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="A21" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>39</v>
+      </c>
       <c r="F21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="5" t="s">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F22" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="15" t="n">
-        <f aca="false">B17/B15</f>
-        <v>0.05</v>
-      </c>
-      <c r="C23" s="15" t="n">
-        <f aca="false">C17/C15</f>
-        <v>0.03</v>
-      </c>
-      <c r="D23" s="15" t="n">
-        <f aca="false">D17/D15</f>
-        <v>0.01</v>
-      </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="5" t="s">
         <v>41</v>
       </c>
       <c r="F23" s="2"/>
@@ -1305,15 +1314,15 @@
         <v>42</v>
       </c>
       <c r="B24" s="15" t="n">
-        <f aca="false">1-(1-B23)^B18</f>
+        <f aca="false">B18/B15</f>
         <v>0.05</v>
       </c>
       <c r="C24" s="15" t="n">
-        <f aca="false">1-(1-C23)^C18</f>
+        <f aca="false">C18/C15</f>
         <v>0.03</v>
       </c>
       <c r="D24" s="15" t="n">
-        <f aca="false">1-(1-D23)^D18</f>
+        <f aca="false">D18/D15</f>
         <v>0.01</v>
       </c>
       <c r="E24" s="8" t="s">
@@ -1325,17 +1334,17 @@
       <c r="A25" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="16" t="n">
-        <f aca="false">B19*B20</f>
-        <v>0.18</v>
-      </c>
-      <c r="C25" s="16" t="n">
-        <f aca="false">C19*C20</f>
-        <v>0.09</v>
-      </c>
-      <c r="D25" s="16" t="n">
-        <f aca="false">D19*D20</f>
-        <v>-0.09</v>
+      <c r="B25" s="15" t="n">
+        <f aca="false">1-(1-B24)^B19</f>
+        <v>0.05</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <f aca="false">1-(1-C24)^C19</f>
+        <v>0.03</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <f aca="false">1-(1-D24)^D19</f>
+        <v>0.01</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>45</v>
@@ -1346,17 +1355,17 @@
       <c r="A26" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="15" t="n">
-        <f aca="false">B24*(1+B25)</f>
-        <v>0.0590000000000001</v>
-      </c>
-      <c r="C26" s="15" t="n">
-        <f aca="false">C24*(1+C25)</f>
-        <v>0.0327</v>
-      </c>
-      <c r="D26" s="15" t="n">
-        <f aca="false">D24*(1+D25)</f>
-        <v>0.00910000000000001</v>
+      <c r="B26" s="16" t="n">
+        <f aca="false">B20*B21</f>
+        <v>0.18</v>
+      </c>
+      <c r="C26" s="16" t="n">
+        <f aca="false">C20*C21</f>
+        <v>0.09</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <f aca="false">D20*D21</f>
+        <v>-0.09</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>47</v>
@@ -1367,17 +1376,17 @@
       <c r="A27" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B27" s="17" t="n">
-        <f aca="false">B43</f>
-        <v>4750</v>
-      </c>
-      <c r="C27" s="17" t="n">
-        <f aca="false">C43</f>
-        <v>4750</v>
-      </c>
-      <c r="D27" s="17" t="n">
-        <f aca="false">D43</f>
-        <v>4750</v>
+      <c r="B27" s="15" t="n">
+        <f aca="false">B25*(1+B26)</f>
+        <v>0.0590000000000001</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <f aca="false">C25*(1+C26)</f>
+        <v>0.0327</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <f aca="false">D25*(1+D26)</f>
+        <v>0.00910000000000001</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>49</v>
@@ -1409,17 +1418,17 @@
       <c r="A29" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="18" t="n">
-        <f aca="false">NORMSDIST((ABS(B26-B24)-$B$10*SQRT(B45*(1-B45)*(1/B44+1/B43)))/SQRT(B24*(1-B24)/B44+B26*(1-B26)/B43))</f>
-        <v>0.322076256263711</v>
-      </c>
-      <c r="C29" s="18" t="n">
-        <f aca="false">NORMSDIST((ABS(C26-C24)-$B$10*SQRT(C45*(1-C45)*(1/C44+1/C43)))/SQRT(C24*(1-C24)/C44+C26*(1-C26)/C43))</f>
-        <v>0.0506120133084721</v>
-      </c>
-      <c r="D29" s="18" t="n">
-        <f aca="false">NORMSDIST((ABS(D26-D24)-$B$10*SQRT(D45*(1-D45)*(1/D44+1/D43)))/SQRT(D24*(1-D24)/D44+D26*(1-D26)/D43))</f>
-        <v>0.0260067764439741</v>
+      <c r="B29" s="17" t="n">
+        <f aca="false">B45</f>
+        <v>4750</v>
+      </c>
+      <c r="C29" s="17" t="n">
+        <f aca="false">C45</f>
+        <v>4750</v>
+      </c>
+      <c r="D29" s="17" t="n">
+        <f aca="false">D45</f>
+        <v>4750</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>53</v>
@@ -1430,17 +1439,17 @@
       <c r="A30" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="16" t="n">
-        <f aca="false">B50/B24</f>
-        <v>0.309686211710248</v>
-      </c>
-      <c r="C30" s="16" t="n">
-        <f aca="false">C50/C24</f>
-        <v>0.413318181612153</v>
-      </c>
-      <c r="D30" s="16" t="n">
-        <f aca="false">D50/D24</f>
-        <v>0.776701739625666</v>
+      <c r="B30" s="18" t="str">
+        <f aca="false">IF(B16+B17&lt;=B15,"Sí: "&amp;TEXT(B16+B17,"#,##0")&amp;" de "&amp;TEXT(B15,"#,##0"),"NO: usas "&amp;TEXT(B16+B17,"#,##0")&amp;" y solo hay "&amp;TEXT(B15,"#,##0"))</f>
+        <v>Sí: 10,000 de 10,000</v>
+      </c>
+      <c r="C30" s="18" t="str">
+        <f aca="false">IF(C16+C17&lt;=C15,"Sí: "&amp;TEXT(C16+C17,"#,##0")&amp;" de "&amp;TEXT(C15,"#,##0"),"NO: usas "&amp;TEXT(C16+C17,"#,##0")&amp;" y solo hay "&amp;TEXT(C15,"#,##0"))</f>
+        <v>Sí: 10,000 de 10,000</v>
+      </c>
+      <c r="D30" s="18" t="str">
+        <f aca="false">IF(D16+D17&lt;=D15,"Sí: "&amp;TEXT(D16+D17,"#,##0")&amp;" de "&amp;TEXT(D15,"#,##0"),"NO: usas "&amp;TEXT(D16+D17,"#,##0")&amp;" y solo hay "&amp;TEXT(D15,"#,##0"))</f>
+        <v>Sí: 10,000 de 10,000</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>55</v>
@@ -1451,38 +1460,38 @@
       <c r="A31" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="16" t="n">
-        <f aca="false">B30/B20</f>
-        <v>0.516143686183747</v>
-      </c>
-      <c r="C31" s="16" t="n">
-        <f aca="false">C30/C20</f>
-        <v>0.688863636020255</v>
-      </c>
-      <c r="D31" s="16" t="n">
-        <f aca="false">D30/D20</f>
-        <v>1.29450289937611</v>
+      <c r="B31" s="19" t="n">
+        <f aca="false">NORMSDIST((ABS(B27-B25)-$B$10*SQRT(B46*(1-B46)*(1/B45+1/B44)))/SQRT(B25*(1-B25)/B45+B27*(1-B27)/B44))</f>
+        <v>0.322076256263711</v>
+      </c>
+      <c r="C31" s="19" t="n">
+        <f aca="false">NORMSDIST((ABS(C27-C25)-$B$10*SQRT(C46*(1-C46)*(1/C45+1/C44)))/SQRT(C25*(1-C25)/C45+C27*(1-C27)/C44))</f>
+        <v>0.0506120133084721</v>
+      </c>
+      <c r="D31" s="19" t="n">
+        <f aca="false">NORMSDIST((ABS(D27-D25)-$B$10*SQRT(D46*(1-D46)*(1/D45+1/D44)))/SQRT(D25*(1-D25)/D45+D27*(1-D27)/D44))</f>
+        <v>0.0260067764439741</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>57</v>
       </c>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B32" s="19" t="str">
-        <f aca="false">IF(B29&gt;=$B$6,"SÍ","NO")</f>
-        <v>NO</v>
-      </c>
-      <c r="C32" s="19" t="str">
-        <f aca="false">IF(C29&gt;=$B$6,"SÍ","NO")</f>
-        <v>NO</v>
-      </c>
-      <c r="D32" s="19" t="str">
-        <f aca="false">IF(D29&gt;=$B$6,"SÍ","NO")</f>
-        <v>NO</v>
+      <c r="B32" s="16" t="n">
+        <f aca="false">B51/B25</f>
+        <v>0.309686211710248</v>
+      </c>
+      <c r="C32" s="16" t="n">
+        <f aca="false">C51/C25</f>
+        <v>0.413318181612153</v>
+      </c>
+      <c r="D32" s="16" t="n">
+        <f aca="false">D51/D25</f>
+        <v>0.776701739625666</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>59</v>
@@ -1490,614 +1499,640 @@
       <c r="F32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="16" t="n">
+        <f aca="false">B32/B21</f>
+        <v>0.516143686183747</v>
+      </c>
+      <c r="C33" s="16" t="n">
+        <f aca="false">C32/C21</f>
+        <v>0.688863636020255</v>
+      </c>
+      <c r="D33" s="16" t="n">
+        <f aca="false">D32/D21</f>
+        <v>1.29450289937611</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="20" t="str">
+        <f aca="false">IF(B31&gt;=$B$6,"SÍ","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="C34" s="20" t="str">
+        <f aca="false">IF(C31&gt;=$B$6,"SÍ","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="D34" s="20" t="str">
+        <f aca="false">IF(D31&gt;=$B$6,"SÍ","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="C36" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D33" s="21" t="s">
+      <c r="D36" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E33" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="F33" s="2"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B34" s="22" t="n">
-        <f aca="false">IF(B25=0,"n/a",ROUNDUP((((($B$10*SQRT(((B24+B42*B26)/(1+B42))*(1-((B24+B42*B26)/(1+B42)))*(1+1/B42))+$B$11*SQRT(B24*(1-B24)+B26*(1-B26)/B42))^2)/(B26-B24)^2)*(1+B42))/(1-$B$8),0))</f>
+      <c r="E36" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="F36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="23" t="n">
+        <f aca="false">IF(B26=0,"n/a",ROUNDUP((((($B$10*SQRT(((B25+B43*B27)/(1+B43))*(1-((B25+B43*B27)/(1+B43)))*(1+1/B43))+$B$11*SQRT(B25*(1-B25)+B27*(1-B27)/B43))^2)/(B27-B25)^2)*(1+B43))/(1-$B$8),0))</f>
         <v>28040</v>
       </c>
-      <c r="C34" s="22" t="n">
-        <f aca="false">IF(C25=0,"n/a",ROUNDUP((((($B$10*SQRT(((C24+C42*C26)/(1+C42))*(1-((C24+C42*C26)/(1+C42)))*(1+1/C42))+$B$11*SQRT(C24*(1-C24)+C26*(1-C26)/C42))^2)/(C26-C24)^2)*(1+C42))/(1-$B$8),0))</f>
+      <c r="C37" s="23" t="n">
+        <f aca="false">IF(C26=0,"n/a",ROUNDUP((((($B$10*SQRT(((C25+C43*C27)/(1+C43))*(1-((C25+C43*C27)/(1+C43)))*(1+1/C43))+$B$11*SQRT(C25*(1-C25)+C27*(1-C27)/C43))^2)/(C27-C25)^2)*(1+C43))/(1-$B$8),0))</f>
         <v>183619</v>
       </c>
-      <c r="D34" s="22" t="n">
-        <f aca="false">IF(D25=0,"n/a",ROUNDUP((((($B$10*SQRT(((D24+D42*D26)/(1+D42))*(1-((D24+D42*D26)/(1+D42)))*(1+1/D42))+$B$11*SQRT(D24*(1-D24)+D26*(1-D26)/D42))^2)/(D26-D24)^2)*(1+D42))/(1-$B$8),0))</f>
+      <c r="D37" s="23" t="n">
+        <f aca="false">IF(D26=0,"n/a",ROUNDUP((((($B$10*SQRT(((D25+D43*D27)/(1+D43))*(1-((D25+D43*D27)/(1+D43)))*(1+1/D43))+$B$11*SQRT(D25*(1-D25)+D27*(1-D27)/D43))^2)/(D27-D25)^2)*(1+D43))/(1-$B$8),0))</f>
         <v>514749</v>
       </c>
-      <c r="E34" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="F34" s="2"/>
-    </row>
-    <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B35" s="23" t="str">
-        <f aca="false">IF(ISNUMBER(B34),IF(B34&lt;=B15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(B34-B15,"#,##0")),"n/a")</f>
+      <c r="E37" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="18" t="str">
+        <f aca="false">IF(ISNUMBER(B37),IF(B37&lt;=B15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(B37-B15,"#,##0")),"n/a")</f>
         <v>No cabe: faltan 18,040</v>
       </c>
-      <c r="C35" s="23" t="str">
-        <f aca="false">IF(ISNUMBER(C34),IF(C34&lt;=C15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(C34-C15,"#,##0")),"n/a")</f>
+      <c r="C38" s="18" t="str">
+        <f aca="false">IF(ISNUMBER(C37),IF(C37&lt;=C15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(C37-C15,"#,##0")),"n/a")</f>
         <v>No cabe: faltan 173,619</v>
       </c>
-      <c r="D35" s="23" t="str">
-        <f aca="false">IF(ISNUMBER(D34),IF(D34&lt;=D15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(D34-D15,"#,##0")),"n/a")</f>
+      <c r="D38" s="18" t="str">
+        <f aca="false">IF(ISNUMBER(D37),IF(D37&lt;=D15,"Sí cabe en tu tope","No cabe: faltan "&amp;TEXT(D37-D15,"#,##0")),"n/a")</f>
         <v>No cabe: faltan 504,749</v>
       </c>
-      <c r="E35" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F35" s="2"/>
-    </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B36" s="24" t="n">
-        <f aca="false">IF(COUNTIF(B54:B65,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(B54:B65,"&lt;"&amp;$B$6)+1)</f>
+      <c r="E38" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B39" s="24" t="n">
+        <f aca="false">IF(COUNTIF(B55:B66,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(B55:B66,"&lt;"&amp;$B$6)+1)</f>
         <v>3</v>
       </c>
-      <c r="C36" s="24" t="str">
-        <f aca="false">IF(COUNTIF(C54:C65,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(C54:C65,"&lt;"&amp;$B$6)+1)</f>
+      <c r="C39" s="24" t="str">
+        <f aca="false">IF(COUNTIF(C55:C66,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(C55:C66,"&lt;"&amp;$B$6)+1)</f>
         <v>&gt;12</v>
       </c>
-      <c r="D36" s="24" t="str">
-        <f aca="false">IF(COUNTIF(D54:D65,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(D54:D65,"&lt;"&amp;$B$6)+1)</f>
+      <c r="D39" s="24" t="str">
+        <f aca="false">IF(COUNTIF(D55:D66,"&gt;="&amp;$B$6)=0,"&gt;12",COUNTIF(D55:D66,"&lt;"&amp;$B$6)+1)</f>
         <v>&gt;12</v>
       </c>
-      <c r="E36" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F36" s="2"/>
-    </row>
-    <row r="37" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B37" s="19" t="str">
-        <f aca="false">IF(B32="SÍ","Corre el experimento con tu tope.",IF(ISNUMBER(B36),"Alarga la ventana a "&amp;B36&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
+      <c r="E39" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B40" s="20" t="str">
+        <f aca="false">IF(B34="SÍ","Corre el experimento con tus usuarios.",IF(ISNUMBER(B39),"Alarga la ventana a "&amp;B39&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
         <v>Alarga la ventana a 3 meses.</v>
       </c>
-      <c r="C37" s="19" t="str">
-        <f aca="false">IF(C32="SÍ","Corre el experimento con tu tope.",IF(ISNUMBER(C36),"Alarga la ventana a "&amp;C36&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
+      <c r="C40" s="20" t="str">
+        <f aca="false">IF(C34="SÍ","Corre el experimento con tus usuarios.",IF(ISNUMBER(C39),"Alarga la ventana a "&amp;C39&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
         <v>No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor.</v>
       </c>
-      <c r="D37" s="19" t="str">
-        <f aca="false">IF(D32="SÍ","Corre el experimento con tu tope.",IF(ISNUMBER(D36),"Alarga la ventana a "&amp;D36&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
+      <c r="D40" s="20" t="str">
+        <f aca="false">IF(D34="SÍ","Corre el experimento con tus usuarios.",IF(ISNUMBER(D39),"Alarga la ventana a "&amp;D39&amp;" meses.","No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor."))</f>
         <v>No alcanza ni a 12 meses: prueba menos tiers o espera un lift mayor.</v>
       </c>
-      <c r="E37" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+      <c r="E40" s="8" t="s">
+        <v>72</v>
+      </c>
       <c r="F40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B41" s="5" t="s">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E41" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="F41" s="2"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B42" s="25" t="n">
-        <f aca="false">B16/(1-B16)</f>
-        <v>1</v>
-      </c>
-      <c r="C42" s="25" t="n">
-        <f aca="false">C16/(1-C16)</f>
-        <v>1</v>
-      </c>
-      <c r="D42" s="25" t="n">
-        <f aca="false">D16/(1-D16)</f>
-        <v>1</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>72</v>
+      <c r="E42" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="F42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B43" s="17" t="n">
-        <f aca="false">B15*B16*(1-$B$8)</f>
-        <v>4750</v>
-      </c>
-      <c r="C43" s="17" t="n">
-        <f aca="false">C15*C16*(1-$B$8)</f>
-        <v>4750</v>
-      </c>
-      <c r="D43" s="17" t="n">
-        <f aca="false">D15*D16*(1-$B$8)</f>
-        <v>4750</v>
+        <v>75</v>
+      </c>
+      <c r="B43" s="25" t="n">
+        <f aca="false">B16/B17</f>
+        <v>1</v>
+      </c>
+      <c r="C43" s="25" t="n">
+        <f aca="false">C16/C17</f>
+        <v>1</v>
+      </c>
+      <c r="D43" s="25" t="n">
+        <f aca="false">D16/D17</f>
+        <v>1</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B44" s="17" t="n">
-        <f aca="false">B15*(1-B16)*(1-$B$8)</f>
+        <f aca="false">B16*(1-$B$8)</f>
         <v>4750</v>
       </c>
       <c r="C44" s="17" t="n">
-        <f aca="false">C15*(1-C16)*(1-$B$8)</f>
+        <f aca="false">C16*(1-$B$8)</f>
         <v>4750</v>
       </c>
       <c r="D44" s="17" t="n">
-        <f aca="false">D15*(1-D16)*(1-$B$8)</f>
+        <f aca="false">D16*(1-$B$8)</f>
         <v>4750</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B45" s="12" t="n">
-        <f aca="false">(B44*B24+B43*B26)/(B44+B43)</f>
-        <v>0.0545000000000001</v>
-      </c>
-      <c r="C45" s="12" t="n">
-        <f aca="false">(C44*C24+C43*C26)/(C44+C43)</f>
-        <v>0.03135</v>
-      </c>
-      <c r="D45" s="12" t="n">
-        <f aca="false">(D44*D24+D43*D26)/(D44+D43)</f>
-        <v>0.00955000000000001</v>
+        <v>79</v>
+      </c>
+      <c r="B45" s="17" t="n">
+        <f aca="false">B17*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="C45" s="17" t="n">
+        <f aca="false">C17*(1-$B$8)</f>
+        <v>4750</v>
+      </c>
+      <c r="D45" s="17" t="n">
+        <f aca="false">D17*(1-$B$8)</f>
+        <v>4750</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B46" s="12" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(B24*(1-B24)*(1/B44+1/B43))</f>
-        <v>0.0144700477174636</v>
+        <f aca="false">(B45*B25+B44*B27)/(B45+B44)</f>
+        <v>0.0545000000000001</v>
       </c>
       <c r="C46" s="12" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(C24*(1-C24)*(1/C44+1/C43))</f>
-        <v>0.0113258199429158</v>
+        <f aca="false">(C45*C25+C44*C27)/(C45+C44)</f>
+        <v>0.03135</v>
       </c>
       <c r="D46" s="12" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(D24*(1-D24)*(1/D44+1/D43))</f>
-        <v>0.00660603325734122</v>
+        <f aca="false">(D45*D25+D44*D27)/(D45+D44)</f>
+        <v>0.00955000000000001</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B47" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B46))/(B44+B43))*(1-((B44*B24+B43*(B24+B46))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B46)*(1-B24-B46)/B43)</f>
-        <v>0.0154205904175831</v>
+        <f aca="false">($B$10+$B$11)*SQRT(B25*(1-B25)*(1/B45+1/B44))</f>
+        <v>0.0144700477174636</v>
       </c>
       <c r="C47" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C46))/(C44+C43))*(1-((C44*C24+C43*(C24+C46))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C46)*(1-C24-C46)/C43)</f>
-        <v>0.0123109990740818</v>
+        <f aca="false">($B$10+$B$11)*SQRT(C25*(1-C25)*(1/C45+1/C44))</f>
+        <v>0.0113258199429158</v>
       </c>
       <c r="D47" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D46))/(D44+D43))*(1-((D44*D24+D43*(D24+D46))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D46)*(1-D24-D46)/D43)</f>
-        <v>0.00760576962692852</v>
-      </c>
-      <c r="E47" s="2"/>
+        <f aca="false">($B$10+$B$11)*SQRT(D25*(1-D25)*(1/D45+1/D44))</f>
+        <v>0.00660603325734122</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>84</v>
+      </c>
       <c r="F47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B48" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B47))/(B44+B43))*(1-((B44*B24+B43*(B24+B47))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B47)*(1-B24-B47)/B43)</f>
-        <v>0.0154803316438639</v>
+        <f aca="false">$B$10*SQRT(((B45*B25+B44*(B25+B47))/(B45+B44))*(1-((B45*B25+B44*(B25+B47))/(B45+B44)))*(1/B45+1/B44))+$B$11*SQRT(B25*(1-B25)/B45+(B25+B47)*(1-B25-B47)/B44)</f>
+        <v>0.0154205904175831</v>
       </c>
       <c r="C48" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C47))/(C44+C43))*(1-((C44*C24+C43*(C24+C47))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C47)*(1-C24-C47)/C43)</f>
-        <v>0.012392313574853</v>
+        <f aca="false">$B$10*SQRT(((C45*C25+C44*(C25+C47))/(C45+C44))*(1-((C45*C25+C44*(C25+C47))/(C45+C44)))*(1/C45+1/C44))+$B$11*SQRT(C25*(1-C25)/C45+(C25+C47)*(1-C25-C47)/C44)</f>
+        <v>0.0123109990740818</v>
       </c>
       <c r="D48" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D47))/(D44+D43))*(1-((D44*D24+D43*(D24+D47))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D47)*(1-D24-D47)/D43)</f>
-        <v>0.00774515165979732</v>
+        <f aca="false">$B$10*SQRT(((D45*D25+D44*(D25+D47))/(D45+D44))*(1-((D45*D25+D44*(D25+D47))/(D45+D44)))*(1/D45+1/D44))+$B$11*SQRT(D25*(1-D25)/D45+(D25+D47)*(1-D25-D47)/D44)</f>
+        <v>0.00760576962692852</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B49" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B48))/(B44+B43))*(1-((B44*B24+B43*(B24+B48))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B48)*(1-B24-B48)/B43)</f>
-        <v>0.015484075950343</v>
+        <f aca="false">$B$10*SQRT(((B45*B25+B44*(B25+B48))/(B45+B44))*(1-((B45*B25+B44*(B25+B48))/(B45+B44)))*(1/B45+1/B44))+$B$11*SQRT(B25*(1-B25)/B45+(B25+B48)*(1-B25-B48)/B44)</f>
+        <v>0.0154803316438639</v>
       </c>
       <c r="C49" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C48))/(C44+C43))*(1-((C44*C24+C43*(C24+C48))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C48)*(1-C24-C48)/C43)</f>
-        <v>0.0123989964120841</v>
+        <f aca="false">$B$10*SQRT(((C45*C25+C44*(C25+C48))/(C45+C44))*(1-((C45*C25+C44*(C25+C48))/(C45+C44)))*(1/C45+1/C44))+$B$11*SQRT(C25*(1-C25)/C45+(C25+C48)*(1-C25-C48)/C44)</f>
+        <v>0.012392313574853</v>
       </c>
       <c r="D49" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D48))/(D44+D43))*(1-((D44*D24+D43*(D24+D48))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D48)*(1-D24-D48)/D43)</f>
-        <v>0.00776437119734043</v>
+        <f aca="false">$B$10*SQRT(((D45*D25+D44*(D25+D48))/(D45+D44))*(1-((D45*D25+D44*(D25+D48))/(D45+D44)))*(1/D45+1/D44))+$B$11*SQRT(D25*(1-D25)/D45+(D25+D48)*(1-D25-D48)/D44)</f>
+        <v>0.00774515165979732</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B50" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((B44*B24+B43*(B24+B49))/(B44+B43))*(1-((B44*B24+B43*(B24+B49))/(B44+B43)))*(1/B44+1/B43))+$B$11*SQRT(B24*(1-B24)/B44+(B24+B49)*(1-B24-B49)/B43)</f>
+        <f aca="false">$B$10*SQRT(((B45*B25+B44*(B25+B49))/(B45+B44))*(1-((B45*B25+B44*(B25+B49))/(B45+B44)))*(1/B45+1/B44))+$B$11*SQRT(B25*(1-B25)/B45+(B25+B49)*(1-B25-B49)/B44)</f>
+        <v>0.015484075950343</v>
+      </c>
+      <c r="C50" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((C45*C25+C44*(C25+C49))/(C45+C44))*(1-((C45*C25+C44*(C25+C49))/(C45+C44)))*(1/C45+1/C44))+$B$11*SQRT(C25*(1-C25)/C45+(C25+C49)*(1-C25-C49)/C44)</f>
+        <v>0.0123989964120841</v>
+      </c>
+      <c r="D50" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((D45*D25+D44*(D25+D49))/(D45+D44))*(1-((D45*D25+D44*(D25+D49))/(D45+D44)))*(1/D45+1/D44))+$B$11*SQRT(D25*(1-D25)/D45+(D25+D49)*(1-D25-D49)/D44)</f>
+        <v>0.00776437119734043</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((B45*B25+B44*(B25+B50))/(B45+B44))*(1-((B45*B25+B44*(B25+B50))/(B45+B44)))*(1/B45+1/B44))+$B$11*SQRT(B25*(1-B25)/B45+(B25+B50)*(1-B25-B50)/B44)</f>
         <v>0.0154843105855124</v>
       </c>
-      <c r="C50" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((C44*C24+C43*(C24+C49))/(C44+C43))*(1-((C44*C24+C43*(C24+C49))/(C44+C43)))*(1/C44+1/C43))+$B$11*SQRT(C24*(1-C24)/C44+(C24+C49)*(1-C24-C49)/C43)</f>
+      <c r="C51" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((C45*C25+C44*(C25+C50))/(C45+C44))*(1-((C45*C25+C44*(C25+C50))/(C45+C44)))*(1/C45+1/C44))+$B$11*SQRT(C25*(1-C25)/C45+(C25+C50)*(1-C25-C50)/C44)</f>
         <v>0.0123995454483646</v>
       </c>
-      <c r="D50" s="12" t="n">
-        <f aca="false">$B$10*SQRT(((D44*D24+D43*(D24+D49))/(D44+D43))*(1-((D44*D24+D43*(D24+D49))/(D44+D43)))*(1/D44+1/D43))+$B$11*SQRT(D24*(1-D24)/D44+(D24+D49)*(1-D24-D49)/D43)</f>
+      <c r="D51" s="12" t="n">
+        <f aca="false">$B$10*SQRT(((D45*D25+D44*(D25+D50))/(D45+D44))*(1-((D45*D25+D44*(D25+D50))/(D45+D44)))*(1/D45+1/D44))+$B$11*SQRT(D25*(1-D25)/D45+(D25+D50)*(1-D25-D50)/D44)</f>
         <v>0.00776701739625667</v>
       </c>
-      <c r="E50" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="F50" s="2"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
+      <c r="E51" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="F51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="B52" s="21" t="s">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B53" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C52" s="21" t="s">
+      <c r="C53" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D52" s="21" t="s">
+      <c r="D53" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E52" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="F52" s="2"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
+      <c r="E53" s="22" t="s">
+        <v>91</v>
+      </c>
       <c r="F53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="B54" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A54)*(1+B$25),0.999)-(1-(1-B$23)^$A54))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A54)+B$43*MIN((1-(1-B$23)^$A54)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A54)+B$43*MIN((1-(1-B$23)^$A54)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A54)*(1-(1-(1-B$23)^$A54))/B$44+MIN((1-(1-B$23)^$A54)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A54)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.322076256263711</v>
-      </c>
-      <c r="C54" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A54)*(1+C$25),0.999)-(1-(1-C$23)^$A54))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A54)+C$43*MIN((1-(1-C$23)^$A54)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A54)+C$43*MIN((1-(1-C$23)^$A54)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A54)*(1-(1-(1-C$23)^$A54))/C$44+MIN((1-(1-C$23)^$A54)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A54)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.0506120133084721</v>
-      </c>
-      <c r="D54" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A54)*(1+D$25),0.999)-(1-(1-D$23)^$A54))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A54)+D$43*MIN((1-(1-D$23)^$A54)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A54)+D$43*MIN((1-(1-D$23)^$A54)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A54)*(1-(1-(1-D$23)^$A54))/D$44+MIN((1-(1-D$23)^$A54)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A54)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.0260067764439741</v>
-      </c>
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B55" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A55)*(1+B$25),0.999)-(1-(1-B$23)^$A55))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A55)+B$43*MIN((1-(1-B$23)^$A55)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A55)+B$43*MIN((1-(1-B$23)^$A55)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A55)*(1-(1-(1-B$23)^$A55))/B$44+MIN((1-(1-B$23)^$A55)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A55)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.648530625309196</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A55)*(1+B$26),0.999)-(1-(1-B$24)^$A55))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A55)+B$44*MIN((1-(1-B$24)^$A55)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A55)+B$44*MIN((1-(1-B$24)^$A55)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A55)*(1-(1-(1-B$24)^$A55))/B$45+MIN((1-(1-B$24)^$A55)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A55)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.322076256263711</v>
       </c>
       <c r="C55" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A55)*(1+C$25),0.999)-(1-(1-C$23)^$A55))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A55)+C$43*MIN((1-(1-C$23)^$A55)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A55)+C$43*MIN((1-(1-C$23)^$A55)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A55)*(1-(1-(1-C$23)^$A55))/C$44+MIN((1-(1-C$23)^$A55)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A55)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.0938830966435802</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A55)*(1+C$26),0.999)-(1-(1-C$24)^$A55))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A55)+C$44*MIN((1-(1-C$24)^$A55)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A55)+C$44*MIN((1-(1-C$24)^$A55)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A55)*(1-(1-(1-C$24)^$A55))/C$45+MIN((1-(1-C$24)^$A55)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A55)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.0506120133084721</v>
       </c>
       <c r="D55" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A55)*(1+D$25),0.999)-(1-(1-D$23)^$A55))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A55)+D$43*MIN((1-(1-D$23)^$A55)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A55)+D$43*MIN((1-(1-D$23)^$A55)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A55)*(1-(1-(1-D$23)^$A55))/D$44+MIN((1-(1-D$23)^$A55)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A55)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.039648899805351</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A55)*(1+D$26),0.999)-(1-(1-D$24)^$A55))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A55)+D$44*MIN((1-(1-D$24)^$A55)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A55)+D$44*MIN((1-(1-D$24)^$A55)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A55)*(1-(1-(1-D$24)^$A55))/D$45+MIN((1-(1-D$24)^$A55)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A55)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.0260067764439741</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B56" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A56)*(1+B$25),0.999)-(1-(1-B$23)^$A56))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A56)+B$43*MIN((1-(1-B$23)^$A56)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A56)+B$43*MIN((1-(1-B$23)^$A56)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A56)*(1-(1-(1-B$23)^$A56))/B$44+MIN((1-(1-B$23)^$A56)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A56)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.855324473869813</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A56)*(1+B$26),0.999)-(1-(1-B$24)^$A56))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A56)+B$44*MIN((1-(1-B$24)^$A56)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A56)+B$44*MIN((1-(1-B$24)^$A56)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A56)*(1-(1-(1-B$24)^$A56))/B$45+MIN((1-(1-B$24)^$A56)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A56)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.648530625309196</v>
       </c>
       <c r="C56" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A56)*(1+C$25),0.999)-(1-(1-C$23)^$A56))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A56)+C$43*MIN((1-(1-C$23)^$A56)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A56)+C$43*MIN((1-(1-C$23)^$A56)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A56)*(1-(1-(1-C$23)^$A56))/C$44+MIN((1-(1-C$23)^$A56)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A56)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.143659104798111</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A56)*(1+C$26),0.999)-(1-(1-C$24)^$A56))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A56)+C$44*MIN((1-(1-C$24)^$A56)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A56)+C$44*MIN((1-(1-C$24)^$A56)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A56)*(1-(1-(1-C$24)^$A56))/C$45+MIN((1-(1-C$24)^$A56)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A56)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.0938830966435802</v>
       </c>
       <c r="D56" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A56)*(1+D$25),0.999)-(1-(1-D$23)^$A56))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A56)+D$43*MIN((1-(1-D$23)^$A56)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A56)+D$43*MIN((1-(1-D$23)^$A56)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A56)*(1-(1-(1-D$23)^$A56))/D$44+MIN((1-(1-D$23)^$A56)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A56)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.0537724436545908</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A56)*(1+D$26),0.999)-(1-(1-D$24)^$A56))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A56)+D$44*MIN((1-(1-D$24)^$A56)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A56)+D$44*MIN((1-(1-D$24)^$A56)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A56)*(1-(1-(1-D$24)^$A56))/D$45+MIN((1-(1-D$24)^$A56)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A56)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.039648899805351</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B57" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A57)*(1+B$25),0.999)-(1-(1-B$23)^$A57))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A57)+B$43*MIN((1-(1-B$23)^$A57)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A57)+B$43*MIN((1-(1-B$23)^$A57)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A57)*(1-(1-(1-B$23)^$A57))/B$44+MIN((1-(1-B$23)^$A57)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A57)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.951427708514472</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A57)*(1+B$26),0.999)-(1-(1-B$24)^$A57))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A57)+B$44*MIN((1-(1-B$24)^$A57)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A57)+B$44*MIN((1-(1-B$24)^$A57)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A57)*(1-(1-(1-B$24)^$A57))/B$45+MIN((1-(1-B$24)^$A57)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A57)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.855324473869813</v>
       </c>
       <c r="C57" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A57)*(1+C$25),0.999)-(1-(1-C$23)^$A57))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A57)+C$43*MIN((1-(1-C$23)^$A57)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A57)+C$43*MIN((1-(1-C$23)^$A57)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A57)*(1-(1-(1-C$23)^$A57))/C$44+MIN((1-(1-C$23)^$A57)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A57)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.199017743143467</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A57)*(1+C$26),0.999)-(1-(1-C$24)^$A57))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A57)+C$44*MIN((1-(1-C$24)^$A57)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A57)+C$44*MIN((1-(1-C$24)^$A57)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A57)*(1-(1-(1-C$24)^$A57))/C$45+MIN((1-(1-C$24)^$A57)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A57)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.143659104798111</v>
       </c>
       <c r="D57" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A57)*(1+D$25),0.999)-(1-(1-D$23)^$A57))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A57)+D$43*MIN((1-(1-D$23)^$A57)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A57)+D$43*MIN((1-(1-D$23)^$A57)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A57)*(1-(1-(1-D$23)^$A57))/D$44+MIN((1-(1-D$23)^$A57)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A57)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.0686574926403583</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A57)*(1+D$26),0.999)-(1-(1-D$24)^$A57))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A57)+D$44*MIN((1-(1-D$24)^$A57)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A57)+D$44*MIN((1-(1-D$24)^$A57)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A57)*(1-(1-(1-D$24)^$A57))/D$45+MIN((1-(1-D$24)^$A57)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A57)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.0537724436545908</v>
       </c>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B58" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A58)*(1+B$25),0.999)-(1-(1-B$23)^$A58))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A58)+B$43*MIN((1-(1-B$23)^$A58)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A58)+B$43*MIN((1-(1-B$23)^$A58)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A58)*(1-(1-(1-B$23)^$A58))/B$44+MIN((1-(1-B$23)^$A58)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A58)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.986534104343037</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A58)*(1+B$26),0.999)-(1-(1-B$24)^$A58))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A58)+B$44*MIN((1-(1-B$24)^$A58)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A58)+B$44*MIN((1-(1-B$24)^$A58)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A58)*(1-(1-(1-B$24)^$A58))/B$45+MIN((1-(1-B$24)^$A58)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A58)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.951427708514472</v>
       </c>
       <c r="C58" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A58)*(1+C$25),0.999)-(1-(1-C$23)^$A58))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A58)+C$43*MIN((1-(1-C$23)^$A58)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A58)+C$43*MIN((1-(1-C$23)^$A58)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A58)*(1-(1-(1-C$23)^$A58))/C$44+MIN((1-(1-C$23)^$A58)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A58)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.258692789591655</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A58)*(1+C$26),0.999)-(1-(1-C$24)^$A58))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A58)+C$44*MIN((1-(1-C$24)^$A58)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A58)+C$44*MIN((1-(1-C$24)^$A58)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A58)*(1-(1-(1-C$24)^$A58))/C$45+MIN((1-(1-C$24)^$A58)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A58)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.199017743143467</v>
       </c>
       <c r="D58" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A58)*(1+D$25),0.999)-(1-(1-D$23)^$A58))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A58)+D$43*MIN((1-(1-D$23)^$A58)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A58)+D$43*MIN((1-(1-D$23)^$A58)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A58)*(1-(1-(1-D$23)^$A58))/D$44+MIN((1-(1-D$23)^$A58)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A58)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.084357351243645</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A58)*(1+D$26),0.999)-(1-(1-D$24)^$A58))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A58)+D$44*MIN((1-(1-D$24)^$A58)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A58)+D$44*MIN((1-(1-D$24)^$A58)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A58)*(1-(1-(1-D$24)^$A58))/D$45+MIN((1-(1-D$24)^$A58)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A58)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.0686574926403583</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B59" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A59)*(1+B$25),0.999)-(1-(1-B$23)^$A59))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A59)+B$43*MIN((1-(1-B$23)^$A59)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A59)+B$43*MIN((1-(1-B$23)^$A59)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A59)*(1-(1-(1-B$23)^$A59))/B$44+MIN((1-(1-B$23)^$A59)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A59)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.996905244060923</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A59)*(1+B$26),0.999)-(1-(1-B$24)^$A59))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A59)+B$44*MIN((1-(1-B$24)^$A59)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A59)+B$44*MIN((1-(1-B$24)^$A59)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A59)*(1-(1-(1-B$24)^$A59))/B$45+MIN((1-(1-B$24)^$A59)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A59)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.986534104343037</v>
       </c>
       <c r="C59" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A59)*(1+C$25),0.999)-(1-(1-C$23)^$A59))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A59)+C$43*MIN((1-(1-C$23)^$A59)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A59)+C$43*MIN((1-(1-C$23)^$A59)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A59)*(1-(1-(1-C$23)^$A59))/C$44+MIN((1-(1-C$23)^$A59)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A59)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.321309020930109</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A59)*(1+C$26),0.999)-(1-(1-C$24)^$A59))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A59)+C$44*MIN((1-(1-C$24)^$A59)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A59)+C$44*MIN((1-(1-C$24)^$A59)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A59)*(1-(1-(1-C$24)^$A59))/C$45+MIN((1-(1-C$24)^$A59)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A59)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.258692789591655</v>
       </c>
       <c r="D59" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A59)*(1+D$25),0.999)-(1-(1-D$23)^$A59))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A59)+D$43*MIN((1-(1-D$23)^$A59)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A59)+D$43*MIN((1-(1-D$23)^$A59)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A59)*(1-(1-(1-D$23)^$A59))/D$44+MIN((1-(1-D$23)^$A59)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A59)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.10086207082924</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A59)*(1+D$26),0.999)-(1-(1-D$24)^$A59))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A59)+D$44*MIN((1-(1-D$24)^$A59)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A59)+D$44*MIN((1-(1-D$24)^$A59)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A59)*(1-(1-(1-D$24)^$A59))/D$45+MIN((1-(1-D$24)^$A59)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A59)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.084357351243645</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B60" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A60)*(1+B$25),0.999)-(1-(1-B$23)^$A60))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A60)+B$43*MIN((1-(1-B$23)^$A60)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A60)+B$43*MIN((1-(1-B$23)^$A60)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A60)*(1-(1-(1-B$23)^$A60))/B$44+MIN((1-(1-B$23)^$A60)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A60)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.999411332147072</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A60)*(1+B$26),0.999)-(1-(1-B$24)^$A60))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A60)+B$44*MIN((1-(1-B$24)^$A60)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A60)+B$44*MIN((1-(1-B$24)^$A60)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A60)*(1-(1-(1-B$24)^$A60))/B$45+MIN((1-(1-B$24)^$A60)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A60)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.996905244060923</v>
       </c>
       <c r="C60" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A60)*(1+C$25),0.999)-(1-(1-C$23)^$A60))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A60)+C$43*MIN((1-(1-C$23)^$A60)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A60)+C$43*MIN((1-(1-C$23)^$A60)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A60)*(1-(1-(1-C$23)^$A60))/C$44+MIN((1-(1-C$23)^$A60)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A60)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.385471506279525</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A60)*(1+C$26),0.999)-(1-(1-C$24)^$A60))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A60)+C$44*MIN((1-(1-C$24)^$A60)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A60)+C$44*MIN((1-(1-C$24)^$A60)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A60)*(1-(1-(1-C$24)^$A60))/C$45+MIN((1-(1-C$24)^$A60)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A60)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.321309020930109</v>
       </c>
       <c r="D60" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A60)*(1+D$25),0.999)-(1-(1-D$23)^$A60))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A60)+D$43*MIN((1-(1-D$23)^$A60)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A60)+D$43*MIN((1-(1-D$23)^$A60)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A60)*(1-(1-(1-D$23)^$A60))/D$44+MIN((1-(1-D$23)^$A60)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A60)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.118136637139437</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A60)*(1+D$26),0.999)-(1-(1-D$24)^$A60))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A60)+D$44*MIN((1-(1-D$24)^$A60)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A60)+D$44*MIN((1-(1-D$24)^$A60)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A60)*(1-(1-(1-D$24)^$A60))/D$45+MIN((1-(1-D$24)^$A60)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A60)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.10086207082924</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B61" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A61)*(1+B$25),0.999)-(1-(1-B$23)^$A61))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A61)+B$43*MIN((1-(1-B$23)^$A61)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A61)+B$43*MIN((1-(1-B$23)^$A61)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A61)*(1-(1-(1-B$23)^$A61))/B$44+MIN((1-(1-B$23)^$A61)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A61)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.999907837749006</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A61)*(1+B$26),0.999)-(1-(1-B$24)^$A61))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A61)+B$44*MIN((1-(1-B$24)^$A61)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A61)+B$44*MIN((1-(1-B$24)^$A61)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A61)*(1-(1-(1-B$24)^$A61))/B$45+MIN((1-(1-B$24)^$A61)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A61)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.999411332147072</v>
       </c>
       <c r="C61" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A61)*(1+C$25),0.999)-(1-(1-C$23)^$A61))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A61)+C$43*MIN((1-(1-C$23)^$A61)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A61)+C$43*MIN((1-(1-C$23)^$A61)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A61)*(1-(1-(1-C$23)^$A61))/C$44+MIN((1-(1-C$23)^$A61)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A61)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.449827485387897</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A61)*(1+C$26),0.999)-(1-(1-C$24)^$A61))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A61)+C$44*MIN((1-(1-C$24)^$A61)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A61)+C$44*MIN((1-(1-C$24)^$A61)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A61)*(1-(1-(1-C$24)^$A61))/C$45+MIN((1-(1-C$24)^$A61)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A61)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.385471506279525</v>
       </c>
       <c r="D61" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A61)*(1+D$25),0.999)-(1-(1-D$23)^$A61))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A61)+D$43*MIN((1-(1-D$23)^$A61)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A61)+D$43*MIN((1-(1-D$23)^$A61)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A61)*(1-(1-(1-D$23)^$A61))/D$44+MIN((1-(1-D$23)^$A61)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A61)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.13613395893133</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A61)*(1+D$26),0.999)-(1-(1-D$24)^$A61))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A61)+D$44*MIN((1-(1-D$24)^$A61)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A61)+D$44*MIN((1-(1-D$24)^$A61)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A61)*(1-(1-(1-D$24)^$A61))/D$45+MIN((1-(1-D$24)^$A61)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A61)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.118136637139437</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="26" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B62" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A62)*(1+B$25),0.999)-(1-(1-B$23)^$A62))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A62)+B$43*MIN((1-(1-B$23)^$A62)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A62)+B$43*MIN((1-(1-B$23)^$A62)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A62)*(1-(1-(1-B$23)^$A62))/B$44+MIN((1-(1-B$23)^$A62)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A62)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.999988227140586</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A62)*(1+B$26),0.999)-(1-(1-B$24)^$A62))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A62)+B$44*MIN((1-(1-B$24)^$A62)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A62)+B$44*MIN((1-(1-B$24)^$A62)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A62)*(1-(1-(1-B$24)^$A62))/B$45+MIN((1-(1-B$24)^$A62)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A62)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.999907837749006</v>
       </c>
       <c r="C62" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A62)*(1+C$25),0.999)-(1-(1-C$23)^$A62))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A62)+C$43*MIN((1-(1-C$23)^$A62)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A62)+C$43*MIN((1-(1-C$23)^$A62)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A62)*(1-(1-(1-C$23)^$A62))/C$44+MIN((1-(1-C$23)^$A62)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A62)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.513116896204362</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A62)*(1+C$26),0.999)-(1-(1-C$24)^$A62))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A62)+C$44*MIN((1-(1-C$24)^$A62)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A62)+C$44*MIN((1-(1-C$24)^$A62)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A62)*(1-(1-(1-C$24)^$A62))/C$45+MIN((1-(1-C$24)^$A62)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A62)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.449827485387897</v>
       </c>
       <c r="D62" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A62)*(1+D$25),0.999)-(1-(1-D$23)^$A62))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A62)+D$43*MIN((1-(1-D$23)^$A62)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A62)+D$43*MIN((1-(1-D$23)^$A62)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A62)*(1-(1-(1-D$23)^$A62))/D$44+MIN((1-(1-D$23)^$A62)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A62)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.15480036499496</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A62)*(1+D$26),0.999)-(1-(1-D$24)^$A62))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A62)+D$44*MIN((1-(1-D$24)^$A62)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A62)+D$44*MIN((1-(1-D$24)^$A62)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A62)*(1-(1-(1-D$24)^$A62))/D$45+MIN((1-(1-D$24)^$A62)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A62)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.13613395893133</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B63" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A63)*(1+B$25),0.999)-(1-(1-B$23)^$A63))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A63)+B$43*MIN((1-(1-B$23)^$A63)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A63)+B$43*MIN((1-(1-B$23)^$A63)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A63)*(1-(1-(1-B$23)^$A63))/B$44+MIN((1-(1-B$23)^$A63)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A63)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.999998787016377</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A63)*(1+B$26),0.999)-(1-(1-B$24)^$A63))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A63)+B$44*MIN((1-(1-B$24)^$A63)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A63)+B$44*MIN((1-(1-B$24)^$A63)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A63)*(1-(1-(1-B$24)^$A63))/B$45+MIN((1-(1-B$24)^$A63)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A63)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.999988227140586</v>
       </c>
       <c r="C63" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A63)*(1+C$25),0.999)-(1-(1-C$23)^$A63))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A63)+C$43*MIN((1-(1-C$23)^$A63)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A63)+C$43*MIN((1-(1-C$23)^$A63)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A63)*(1-(1-(1-C$23)^$A63))/C$44+MIN((1-(1-C$23)^$A63)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A63)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.574213765368228</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A63)*(1+C$26),0.999)-(1-(1-C$24)^$A63))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A63)+C$44*MIN((1-(1-C$24)^$A63)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A63)+C$44*MIN((1-(1-C$24)^$A63)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A63)*(1-(1-(1-C$24)^$A63))/C$45+MIN((1-(1-C$24)^$A63)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A63)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.513116896204362</v>
       </c>
       <c r="D63" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A63)*(1+D$25),0.999)-(1-(1-D$23)^$A63))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A63)+D$43*MIN((1-(1-D$23)^$A63)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A63)+D$43*MIN((1-(1-D$23)^$A63)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A63)*(1-(1-(1-D$23)^$A63))/D$44+MIN((1-(1-D$23)^$A63)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A63)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.174078332095706</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A63)*(1+D$26),0.999)-(1-(1-D$24)^$A63))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A63)+D$44*MIN((1-(1-D$24)^$A63)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A63)+D$44*MIN((1-(1-D$24)^$A63)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A63)*(1-(1-(1-D$24)^$A63))/D$45+MIN((1-(1-D$24)^$A63)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A63)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.15480036499496</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="26" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B64" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A64)*(1+B$25),0.999)-(1-(1-B$23)^$A64))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A64)+B$43*MIN((1-(1-B$23)^$A64)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A64)+B$43*MIN((1-(1-B$23)^$A64)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A64)*(1-(1-(1-B$23)^$A64))/B$44+MIN((1-(1-B$23)^$A64)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A64)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.999999900613897</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A64)*(1+B$26),0.999)-(1-(1-B$24)^$A64))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A64)+B$44*MIN((1-(1-B$24)^$A64)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A64)+B$44*MIN((1-(1-B$24)^$A64)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A64)*(1-(1-(1-B$24)^$A64))/B$45+MIN((1-(1-B$24)^$A64)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A64)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.999998787016377</v>
       </c>
       <c r="C64" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A64)*(1+C$25),0.999)-(1-(1-C$23)^$A64))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A64)+C$43*MIN((1-(1-C$23)^$A64)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A64)+C$43*MIN((1-(1-C$23)^$A64)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A64)*(1-(1-(1-C$23)^$A64))/C$44+MIN((1-(1-C$23)^$A64)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A64)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.632158101020602</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A64)*(1+C$26),0.999)-(1-(1-C$24)^$A64))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A64)+C$44*MIN((1-(1-C$24)^$A64)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A64)+C$44*MIN((1-(1-C$24)^$A64)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A64)*(1-(1-(1-C$24)^$A64))/C$45+MIN((1-(1-C$24)^$A64)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A64)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.574213765368228</v>
       </c>
       <c r="D64" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A64)*(1+D$25),0.999)-(1-(1-D$23)^$A64))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A64)+D$43*MIN((1-(1-D$23)^$A64)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A64)+D$43*MIN((1-(1-D$23)^$A64)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A64)*(1-(1-(1-D$23)^$A64))/D$44+MIN((1-(1-D$23)^$A64)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A64)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.193908029867781</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A64)*(1+D$26),0.999)-(1-(1-D$24)^$A64))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A64)+D$44*MIN((1-(1-D$24)^$A64)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A64)+D$44*MIN((1-(1-D$24)^$A64)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A64)*(1-(1-(1-D$24)^$A64))/D$45+MIN((1-(1-D$24)^$A64)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A64)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.174078332095706</v>
       </c>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="26" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B65" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$23)^$A65)*(1+B$25),0.999)-(1-(1-B$23)^$A65))-$B$10*SQRT(((B$44*(1-(1-B$23)^$A65)+B$43*MIN((1-(1-B$23)^$A65)*(1+B$25),0.999))/(B$44+B$43))*(1-((B$44*(1-(1-B$23)^$A65)+B$43*MIN((1-(1-B$23)^$A65)*(1+B$25),0.999))/(B$44+B$43)))*(1/B$44+1/B$43)))/SQRT((1-(1-B$23)^$A65)*(1-(1-(1-B$23)^$A65))/B$44+MIN((1-(1-B$23)^$A65)*(1+B$25),0.999)*(1-MIN((1-(1-B$23)^$A65)*(1+B$25),0.999))/B$43)),0)</f>
-        <v>0.999999993632062</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A65)*(1+B$26),0.999)-(1-(1-B$24)^$A65))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A65)+B$44*MIN((1-(1-B$24)^$A65)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A65)+B$44*MIN((1-(1-B$24)^$A65)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A65)*(1-(1-(1-B$24)^$A65))/B$45+MIN((1-(1-B$24)^$A65)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A65)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.999999900613897</v>
       </c>
       <c r="C65" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$23)^$A65)*(1+C$25),0.999)-(1-(1-C$23)^$A65))-$B$10*SQRT(((C$44*(1-(1-C$23)^$A65)+C$43*MIN((1-(1-C$23)^$A65)*(1+C$25),0.999))/(C$44+C$43))*(1-((C$44*(1-(1-C$23)^$A65)+C$43*MIN((1-(1-C$23)^$A65)*(1+C$25),0.999))/(C$44+C$43)))*(1/C$44+1/C$43)))/SQRT((1-(1-C$23)^$A65)*(1-(1-(1-C$23)^$A65))/C$44+MIN((1-(1-C$23)^$A65)*(1+C$25),0.999)*(1-MIN((1-(1-C$23)^$A65)*(1+C$25),0.999))/C$43)),0)</f>
-        <v>0.686177648758822</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A65)*(1+C$26),0.999)-(1-(1-C$24)^$A65))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A65)+C$44*MIN((1-(1-C$24)^$A65)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A65)+C$44*MIN((1-(1-C$24)^$A65)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A65)*(1-(1-(1-C$24)^$A65))/C$45+MIN((1-(1-C$24)^$A65)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A65)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.632158101020602</v>
       </c>
       <c r="D65" s="16" t="n">
-        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$23)^$A65)*(1+D$25),0.999)-(1-(1-D$23)^$A65))-$B$10*SQRT(((D$44*(1-(1-D$23)^$A65)+D$43*MIN((1-(1-D$23)^$A65)*(1+D$25),0.999))/(D$44+D$43))*(1-((D$44*(1-(1-D$23)^$A65)+D$43*MIN((1-(1-D$23)^$A65)*(1+D$25),0.999))/(D$44+D$43)))*(1/D$44+1/D$43)))/SQRT((1-(1-D$23)^$A65)*(1-(1-(1-D$23)^$A65))/D$44+MIN((1-(1-D$23)^$A65)*(1+D$25),0.999)*(1-MIN((1-(1-D$23)^$A65)*(1+D$25),0.999))/D$43)),0)</f>
-        <v>0.214228302973138</v>
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A65)*(1+D$26),0.999)-(1-(1-D$24)^$A65))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A65)+D$44*MIN((1-(1-D$24)^$A65)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A65)+D$44*MIN((1-(1-D$24)^$A65)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A65)*(1-(1-(1-D$24)^$A65))/D$45+MIN((1-(1-D$24)^$A65)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A65)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.193908029867781</v>
       </c>
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
+      <c r="A66" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="B66" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-B$24)^$A66)*(1+B$26),0.999)-(1-(1-B$24)^$A66))-$B$10*SQRT(((B$45*(1-(1-B$24)^$A66)+B$44*MIN((1-(1-B$24)^$A66)*(1+B$26),0.999))/(B$45+B$44))*(1-((B$45*(1-(1-B$24)^$A66)+B$44*MIN((1-(1-B$24)^$A66)*(1+B$26),0.999))/(B$45+B$44)))*(1/B$45+1/B$44)))/SQRT((1-(1-B$24)^$A66)*(1-(1-(1-B$24)^$A66))/B$45+MIN((1-(1-B$24)^$A66)*(1+B$26),0.999)*(1-MIN((1-(1-B$24)^$A66)*(1+B$26),0.999))/B$44)),0)</f>
+        <v>0.999999993632062</v>
+      </c>
+      <c r="C66" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-C$24)^$A66)*(1+C$26),0.999)-(1-(1-C$24)^$A66))-$B$10*SQRT(((C$45*(1-(1-C$24)^$A66)+C$44*MIN((1-(1-C$24)^$A66)*(1+C$26),0.999))/(C$45+C$44))*(1-((C$45*(1-(1-C$24)^$A66)+C$44*MIN((1-(1-C$24)^$A66)*(1+C$26),0.999))/(C$45+C$44)))*(1/C$45+1/C$44)))/SQRT((1-(1-C$24)^$A66)*(1-(1-(1-C$24)^$A66))/C$45+MIN((1-(1-C$24)^$A66)*(1+C$26),0.999)*(1-MIN((1-(1-C$24)^$A66)*(1+C$26),0.999))/C$44)),0)</f>
+        <v>0.686177648758822</v>
+      </c>
+      <c r="D66" s="16" t="n">
+        <f aca="false">IFERROR(NORMSDIST((ABS(MIN((1-(1-D$24)^$A66)*(1+D$26),0.999)-(1-(1-D$24)^$A66))-$B$10*SQRT(((D$45*(1-(1-D$24)^$A66)+D$44*MIN((1-(1-D$24)^$A66)*(1+D$26),0.999))/(D$45+D$44))*(1-((D$45*(1-(1-D$24)^$A66)+D$44*MIN((1-(1-D$24)^$A66)*(1+D$26),0.999))/(D$45+D$44)))*(1/D$45+1/D$44)))/SQRT((1-(1-D$24)^$A66)*(1-(1-(1-D$24)^$A66))/D$45+MIN((1-(1-D$24)^$A66)*(1+D$26),0.999)*(1-MIN((1-(1-D$24)^$A66)*(1+D$26),0.999))/D$44)),0)</f>
+        <v>0.214228302973138</v>
+      </c>
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="27" t="s">
-        <v>88</v>
-      </c>
-      <c r="B67" s="27"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="27"/>
-      <c r="E67" s="27"/>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
       <c r="F67" s="2"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="27"/>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="27" t="s">
+        <v>92</v>
+      </c>
       <c r="B68" s="27"/>
       <c r="C68" s="27"/>
       <c r="D68" s="27"/>
@@ -2113,18 +2148,18 @@
       <c r="F69" s="2"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
+      <c r="A70" s="27"/>
+      <c r="B70" s="27"/>
+      <c r="C70" s="27"/>
+      <c r="D70" s="27"/>
+      <c r="E70" s="27"/>
       <c r="F70" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A67:E69"/>
+    <mergeCell ref="A68:E70"/>
   </mergeCells>
-  <conditionalFormatting sqref="B32:D32">
+  <conditionalFormatting sqref="B34:D34">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"SÍ"</formula>
     </cfRule>
@@ -2132,12 +2167,20 @@
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B35:D35">
+  <conditionalFormatting sqref="B38:D38">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>LEFT(B35,2)="Sí"</formula>
+      <formula>LEFT(B38,2)="Sí"</formula>
     </cfRule>
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>LEFT(B35,2)="No"</formula>
+      <formula>LEFT(B38,2)="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30:D30">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>LEFT(B30,2)="Sí"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>LEFT(B30,2)="NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2164,28 +2207,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B3" s="11" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B5" s="29" t="n">
         <v>0.1</v>
@@ -2405,7 +2448,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2432,42 +2475,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2475,17 +2518,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2493,7 +2536,7 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calculator v5: drop take-up row, fix minimum-users lookup
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ygiEd3g3fKiFCARJZcKLp
</commit_message>
<xml_diff>
--- a/calculadora-sample-size.xlsx
+++ b/calculadora-sample-size.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="82">
   <si>
     <t xml:space="preserve">Calculadora de poder: experimento de crédito por score (ventana de 1 mes)</t>
   </si>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Tiers que pruebas a la vez</t>
   </si>
   <si>
-    <t xml:space="preserve">2 si pruebas Bueno y Bajo. 1 si pruebas uno solo. 3 si los tres.</t>
+    <t xml:space="preserve">1 si pruebas un solo tier (ej. Excelente). 2 o 3 si corres varios a la vez.</t>
   </si>
   <si>
     <t xml:space="preserve">Pérdidas / inactivos</t>
@@ -80,10 +80,10 @@
     <t xml:space="preserve">Nombre de la métrica (solo etiqueta)</t>
   </si>
   <si>
-    <t xml:space="preserve">Referidor trae referido con loan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lo que cuentas por usuario cada mes: sí/no. Cámbiala cuando quieras; solo ajusta la fila 'Eventos al mes'.</t>
+    <t xml:space="preserve">Referidor trae referido con primer loan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo que cuentas por referidor cada mes (sí/no). Hoy: trajo un referido con primer loan.</t>
   </si>
   <si>
     <t xml:space="preserve">DATOS POR TIER</t>
@@ -104,25 +104,25 @@
     <t xml:space="preserve">Crédito hoy (MXN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lo que todos reciben hoy.</t>
+    <t xml:space="preserve">Lo que se paga hoy por cada primer loan de un referido.</t>
   </si>
   <si>
     <t xml:space="preserve">Crédito nuevo (MXN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lo que recibirá el tratamiento.</t>
+    <t xml:space="preserve">Lo que se pagará en el grupo de tratamiento.</t>
   </si>
   <si>
     <t xml:space="preserve">Referidores potenciales (pool)</t>
   </si>
   <si>
-    <t xml:space="preserve">Tu tabla de usuarios por rango de score.</t>
+    <t xml:space="preserve">Tu tabla por score. Si prefieres, pon solo las personas que ya han referido (y ajusta la fila de eventos).</t>
   </si>
   <si>
     <t xml:space="preserve">Eventos al mes del tier HOY (con 500 MXN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cuántos usuarios del tier cumplen la métrica en un mes. Hoy: 5,000 loans repartidos por tamaño del tier. Si cambias la métrica, cambia este número.</t>
+    <t xml:space="preserve">Primeros loans que trajo el tier el mes pasado. Hoy: 5,000 repartidos por tamaño del tier. Si usas solo gente que ya refirió, pon aquí los loans que trajeron ellos.</t>
   </si>
   <si>
     <t xml:space="preserve">Usuarios en TRATAMIENTO (tú eliges)</t>
@@ -131,16 +131,10 @@
     <t xml:space="preserve">Cuántos reciben el crédito nuevo. El resto del pool queda en control con 500. Si no alcanza, mira la fila 'Mínimo para llegar al poder'.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambio esperado en la métrica entre quienes usan el crédito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tu hipótesis. Positivo si esperas subir, negativo si esperas bajar (Bajo).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Take-up (% que usa el crédito)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pon 100% si no aplica a la métrica o si el crédito se aplica solo.</t>
+    <t xml:space="preserve">Cuánto crees que suban los eventos con el crédito nuevo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tu apuesta. 30% = si hoy traen 100 loans, crees que con el crédito nuevo traerán 130. Negativo si esperas que bajen (Bajo).</t>
   </si>
   <si>
     <t xml:space="preserve">RESULTADOS (1 mes)</t>
@@ -170,10 +164,7 @@
     <t xml:space="preserve">Eventos al mes esperados en control</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambio efectivo en todo el grupo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cambio esperado × take-up. Es lo que de verdad se mide.</t>
+    <t xml:space="preserve">Cambio esperado (relativo)</t>
   </si>
   <si>
     <t xml:space="preserve">Tasa esperada en tratamiento</t>
@@ -188,16 +179,10 @@
     <t xml:space="preserve">¿Detecta el cambio esperado?</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambio mínimo detectable (todo el grupo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con tus usuarios solo ves cambios de este tamaño o mayores.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cambio mínimo detectable entre quienes usan el crédito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lo mismo, corregido por take-up. Compáralo con tu hipótesis.</t>
+    <t xml:space="preserve">Cambio mínimo que sí verías</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con tus usuarios solo ves subidas (o bajadas) de este tamaño o mayores. Si tu apuesta es menor que esto, no alcanza.</t>
   </si>
   <si>
     <t xml:space="preserve">Eventos extra al mes si el cambio es real</t>
@@ -254,6 +239,9 @@
     <t xml:space="preserve">Usa esta tabla para escoger cuántos usuarios meter</t>
   </si>
   <si>
+    <t xml:space="preserve">auxiliar</t>
+  </si>
+  <si>
     <t xml:space="preserve">Supuestos: prueba de dos proporciones, dos colas, grupos de distinto tamaño, ventana de 1 mes. La tasa base asume 1 evento por usuario al mes. Los eventos por tier están repartidos en proporción al tamaño del tier porque solo se conoce el total mensual; cámbialos si tienes el dato real.</t>
   </si>
   <si>
@@ -263,22 +251,22 @@
     <t xml:space="preserve">1. La fila que decides es 'Usuarios en TRATAMIENTO' (fila 21). Todo lo demás ya tiene tus datos.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Mira 'PODER con tus usuarios' (fila 32). Si está en 80% o más, listo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Si no, mira 'Mínimo de usuarios en tratamiento para llegar al poder' (fila 38) y escribe ese número en la fila 21.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. 'Qué hacer' (fila 39) te lo dice en una línea.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Para cambiar la métrica: escribe su nombre en la fila 14 y pon en la fila 20 cuántos usuarios de cada tier la cumplen al mes hoy. Si no depende de usar el crédito, pon take-up 100%.</t>
+    <t xml:space="preserve">2. Mira 'PODER con tus usuarios' (fila 31). Si está en 80% o más, listo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Si no, mira 'Mínimo de usuarios en tratamiento para llegar al poder' (fila 36) y escribe ese número en la fila 21.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. 'Qué hacer' (fila 37) te lo dice en una línea.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Para cambiar la métrica: escribe su nombre en la fila 14 y pon en la fila 20 cuántos usuarios de cada tier la cumplen al mes hoy.</t>
   </si>
   <si>
     <t xml:space="preserve">6. 'Tiers que pruebas a la vez' (B7): pon cuántos tiers corres al mismo tiempo. Si solo uno, pon 1 y el poder sube.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lectura rápida: lo que manda son los EVENTOS en el grupo de tratamiento (fila 28), no los usuarios. Con menos de ~80 eventos al mes casi nada se puede medir en un mes.</t>
+    <t xml:space="preserve">Lectura rápida: lo que manda son los EVENTOS en el grupo de tratamiento (fila 27), no los usuarios. Con menos de ~80 eventos al mes casi nada se puede medir en un mes.</t>
   </si>
 </sst>
 </file>
@@ -297,7 +285,7 @@
     <numFmt numFmtId="172" formatCode="\$#,##0;[RED]&quot;-$&quot;#,##0"/>
     <numFmt numFmtId="173" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -359,6 +347,13 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF999999"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -452,7 +447,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -559,6 +554,10 @@
     </xf>
     <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -683,7 +682,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF555555"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF1F3864"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -877,7 +876,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -935,7 +934,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>10</v>
@@ -958,7 +957,7 @@
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">B5/B7</f>
-        <v>0.025</v>
+        <v>0.05</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>14</v>
@@ -970,7 +969,7 @@
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">NORMSINV(1-B9/2)</f>
-        <v>2.24140272760495</v>
+        <v>1.95996398454005</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1057,7 +1056,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
         <v>30</v>
       </c>
@@ -1096,19 +1095,19 @@
         <v>34</v>
       </c>
       <c r="B21" s="14" t="n">
-        <v>100000</v>
+        <v>281000</v>
       </c>
       <c r="C21" s="14" t="n">
         <v>334192</v>
       </c>
       <c r="D21" s="14" t="n">
-        <v>1000000</v>
+        <v>2327000</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>36</v>
       </c>
@@ -1125,37 +1124,40 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C23" s="10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D23" s="10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E23" s="7" t="s">
+      <c r="B24" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E25" s="4" t="s">
+      <c r="B25" s="15" t="n">
+        <f aca="false">B20/B19</f>
+        <v>0.000820052689719457</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <f aca="false">C20/C19</f>
+        <v>0.000821384114520994</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <f aca="false">D20/D19</f>
+        <v>0.000820727891105308</v>
+      </c>
+      <c r="E25" s="7" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1163,17 +1165,17 @@
       <c r="A26" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="15" t="n">
-        <f aca="false">B20/B19</f>
-        <v>0.000820052689719457</v>
-      </c>
-      <c r="C26" s="15" t="n">
-        <f aca="false">C20/C19</f>
-        <v>0.000821384114520994</v>
-      </c>
-      <c r="D26" s="15" t="n">
-        <f aca="false">D20/D19</f>
-        <v>0.000820727891105308</v>
+      <c r="B26" s="16" t="n">
+        <f aca="false">B19-B21</f>
+        <v>281159</v>
+      </c>
+      <c r="C26" s="16" t="n">
+        <f aca="false">C19-C21</f>
+        <v>334192</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <f aca="false">D19-D21</f>
+        <v>2327405</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>43</v>
@@ -1184,16 +1186,16 @@
         <v>44</v>
       </c>
       <c r="B27" s="16" t="n">
-        <f aca="false">B19-B21</f>
-        <v>462159</v>
+        <f aca="false">B21*B25</f>
+        <v>230.434805811167</v>
       </c>
       <c r="C27" s="16" t="n">
-        <f aca="false">C19-C21</f>
-        <v>334192</v>
+        <f aca="false">C21*C25</f>
+        <v>274.5</v>
       </c>
       <c r="D27" s="16" t="n">
-        <f aca="false">D19-D21</f>
-        <v>3654405</v>
+        <f aca="false">D21*D25</f>
+        <v>1909.83380260205</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>45</v>
@@ -1204,560 +1206,616 @@
         <v>46</v>
       </c>
       <c r="B28" s="16" t="n">
-        <f aca="false">B21*B26</f>
-        <v>82.0052689719457</v>
+        <f aca="false">B26*B25</f>
+        <v>230.565194188833</v>
       </c>
       <c r="C28" s="16" t="n">
-        <f aca="false">C21*C26</f>
+        <f aca="false">C26*C25</f>
         <v>274.5</v>
       </c>
       <c r="D28" s="16" t="n">
-        <f aca="false">D21*D26</f>
-        <v>820.727891105308</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>47</v>
+        <f aca="false">D26*D25</f>
+        <v>1910.16619739795</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29" s="16" t="n">
-        <f aca="false">B27*B26</f>
-        <v>378.994731028054</v>
-      </c>
-      <c r="C29" s="16" t="n">
-        <f aca="false">C27*C26</f>
-        <v>274.5</v>
-      </c>
-      <c r="D29" s="16" t="n">
-        <f aca="false">D27*D26</f>
-        <v>2999.27210889469</v>
+        <v>47</v>
+      </c>
+      <c r="B29" s="17" t="n">
+        <f aca="false">B22</f>
+        <v>0.3</v>
+      </c>
+      <c r="C29" s="17" t="n">
+        <f aca="false">C22</f>
+        <v>0.15</v>
+      </c>
+      <c r="D29" s="17" t="n">
+        <f aca="false">D22</f>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30" s="15" t="n">
+        <f aca="false">B25*(1+B29)</f>
+        <v>0.00106606849663529</v>
+      </c>
+      <c r="C30" s="15" t="n">
+        <f aca="false">C25*(1+C29)</f>
+        <v>0.000944591731699143</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <f aca="false">D25*(1+D29)</f>
+        <v>0.000697618707439512</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="17" t="n">
-        <f aca="false">B22*B23</f>
-        <v>0.18</v>
-      </c>
-      <c r="C30" s="17" t="n">
-        <f aca="false">C22*C23</f>
-        <v>0.09</v>
-      </c>
-      <c r="D30" s="17" t="n">
-        <f aca="false">D22*D23</f>
-        <v>-0.09</v>
-      </c>
-      <c r="E30" s="7" t="s">
+      <c r="B31" s="19" t="n">
+        <f aca="false">IF(OR(B26&lt;=0,B29=0),0,NORMSDIST((ABS(B30-B25)-$B$10*SQRT(B42*(1-B42)*(1/B41+1/B40)))/SQRT(B25*(1-B25)/B41+B30*(1-B30)/B40)))</f>
+        <v>0.833642091009647</v>
+      </c>
+      <c r="C31" s="19" t="n">
+        <f aca="false">IF(OR(C26&lt;=0,C29=0),0,NORMSDIST((ABS(C30-C25)-$B$10*SQRT(C42*(1-C42)*(1/C41+1/C40)))/SQRT(C25*(1-C25)/C41+C30*(1-C30)/C40)))</f>
+        <v>0.379325029852179</v>
+      </c>
+      <c r="D31" s="19" t="n">
+        <f aca="false">IF(OR(D26&lt;=0,D29=0),0,NORMSDIST((ABS(D30-D25)-$B$10*SQRT(D42*(1-D42)*(1/D41+1/D40)))/SQRT(D25*(1-D25)/D41+D30*(1-D30)/D40)))</f>
+        <v>0.996923501492287</v>
+      </c>
+      <c r="E31" s="7" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B31" s="15" t="n">
-        <f aca="false">B26*(1+B30)</f>
-        <v>0.000967662173868959</v>
-      </c>
-      <c r="C31" s="15" t="n">
-        <f aca="false">C26*(1+C30)</f>
-        <v>0.000895308684827884</v>
-      </c>
-      <c r="D31" s="15" t="n">
-        <f aca="false">D26*(1+D30)</f>
-        <v>0.00074686238090583</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="20" t="str">
+        <f aca="false">IF(B31&gt;=$B$6,"SÍ","NO")</f>
+        <v>SÍ</v>
+      </c>
+      <c r="C32" s="20" t="str">
+        <f aca="false">IF(C31&gt;=$B$6,"SÍ","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="D32" s="20" t="str">
+        <f aca="false">IF(D31&gt;=$B$6,"SÍ","NO")</f>
+        <v>SÍ</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B32" s="19" t="n">
-        <f aca="false">IF(OR(B27&lt;=0,B30=0),0,NORMSDIST((ABS(B31-B26)-$B$10*SQRT(B44*(1-B44)*(1/B43+1/B42)))/SQRT(B26*(1-B26)/B43+B31*(1-B31)/B42)))</f>
-        <v>0.217644169186768</v>
-      </c>
-      <c r="C32" s="19" t="n">
-        <f aca="false">IF(OR(C27&lt;=0,C30=0),0,NORMSDIST((ABS(C31-C26)-$B$10*SQRT(C44*(1-C44)*(1/C43+1/C42)))/SQRT(C26*(1-C26)/C43+C31*(1-C31)/C42)))</f>
-        <v>0.108293125392718</v>
-      </c>
-      <c r="D32" s="19" t="n">
-        <f aca="false">IF(OR(D27&lt;=0,D30=0),0,NORMSDIST((ABS(D31-D26)-$B$10*SQRT(D44*(1-D44)*(1/D43+1/D42)))/SQRT(D26*(1-D26)/D43+D31*(1-D31)/D42)))</f>
-        <v>0.503337360450257</v>
-      </c>
-      <c r="E32" s="7" t="s">
+      <c r="B33" s="17" t="n">
+        <f aca="false">IF(B26&lt;=0,"n/a",B47/B25)</f>
+        <v>0.28611986853037</v>
+      </c>
+      <c r="C33" s="17" t="n">
+        <f aca="false">IF(C26&lt;=0,"n/a",C47/C25)</f>
+        <v>0.260730906417824</v>
+      </c>
+      <c r="D33" s="17" t="n">
+        <f aca="false">IF(D26&lt;=0,"n/a",D47/D25)</f>
+        <v>0.0951582685017244</v>
+      </c>
+      <c r="E33" s="7" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="20" t="str">
-        <f aca="false">IF(B32&gt;=$B$6,"SÍ","NO")</f>
-        <v>NO</v>
-      </c>
-      <c r="C33" s="20" t="str">
-        <f aca="false">IF(C32&gt;=$B$6,"SÍ","NO")</f>
-        <v>NO</v>
-      </c>
-      <c r="D33" s="20" t="str">
-        <f aca="false">IF(D32&gt;=$B$6,"SÍ","NO")</f>
-        <v>NO</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="16" t="n">
+        <f aca="false">B27*B29</f>
+        <v>69.1304417433502</v>
+      </c>
+      <c r="C34" s="16" t="n">
+        <f aca="false">C27*C29</f>
+        <v>41.175</v>
+      </c>
+      <c r="D34" s="16" t="n">
+        <f aca="false">D27*D29</f>
+        <v>-286.475070390308</v>
+      </c>
+      <c r="E34" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="17" t="n">
-        <f aca="false">IF(B27&lt;=0,"n/a",B49/B26)</f>
-        <v>0.411612809264785</v>
-      </c>
-      <c r="C34" s="17" t="n">
-        <f aca="false">IF(C27&lt;=0,"n/a",C49/C26)</f>
-        <v>0.288690113308856</v>
-      </c>
-      <c r="D34" s="17" t="n">
-        <f aca="false">IF(D27&lt;=0,"n/a",D49/D26)</f>
-        <v>0.127444376351998</v>
-      </c>
-      <c r="E34" s="7" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
+      <c r="B35" s="21" t="n">
+        <f aca="false">(B27+B34)*(B18-B17)</f>
+        <v>149782.623777259</v>
+      </c>
+      <c r="C35" s="21" t="n">
+        <f aca="false">(C27+C34)*(C18-C17)</f>
+        <v>78918.75</v>
+      </c>
+      <c r="D35" s="21" t="n">
+        <f aca="false">(D27+D34)*(D18-D17)</f>
+        <v>-405839.683052936</v>
+      </c>
+      <c r="E35" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="17" t="n">
-        <f aca="false">IF(ISNUMBER(B34),B34/B23,"n/a")</f>
-        <v>0.686021348774642</v>
-      </c>
-      <c r="C35" s="17" t="n">
-        <f aca="false">IF(ISNUMBER(C34),C34/C23,"n/a")</f>
-        <v>0.481150188848094</v>
-      </c>
-      <c r="D35" s="17" t="n">
-        <f aca="false">IF(ISNUMBER(D34),D34/D23,"n/a")</f>
-        <v>0.212407293919996</v>
-      </c>
-      <c r="E35" s="7" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="18" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
+      <c r="B36" s="22" t="n">
+        <f aca="false">IF(COUNT(F50:F57)=0,"No llega ni con todo el pool",MIN(F50:F57))</f>
+        <v>250000</v>
+      </c>
+      <c r="C36" s="22" t="str">
+        <f aca="false">IF(COUNT(G50:G57)=0,"No llega ni con todo el pool",MIN(G50:G57))</f>
+        <v>No llega ni con todo el pool</v>
+      </c>
+      <c r="D36" s="22" t="n">
+        <f aca="false">IF(COUNT(H50:H57)=0,"No llega ni con todo el pool",MIN(H50:H57))</f>
+        <v>500000</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="16" t="n">
-        <f aca="false">B28*B30</f>
-        <v>14.7609484149502</v>
-      </c>
-      <c r="C36" s="16" t="n">
-        <f aca="false">C28*C30</f>
-        <v>24.705</v>
-      </c>
-      <c r="D36" s="16" t="n">
-        <f aca="false">D28*D30</f>
-        <v>-73.8655101994777</v>
-      </c>
-      <c r="E36" s="7" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+      <c r="B37" s="20" t="str">
+        <f aca="false">IF(B26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(B32="SÍ","Corre con "&amp;TEXT(B21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(B36),"Sube tratamiento a "&amp;TEXT(B36,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
+        <v>Corre con 281,000 en tratamiento.</v>
+      </c>
+      <c r="C37" s="20" t="str">
+        <f aca="false">IF(C26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(C32="SÍ","Corre con "&amp;TEXT(C21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(C36),"Sube tratamiento a "&amp;TEXT(C36,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
+        <v>No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.</v>
+      </c>
+      <c r="D37" s="20" t="str">
+        <f aca="false">IF(D26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(D32="SÍ","Corre con "&amp;TEXT(D21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(D36),"Sube tratamiento a "&amp;TEXT(D36,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
+        <v>Corre con 2,327,000 en tratamiento.</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="21" t="n">
-        <f aca="false">(B28+B36)*(B18-B17)</f>
-        <v>48383.1086934479</v>
-      </c>
-      <c r="C37" s="21" t="n">
-        <f aca="false">(C28+C36)*(C18-C17)</f>
-        <v>74801.25</v>
-      </c>
-      <c r="D37" s="21" t="n">
-        <f aca="false">(D28+D36)*(D18-D17)</f>
-        <v>-186715.595226458</v>
-      </c>
-      <c r="E37" s="7" t="s">
+      <c r="B39" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C39" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" s="24"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="s">
+      <c r="B40" s="16" t="n">
+        <f aca="false">B21*(1-$B$8)</f>
+        <v>266950</v>
+      </c>
+      <c r="C40" s="16" t="n">
+        <f aca="false">C21*(1-$B$8)</f>
+        <v>317482.4</v>
+      </c>
+      <c r="D40" s="16" t="n">
+        <f aca="false">D21*(1-$B$8)</f>
+        <v>2210650</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="22" t="str">
-        <f aca="false">IF(COUNT(B52:B59)=0,"n/a",IF(COUNTIF(B52:B59,"&lt;"&amp;$B$6)=COUNT(B52:B59),"No llega ni con todo el pool",INDEX($A$52:$A$59,COUNTIF(B52:B59,"&lt;"&amp;$B$6)+1)))</f>
-        <v>No llega ni con todo el pool</v>
-      </c>
-      <c r="C38" s="22" t="str">
-        <f aca="false">IF(COUNT(C52:C59)=0,"n/a",IF(COUNTIF(C52:C59,"&lt;"&amp;$B$6)=COUNT(C52:C59),"No llega ni con todo el pool",INDEX($A$52:$A$59,COUNTIF(C52:C59,"&lt;"&amp;$B$6)+1)))</f>
-        <v>No llega ni con todo el pool</v>
-      </c>
-      <c r="D38" s="22" t="str">
-        <f aca="false">IF(COUNT(D52:D59)=0,"n/a",IF(COUNTIF(D52:D59,"&lt;"&amp;$B$6)=COUNT(D52:D59),"No llega ni con todo el pool",INDEX($A$52:$A$59,COUNTIF(D52:D59,"&lt;"&amp;$B$6)+1)))</f>
-        <v>No llega ni con todo el pool</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="B39" s="20" t="str">
-        <f aca="false">IF(B27&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(B33="SÍ","Corre con "&amp;TEXT(B21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(B38),"Sube tratamiento a "&amp;TEXT(B38,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
-        <v>No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.</v>
-      </c>
-      <c r="C39" s="20" t="str">
-        <f aca="false">IF(C27&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(C33="SÍ","Corre con "&amp;TEXT(C21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(C38),"Sube tratamiento a "&amp;TEXT(C38,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
-        <v>No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.</v>
-      </c>
-      <c r="D39" s="20" t="str">
-        <f aca="false">IF(D27&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(D33="SÍ","Corre con "&amp;TEXT(D21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(D38),"Sube tratamiento a "&amp;TEXT(D38,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
-        <v>No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C41" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="D41" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E41" s="24"/>
+      <c r="B41" s="16" t="n">
+        <f aca="false">MAX(B26,1)*(1-$B$8)</f>
+        <v>267101.05</v>
+      </c>
+      <c r="C41" s="16" t="n">
+        <f aca="false">MAX(C26,1)*(1-$B$8)</f>
+        <v>317482.4</v>
+      </c>
+      <c r="D41" s="16" t="n">
+        <f aca="false">MAX(D26,1)*(1-$B$8)</f>
+        <v>2211034.75</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B42" s="16" t="n">
-        <f aca="false">B21*(1-$B$8)</f>
-        <v>95000</v>
-      </c>
-      <c r="C42" s="16" t="n">
-        <f aca="false">C21*(1-$B$8)</f>
-        <v>317482.4</v>
-      </c>
-      <c r="D42" s="16" t="n">
-        <f aca="false">D21*(1-$B$8)</f>
-        <v>950000</v>
+        <v>64</v>
+      </c>
+      <c r="B42" s="25" t="n">
+        <f aca="false">(B41*B25+B40*B30)/(B41+B40)</f>
+        <v>0.000943025801852056</v>
+      </c>
+      <c r="C42" s="25" t="n">
+        <f aca="false">(C41*C25+C40*C30)/(C41+C40)</f>
+        <v>0.000882987923110069</v>
+      </c>
+      <c r="D42" s="25" t="n">
+        <f aca="false">(D41*D25+D40*D30)/(D41+D40)</f>
+        <v>0.000759178655404867</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B43" s="16" t="n">
-        <f aca="false">MAX(B27,1)*(1-$B$8)</f>
-        <v>439051.05</v>
-      </c>
-      <c r="C43" s="16" t="n">
-        <f aca="false">MAX(C27,1)*(1-$B$8)</f>
-        <v>317482.4</v>
-      </c>
-      <c r="D43" s="16" t="n">
-        <f aca="false">MAX(D27,1)*(1-$B$8)</f>
-        <v>3471684.75</v>
+        <v>65</v>
+      </c>
+      <c r="B43" s="25" t="n">
+        <f aca="false">($B$10+$B$11)*SQRT(B25*(1-B25)*(1/B41+1/B40))</f>
+        <v>0.000219475070481767</v>
+      </c>
+      <c r="C43" s="25" t="n">
+        <f aca="false">($B$10+$B$11)*SQRT(C25*(1-C25)*(1/C41+1/C40))</f>
+        <v>0.000201443715395474</v>
+      </c>
+      <c r="D43" s="25" t="n">
+        <f aca="false">($B$10+$B$11)*SQRT(D25*(1-D25)*(1/D41+1/D40))</f>
+        <v>7.63064502860877E-005</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B44" s="25" t="n">
-        <f aca="false">(B43*B26+B42*B31)/(B43+B42)</f>
-        <v>0.000846310293733535</v>
+        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B43))/(B41+B40))*(1-((B41*B25+B40*(B25+B43))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B43)*(1-B25-B43)/B40)</f>
+        <v>0.00023368413016945</v>
       </c>
       <c r="C44" s="25" t="n">
-        <f aca="false">(C43*C26+C42*C31)/(C43+C42)</f>
-        <v>0.000858346399674439</v>
+        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C43))/(C41+C40))*(1-((C41*C25+C40*(C25+C43))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C43)*(1-C25-C43)/C40)</f>
+        <v>0.000213426519316081</v>
       </c>
       <c r="D44" s="25" t="n">
-        <f aca="false">(D43*D26+D42*D31)/(D43+D42)</f>
-        <v>0.000804857869008074</v>
+        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D43))/(D41+D40))*(1-((D41*D25+D40*(D25+D43))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D43)*(1-D25-D43)/D40)</f>
+        <v>7.80583639702972E-005</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B45" s="25" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(B26*(1-B26)*(1/B43+1/B42))</f>
-        <v>0.000315785153121956</v>
+        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B44))/(B41+B40))*(1-((B41*B25+B40*(B25+B44))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B44)*(1-B25-B44)/B40)</f>
+        <v>0.00023457424210403</v>
       </c>
       <c r="C45" s="25" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(C26*(1-C26)*(1/C43+1/C42))</f>
-        <v>0.000221680139293159</v>
+        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C44))/(C41+C40))*(1-((C41*C25+C40*(C25+C44))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C44)*(1-C25-C44)/C40)</f>
+        <v>0.000214118085343449</v>
       </c>
       <c r="D45" s="25" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(D26*(1-D26)*(1/D43+1/D42))</f>
-        <v>0.00010222571308195</v>
+        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D44))/(D41+D40))*(1-((D41*D25+D40*(D25+D44))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D44)*(1-D25-D44)/D40)</f>
+        <v>7.80981225045379E-005</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B46" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B43*B26+B42*(B26+B45))/(B43+B42))*(1-((B43*B26+B42*(B26+B45))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B26*(1-B26)/B43+(B26+B45)*(1-B26-B45)/B42)</f>
-        <v>0.000336206414330931</v>
+        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B45))/(B41+B40))*(1-((B41*B25+B40*(B25+B45))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B45)*(1-B25-B45)/B40)</f>
+        <v>0.00023462988930975</v>
       </c>
       <c r="C46" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C43*C26+C42*(C26+C45))/(C43+C42))*(1-((C43*C26+C42*(C26+C45))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C26*(1-C26)/C43+(C26+C45)*(1-C26-C45)/C42)</f>
-        <v>0.000236150542166816</v>
+        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C45))/(C41+C40))*(1-((C41*C25+C40*(C25+C45))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C45)*(1-C25-C45)/C40)</f>
+        <v>0.00021415792934427</v>
       </c>
       <c r="D46" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D43*D26+D42*(D26+D45))/(D43+D42))*(1-((D43*D26+D42*(D26+D45))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D26*(1-D26)/D43+(D26+D45)*(1-D26-D45)/D42)</f>
-        <v>0.000104544245358493</v>
+        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D45))/(D41+D40))*(1-((D41*D25+D40*(D25+D45))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D45)*(1-D25-D45)/D40)</f>
+        <v>7.80990245625121E-005</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B47" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B46))/(B41+B40))*(1-((B41*B25+B40*(B25+B46))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B46)*(1-B25-B46)/B40)</f>
+        <v>0.000234633367770507</v>
+      </c>
+      <c r="C47" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C46))/(C41+C40))*(1-((C41*C25+C40*(C25+C46))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C46)*(1-C25-C46)/C40)</f>
+        <v>0.00021416022469626</v>
+      </c>
+      <c r="D47" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D46))/(D41+D40))*(1-((D41*D25+D40*(D25+D46))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D46)*(1-D25-D46)/D40)</f>
+        <v>7.80990450286529E-005</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B49" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C49" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="D49" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="E49" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="F49" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B43*B26+B42*(B26+B46))/(B43+B42))*(1-((B43*B26+B42*(B26+B46))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B26*(1-B26)/B43+(B26+B46)*(1-B26-B46)/B42)</f>
-        <v>0.000337462441280728</v>
-      </c>
-      <c r="C47" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C43*C26+C42*(C26+C46))/(C43+C42))*(1-((C43*C26+C42*(C26+C46))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C26*(1-C26)/C43+(C26+C46)*(1-C26-C46)/C42)</f>
-        <v>0.000237064267415081</v>
-      </c>
-      <c r="D47" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D43*D26+D42*(D26+D46))/(D43+D42))*(1-((D43*D26+D42*(D26+D46))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D26*(1-D26)/D43+(D26+D46)*(1-D26-D46)/D42)</f>
-        <v>0.000104595974771253</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B48" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B43*B26+B42*(B26+B47))/(B43+B42))*(1-((B43*B26+B42*(B26+B47))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B26*(1-B26)/B43+(B26+B47)*(1-B26-B47)/B42)</f>
-        <v>0.000337539468435922</v>
-      </c>
-      <c r="C48" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C43*C26+C42*(C26+C47))/(C43+C42))*(1-((C43*C26+C42*(C26+C47))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C26*(1-C26)/C43+(C26+C47)*(1-C26-C47)/C42)</f>
-        <v>0.000237121845320855</v>
-      </c>
-      <c r="D48" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D43*D26+D42*(D26+D47))/(D43+D42))*(1-((D43*D26+D42*(D26+D47))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D26*(1-D26)/D43+(D26+D47)*(1-D26-D47)/D42)</f>
-        <v>0.000104597128504815</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B49" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B43*B26+B42*(B26+B48))/(B43+B42))*(1-((B43*B26+B42*(B26+B48))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B26*(1-B26)/B43+(B26+B48)*(1-B26-B48)/B42)</f>
-        <v>0.000337544191360569</v>
-      </c>
-      <c r="C49" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C43*C26+C42*(C26+C48))/(C43+C42))*(1-((C43*C26+C42*(C26+C48))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C26*(1-C26)/C43+(C26+C48)*(1-C26-C48)/C42)</f>
-        <v>0.00023712547309116</v>
-      </c>
-      <c r="D49" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D43*D26+D42*(D26+D48))/(D43+D42))*(1-((D43*D26+D42*(D26+D48))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D26*(1-D26)/D43+(D26+D48)*(1-D26-D48)/D42)</f>
-        <v>0.000104597154236606</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="B51" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C51" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="D51" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E51" s="24" t="s">
-        <v>76</v>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="B50" s="17" t="n">
+        <f aca="false">IF(OR($A50&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A50)*(1-$B$8))*B$25+($A50*(1-$B$8))*B$30)/(((B$19-$A50)*(1-$B$8))+($A50*(1-$B$8))))*(1-((((B$19-$A50)*(1-$B$8))*B$25+($A50*(1-$B$8))*B$30)/(((B$19-$A50)*(1-$B$8))+($A50*(1-$B$8)))))*(1/((B$19-$A50)*(1-$B$8))+1/($A50*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A50)*(1-$B$8))+B$30*(1-B$30)/($A50*(1-$B$8)))))</f>
+        <v>0.159233528632258</v>
+      </c>
+      <c r="C50" s="17" t="n">
+        <f aca="false">IF(OR($A50&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A50)*(1-$B$8))*C$25+($A50*(1-$B$8))*C$30)/(((C$19-$A50)*(1-$B$8))+($A50*(1-$B$8))))*(1-((((C$19-$A50)*(1-$B$8))*C$25+($A50*(1-$B$8))*C$30)/(((C$19-$A50)*(1-$B$8))+($A50*(1-$B$8)))))*(1/((C$19-$A50)*(1-$B$8))+1/($A50*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A50)*(1-$B$8))+C$30*(1-C$30)/($A50*(1-$B$8)))))</f>
+        <v>0.0744729646625192</v>
+      </c>
+      <c r="D50" s="17" t="n">
+        <f aca="false">IF(OR($A50&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A50)*(1-$B$8))*D$25+($A50*(1-$B$8))*D$30)/(((D$19-$A50)*(1-$B$8))+($A50*(1-$B$8))))*(1-((((D$19-$A50)*(1-$B$8))*D$25+($A50*(1-$B$8))*D$30)/(((D$19-$A50)*(1-$B$8))+($A50*(1-$B$8)))))*(1/((D$19-$A50)*(1-$B$8))+1/($A50*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A50)*(1-$B$8))+D$30*(1-D$30)/($A50*(1-$B$8)))))</f>
+        <v>0.0473490763527856</v>
+      </c>
+      <c r="F50" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B50),B50&gt;=$B$6),$A50,"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C50),C50&gt;=$B$6),$A50,"")</f>
+        <v/>
+      </c>
+      <c r="H50" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(D50),D50&gt;=$B$6),$A50,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="26" t="n">
+        <v>25000</v>
+      </c>
+      <c r="B51" s="17" t="n">
+        <f aca="false">IF(OR($A51&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A51)*(1-$B$8))*B$25+($A51*(1-$B$8))*B$30)/(((B$19-$A51)*(1-$B$8))+($A51*(1-$B$8))))*(1-((((B$19-$A51)*(1-$B$8))*B$25+($A51*(1-$B$8))*B$30)/(((B$19-$A51)*(1-$B$8))+($A51*(1-$B$8)))))*(1/((B$19-$A51)*(1-$B$8))+1/($A51*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A51)*(1-$B$8))+B$30*(1-B$30)/($A51*(1-$B$8)))))</f>
+        <v>0.274910152696791</v>
+      </c>
+      <c r="C51" s="17" t="n">
+        <f aca="false">IF(OR($A51&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A51)*(1-$B$8))*C$25+($A51*(1-$B$8))*C$30)/(((C$19-$A51)*(1-$B$8))+($A51*(1-$B$8))))*(1-((((C$19-$A51)*(1-$B$8))*C$25+($A51*(1-$B$8))*C$30)/(((C$19-$A51)*(1-$B$8))+($A51*(1-$B$8)))))*(1/((C$19-$A51)*(1-$B$8))+1/($A51*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A51)*(1-$B$8))+C$30*(1-C$30)/($A51*(1-$B$8)))))</f>
+        <v>0.109445307468781</v>
+      </c>
+      <c r="D51" s="17" t="n">
+        <f aca="false">IF(OR($A51&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A51)*(1-$B$8))*D$25+($A51*(1-$B$8))*D$30)/(((D$19-$A51)*(1-$B$8))+($A51*(1-$B$8))))*(1-((((D$19-$A51)*(1-$B$8))*D$25+($A51*(1-$B$8))*D$30)/(((D$19-$A51)*(1-$B$8))+($A51*(1-$B$8)))))*(1/((D$19-$A51)*(1-$B$8))+1/($A51*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A51)*(1-$B$8))+D$30*(1-D$30)/($A51*(1-$B$8)))))</f>
+        <v>0.0796253915860124</v>
+      </c>
+      <c r="F51" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B51),B51&gt;=$B$6),$A51,"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C51),C51&gt;=$B$6),$A51,"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(D51),D51&gt;=$B$6),$A51,"")</f>
+        <v/>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="26" t="n">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="B52" s="17" t="n">
-        <f aca="false">IF(OR($A52&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A52)*(1-$B$8))*B$26+($A52*(1-$B$8))*B$31)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((B$19-$A52)*(1-$B$8))*B$26+($A52*(1-$B$8))*B$31)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((B$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A52)*(1-$B$8))+B$31*(1-B$31)/($A52*(1-$B$8)))))</f>
-        <v>0.0536529495750876</v>
+        <f aca="false">IF(OR($A52&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A52)*(1-$B$8))*B$25+($A52*(1-$B$8))*B$30)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((B$19-$A52)*(1-$B$8))*B$25+($A52*(1-$B$8))*B$30)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((B$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A52)*(1-$B$8))+B$30*(1-B$30)/($A52*(1-$B$8)))))</f>
+        <v>0.430336919216376</v>
       </c>
       <c r="C52" s="17" t="n">
-        <f aca="false">IF(OR($A52&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A52)*(1-$B$8))*C$26+($A52*(1-$B$8))*C$31)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((C$19-$A52)*(1-$B$8))*C$26+($A52*(1-$B$8))*C$31)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((C$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A52)*(1-$B$8))+C$31*(1-C$31)/($A52*(1-$B$8)))))</f>
-        <v>0.0280361088736851</v>
+        <f aca="false">IF(OR($A52&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A52)*(1-$B$8))*C$25+($A52*(1-$B$8))*C$30)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((C$19-$A52)*(1-$B$8))*C$25+($A52*(1-$B$8))*C$30)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((C$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A52)*(1-$B$8))+C$30*(1-C$30)/($A52*(1-$B$8)))))</f>
+        <v>0.158142581595719</v>
       </c>
       <c r="D52" s="17" t="n">
-        <f aca="false">IF(OR($A52&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A52)*(1-$B$8))*D$26+($A52*(1-$B$8))*D$31)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((D$19-$A52)*(1-$B$8))*D$26+($A52*(1-$B$8))*D$31)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((D$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A52)*(1-$B$8))+D$31*(1-D$31)/($A52*(1-$B$8)))))</f>
-        <v>0.0184966876327773</v>
+        <f aca="false">IF(OR($A52&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A52)*(1-$B$8))*D$25+($A52*(1-$B$8))*D$30)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((D$19-$A52)*(1-$B$8))*D$25+($A52*(1-$B$8))*D$30)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((D$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A52)*(1-$B$8))+D$30*(1-D$30)/($A52*(1-$B$8)))))</f>
+        <v>0.133014193269905</v>
+      </c>
+      <c r="F52" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B52),B52&gt;=$B$6),$A52,"")</f>
+        <v/>
+      </c>
+      <c r="G52" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C52),C52&gt;=$B$6),$A52,"")</f>
+        <v/>
+      </c>
+      <c r="H52" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(D52),D52&gt;=$B$6),$A52,"")</f>
+        <v/>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="26" t="n">
-        <v>25000</v>
+        <v>100000</v>
       </c>
       <c r="B53" s="17" t="n">
-        <f aca="false">IF(OR($A53&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A53)*(1-$B$8))*B$26+($A53*(1-$B$8))*B$31)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((B$19-$A53)*(1-$B$8))*B$26+($A53*(1-$B$8))*B$31)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((B$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A53)*(1-$B$8))+B$31*(1-B$31)/($A53*(1-$B$8)))))</f>
-        <v>0.0867242384749355</v>
+        <f aca="false">IF(OR($A53&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A53)*(1-$B$8))*B$25+($A53*(1-$B$8))*B$30)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((B$19-$A53)*(1-$B$8))*B$25+($A53*(1-$B$8))*B$30)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((B$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A53)*(1-$B$8))+B$30*(1-B$30)/($A53*(1-$B$8)))))</f>
+        <v>0.636690055383955</v>
       </c>
       <c r="C53" s="17" t="n">
-        <f aca="false">IF(OR($A53&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A53)*(1-$B$8))*C$26+($A53*(1-$B$8))*C$31)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((C$19-$A53)*(1-$B$8))*C$26+($A53*(1-$B$8))*C$31)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((C$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A53)*(1-$B$8))+C$31*(1-C$31)/($A53*(1-$B$8)))))</f>
-        <v>0.0375719061445862</v>
+        <f aca="false">IF(OR($A53&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A53)*(1-$B$8))*C$25+($A53*(1-$B$8))*C$30)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((C$19-$A53)*(1-$B$8))*C$25+($A53*(1-$B$8))*C$30)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((C$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A53)*(1-$B$8))+C$30*(1-C$30)/($A53*(1-$B$8)))))</f>
+        <v>0.237238824135504</v>
       </c>
       <c r="D53" s="17" t="n">
-        <f aca="false">IF(OR($A53&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A53)*(1-$B$8))*D$26+($A53*(1-$B$8))*D$31)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((D$19-$A53)*(1-$B$8))*D$26+($A53*(1-$B$8))*D$31)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((D$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A53)*(1-$B$8))+D$31*(1-D$31)/($A53*(1-$B$8)))))</f>
-        <v>0.0266249031538368</v>
+        <f aca="false">IF(OR($A53&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A53)*(1-$B$8))*D$25+($A53*(1-$B$8))*D$30)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((D$19-$A53)*(1-$B$8))*D$25+($A53*(1-$B$8))*D$30)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((D$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A53)*(1-$B$8))+D$30*(1-D$30)/($A53*(1-$B$8)))))</f>
+        <v>0.242152249674039</v>
+      </c>
+      <c r="F53" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B53),B53&gt;=$B$6),$A53,"")</f>
+        <v/>
+      </c>
+      <c r="G53" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C53),C53&gt;=$B$6),$A53,"")</f>
+        <v/>
+      </c>
+      <c r="H53" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(D53),D53&gt;=$B$6),$A53,"")</f>
+        <v/>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="26" t="n">
-        <v>50000</v>
+        <v>250000</v>
       </c>
       <c r="B54" s="17" t="n">
-        <f aca="false">IF(OR($A54&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A54)*(1-$B$8))*B$26+($A54*(1-$B$8))*B$31)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((B$19-$A54)*(1-$B$8))*B$26+($A54*(1-$B$8))*B$31)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((B$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A54)*(1-$B$8))+B$31*(1-B$31)/($A54*(1-$B$8)))))</f>
-        <v>0.135699240566072</v>
+        <f aca="false">IF(OR($A54&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A54)*(1-$B$8))*B$25+($A54*(1-$B$8))*B$30)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((B$19-$A54)*(1-$B$8))*B$25+($A54*(1-$B$8))*B$30)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((B$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A54)*(1-$B$8))+B$30*(1-B$30)/($A54*(1-$B$8)))))</f>
+        <v>0.830962778781712</v>
       </c>
       <c r="C54" s="17" t="n">
-        <f aca="false">IF(OR($A54&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A54)*(1-$B$8))*C$26+($A54*(1-$B$8))*C$31)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((C$19-$A54)*(1-$B$8))*C$26+($A54*(1-$B$8))*C$31)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((C$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A54)*(1-$B$8))+C$31*(1-C$31)/($A54*(1-$B$8)))))</f>
-        <v>0.050390411893423</v>
+        <f aca="false">IF(OR($A54&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A54)*(1-$B$8))*C$25+($A54*(1-$B$8))*C$30)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((C$19-$A54)*(1-$B$8))*C$25+($A54*(1-$B$8))*C$30)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((C$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A54)*(1-$B$8))+C$30*(1-C$30)/($A54*(1-$B$8)))))</f>
+        <v>0.36681549520206</v>
       </c>
       <c r="D54" s="17" t="n">
-        <f aca="false">IF(OR($A54&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A54)*(1-$B$8))*D$26+($A54*(1-$B$8))*D$31)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((D$19-$A54)*(1-$B$8))*D$26+($A54*(1-$B$8))*D$31)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((D$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A54)*(1-$B$8))+D$31*(1-D$31)/($A54*(1-$B$8)))))</f>
-        <v>0.0390892731725304</v>
+        <f aca="false">IF(OR($A54&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A54)*(1-$B$8))*D$25+($A54*(1-$B$8))*D$30)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((D$19-$A54)*(1-$B$8))*D$25+($A54*(1-$B$8))*D$30)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((D$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A54)*(1-$B$8))+D$30*(1-D$30)/($A54*(1-$B$8)))))</f>
+        <v>0.536974464177551</v>
+      </c>
+      <c r="F54" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(B54),B54&gt;=$B$6),$A54,"")</f>
+        <v>250000</v>
+      </c>
+      <c r="G54" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C54),C54&gt;=$B$6),$A54,"")</f>
+        <v/>
+      </c>
+      <c r="H54" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(D54),D54&gt;=$B$6),$A54,"")</f>
+        <v/>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="26" t="n">
-        <v>100000</v>
+        <v>500000</v>
       </c>
       <c r="B55" s="17" t="n">
-        <f aca="false">IF(OR($A55&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A55)*(1-$B$8))*B$26+($A55*(1-$B$8))*B$31)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((B$19-$A55)*(1-$B$8))*B$26+($A55*(1-$B$8))*B$31)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((B$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A55)*(1-$B$8))+B$31*(1-B$31)/($A55*(1-$B$8)))))</f>
-        <v>0.217644169186768</v>
+        <f aca="false">IF(OR($A55&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A55)*(1-$B$8))*B$25+($A55*(1-$B$8))*B$30)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((B$19-$A55)*(1-$B$8))*B$25+($A55*(1-$B$8))*B$30)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((B$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A55)*(1-$B$8))+B$30*(1-B$30)/($A55*(1-$B$8)))))</f>
+        <v>0.408153831705151</v>
       </c>
       <c r="C55" s="17" t="n">
-        <f aca="false">IF(OR($A55&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A55)*(1-$B$8))*C$26+($A55*(1-$B$8))*C$31)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((C$19-$A55)*(1-$B$8))*C$26+($A55*(1-$B$8))*C$31)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((C$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A55)*(1-$B$8))+C$31*(1-C$31)/($A55*(1-$B$8)))))</f>
-        <v>0.0710652852568584</v>
+        <f aca="false">IF(OR($A55&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A55)*(1-$B$8))*C$25+($A55*(1-$B$8))*C$30)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((C$19-$A55)*(1-$B$8))*C$25+($A55*(1-$B$8))*C$30)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((C$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A55)*(1-$B$8))+C$30*(1-C$30)/($A55*(1-$B$8)))))</f>
+        <v>0.28483495767885</v>
       </c>
       <c r="D55" s="17" t="n">
-        <f aca="false">IF(OR($A55&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A55)*(1-$B$8))*D$26+($A55*(1-$B$8))*D$31)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((D$19-$A55)*(1-$B$8))*D$26+($A55*(1-$B$8))*D$31)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((D$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A55)*(1-$B$8))+D$31*(1-D$31)/($A55*(1-$B$8)))))</f>
-        <v>0.0640956190702727</v>
+        <f aca="false">IF(OR($A55&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A55)*(1-$B$8))*D$25+($A55*(1-$B$8))*D$30)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((D$19-$A55)*(1-$B$8))*D$25+($A55*(1-$B$8))*D$30)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((D$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A55)*(1-$B$8))+D$30*(1-D$30)/($A55*(1-$B$8)))))</f>
+        <v>0.820893449627511</v>
+      </c>
+      <c r="F55" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B55),B55&gt;=$B$6),$A55,"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C55),C55&gt;=$B$6),$A55,"")</f>
+        <v/>
+      </c>
+      <c r="H55" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D55),D55&gt;=$B$6),$A55,"")</f>
+        <v>500000</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="26" t="n">
-        <v>250000</v>
-      </c>
-      <c r="B56" s="17" t="n">
-        <f aca="false">IF(OR($A56&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A56)*(1-$B$8))*B$26+($A56*(1-$B$8))*B$31)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((B$19-$A56)*(1-$B$8))*B$26+($A56*(1-$B$8))*B$31)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((B$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A56)*(1-$B$8))+B$31*(1-B$31)/($A56*(1-$B$8)))))</f>
-        <v>0.331630243365877</v>
-      </c>
-      <c r="C56" s="17" t="n">
-        <f aca="false">IF(OR($A56&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A56)*(1-$B$8))*C$26+($A56*(1-$B$8))*C$31)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((C$19-$A56)*(1-$B$8))*C$26+($A56*(1-$B$8))*C$31)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((C$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A56)*(1-$B$8))+C$31*(1-C$31)/($A56*(1-$B$8)))))</f>
-        <v>0.105802686346464</v>
+        <v>1000000</v>
+      </c>
+      <c r="B56" s="17" t="str">
+        <f aca="false">IF(OR($A56&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A56)*(1-$B$8))*B$25+($A56*(1-$B$8))*B$30)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((B$19-$A56)*(1-$B$8))*B$25+($A56*(1-$B$8))*B$30)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((B$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A56)*(1-$B$8))+B$30*(1-B$30)/($A56*(1-$B$8)))))</f>
+        <v/>
+      </c>
+      <c r="C56" s="17" t="str">
+        <f aca="false">IF(OR($A56&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A56)*(1-$B$8))*C$25+($A56*(1-$B$8))*C$30)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((C$19-$A56)*(1-$B$8))*C$25+($A56*(1-$B$8))*C$30)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((C$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A56)*(1-$B$8))+C$30*(1-C$30)/($A56*(1-$B$8)))))</f>
+        <v/>
       </c>
       <c r="D56" s="17" t="n">
-        <f aca="false">IF(OR($A56&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A56)*(1-$B$8))*D$26+($A56*(1-$B$8))*D$31)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((D$19-$A56)*(1-$B$8))*D$26+($A56*(1-$B$8))*D$31)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((D$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A56)*(1-$B$8))+D$31*(1-D$31)/($A56*(1-$B$8)))))</f>
-        <v>0.144746804199576</v>
+        <f aca="false">IF(OR($A56&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A56)*(1-$B$8))*D$25+($A56*(1-$B$8))*D$30)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((D$19-$A56)*(1-$B$8))*D$25+($A56*(1-$B$8))*D$30)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((D$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A56)*(1-$B$8))+D$30*(1-D$30)/($A56*(1-$B$8)))))</f>
+        <v>0.971283737774168</v>
+      </c>
+      <c r="F56" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B56),B56&gt;=$B$6),$A56,"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C56),C56&gt;=$B$6),$A56,"")</f>
+        <v/>
+      </c>
+      <c r="H56" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D56),D56&gt;=$B$6),$A56,"")</f>
+        <v>1000000</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="B57" s="17" t="n">
-        <f aca="false">IF(OR($A57&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A57)*(1-$B$8))*B$26+($A57*(1-$B$8))*B$31)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((B$19-$A57)*(1-$B$8))*B$26+($A57*(1-$B$8))*B$31)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((B$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A57)*(1-$B$8))+B$31*(1-B$31)/($A57*(1-$B$8)))))</f>
-        <v>0.11120495607459</v>
-      </c>
-      <c r="C57" s="17" t="n">
-        <f aca="false">IF(OR($A57&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A57)*(1-$B$8))*C$26+($A57*(1-$B$8))*C$31)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((C$19-$A57)*(1-$B$8))*C$26+($A57*(1-$B$8))*C$31)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((C$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A57)*(1-$B$8))+C$31*(1-C$31)/($A57*(1-$B$8)))))</f>
-        <v>0.0797032207645197</v>
+        <v>2000000</v>
+      </c>
+      <c r="B57" s="17" t="str">
+        <f aca="false">IF(OR($A57&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A57)*(1-$B$8))*B$25+($A57*(1-$B$8))*B$30)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((B$19-$A57)*(1-$B$8))*B$25+($A57*(1-$B$8))*B$30)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((B$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A57)*(1-$B$8))+B$30*(1-B$30)/($A57*(1-$B$8)))))</f>
+        <v/>
+      </c>
+      <c r="C57" s="17" t="str">
+        <f aca="false">IF(OR($A57&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A57)*(1-$B$8))*C$25+($A57*(1-$B$8))*C$30)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((C$19-$A57)*(1-$B$8))*C$25+($A57*(1-$B$8))*C$30)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((C$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A57)*(1-$B$8))+C$30*(1-C$30)/($A57*(1-$B$8)))))</f>
+        <v/>
       </c>
       <c r="D57" s="17" t="n">
-        <f aca="false">IF(OR($A57&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A57)*(1-$B$8))*D$26+($A57*(1-$B$8))*D$31)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((D$19-$A57)*(1-$B$8))*D$26+($A57*(1-$B$8))*D$31)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((D$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A57)*(1-$B$8))+D$31*(1-D$31)/($A57*(1-$B$8)))))</f>
-        <v>0.282795870586124</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="26" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="B58" s="17" t="str">
-        <f aca="false">IF(OR($A58&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A58)*(1-$B$8))*B$26+($A58*(1-$B$8))*B$31)/(((B$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((B$19-$A58)*(1-$B$8))*B$26+($A58*(1-$B$8))*B$31)/(((B$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((B$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A58)*(1-$B$8))+B$31*(1-B$31)/($A58*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="C58" s="17" t="str">
-        <f aca="false">IF(OR($A58&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A58)*(1-$B$8))*C$26+($A58*(1-$B$8))*C$31)/(((C$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((C$19-$A58)*(1-$B$8))*C$26+($A58*(1-$B$8))*C$31)/(((C$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((C$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A58)*(1-$B$8))+C$31*(1-C$31)/($A58*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="D58" s="17" t="n">
-        <f aca="false">IF(OR($A58&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A58)*(1-$B$8))*D$26+($A58*(1-$B$8))*D$31)/(((D$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((D$19-$A58)*(1-$B$8))*D$26+($A58*(1-$B$8))*D$31)/(((D$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((D$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A58)*(1-$B$8))+D$31*(1-D$31)/($A58*(1-$B$8)))))</f>
-        <v>0.503337360450257</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="26" t="n">
+        <f aca="false">IF(OR($A57&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A57)*(1-$B$8))*D$25+($A57*(1-$B$8))*D$30)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((D$19-$A57)*(1-$B$8))*D$25+($A57*(1-$B$8))*D$30)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((D$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A57)*(1-$B$8))+D$30*(1-D$30)/($A57*(1-$B$8)))))</f>
+        <v>0.996502733288146</v>
+      </c>
+      <c r="F57" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B57),B57&gt;=$B$6),$A57,"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C57),C57&gt;=$B$6),$A57,"")</f>
+        <v/>
+      </c>
+      <c r="H57" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D57),D57&gt;=$B$6),$A57,"")</f>
         <v>2000000</v>
       </c>
-      <c r="B59" s="17" t="str">
-        <f aca="false">IF(OR($A59&gt;=B$19,B$30=0),"",NORMSDIST((ABS(B$31-B$26)-$B$10*SQRT(((((B$19-$A59)*(1-$B$8))*B$26+($A59*(1-$B$8))*B$31)/(((B$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((B$19-$A59)*(1-$B$8))*B$26+($A59*(1-$B$8))*B$31)/(((B$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((B$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(B$26*(1-B$26)/((B$19-$A59)*(1-$B$8))+B$31*(1-B$31)/($A59*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="C59" s="17" t="str">
-        <f aca="false">IF(OR($A59&gt;=C$19,C$30=0),"",NORMSDIST((ABS(C$31-C$26)-$B$10*SQRT(((((C$19-$A59)*(1-$B$8))*C$26+($A59*(1-$B$8))*C$31)/(((C$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((C$19-$A59)*(1-$B$8))*C$26+($A59*(1-$B$8))*C$31)/(((C$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((C$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(C$26*(1-C$26)/((C$19-$A59)*(1-$B$8))+C$31*(1-C$31)/($A59*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="D59" s="17" t="n">
-        <f aca="false">IF(OR($A59&gt;=D$19,D$30=0),"",NORMSDIST((ABS(D$31-D$26)-$B$10*SQRT(((((D$19-$A59)*(1-$B$8))*D$26+($A59*(1-$B$8))*D$31)/(((D$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((D$19-$A59)*(1-$B$8))*D$26+($A59*(1-$B$8))*D$31)/(((D$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((D$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(D$26*(1-D$26)/((D$19-$A59)*(1-$B$8))+D$31*(1-D$31)/($A59*(1-$B$8)))))</f>
-        <v>0.691588543720377</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="B61" s="27"/>
-      <c r="C61" s="27"/>
-      <c r="D61" s="27"/>
-      <c r="E61" s="27"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="27"/>
-      <c r="B62" s="27"/>
-      <c r="C62" s="27"/>
-      <c r="D62" s="27"/>
-      <c r="E62" s="27"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B59" s="28"/>
+      <c r="C59" s="28"/>
+      <c r="D59" s="28"/>
+      <c r="E59" s="28"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="28"/>
+      <c r="B60" s="28"/>
+      <c r="C60" s="28"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="A61:E62"/>
+    <mergeCell ref="A59:E60"/>
   </mergeCells>
-  <conditionalFormatting sqref="B52:D59">
+  <conditionalFormatting sqref="B50:D57">
     <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$B$6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B33:D33">
+  <conditionalFormatting sqref="B32:D32">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"SÍ"</formula>
     </cfRule>
@@ -1765,7 +1823,7 @@
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B27:D27">
+  <conditionalFormatting sqref="B26:D26">
     <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -1793,45 +1851,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="29" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="29" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="29" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="28" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="29" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="29" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="29"/>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="29" t="s">
         <v>81</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28"/>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
-        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calculator v6: explicit sample size per arm and pool fit rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ygiEd3g3fKiFCARJZcKLp
</commit_message>
<xml_diff>
--- a/calculadora-sample-size.xlsx
+++ b/calculadora-sample-size.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="87">
   <si>
     <t xml:space="preserve">Calculadora de poder: experimento de crédito por score (ventana de 1 mes)</t>
   </si>
@@ -197,6 +197,18 @@
     <t xml:space="preserve">Diferencia de crédito × eventos del grupo tratado. Negativo = ahorro. Asume que el crédito se paga por evento.</t>
   </si>
   <si>
+    <t xml:space="preserve">SAMPLE SIZE: usuarios por brazo que necesitas (50/50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El número clásico. Tantos en tratamiento y otros tantos en control para ver tu cambio esperado con el poder elegido. Es el que te pedirían en cualquier lado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Existen en tu pool? (necesitas 2 × sample size)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si dice NO, ningún presupuesto lo arregla: sube el cambio esperado, alarga la ventana o cambia la métrica.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mínimo de usuarios en tratamiento para llegar al poder</t>
   </si>
   <si>
@@ -254,10 +266,13 @@
     <t xml:space="preserve">2. Mira 'PODER con tus usuarios' (fila 31). Si está en 80% o más, listo.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Si no, mira 'Mínimo de usuarios en tratamiento para llegar al poder' (fila 36) y escribe ese número en la fila 21.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. 'Qué hacer' (fila 37) te lo dice en una línea.</t>
+    <t xml:space="preserve">3. Si no, mira 'Mínimo de usuarios en tratamiento para llegar al poder' (fila 38) y escribe ese número en la fila 21.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3b. 'SAMPLE SIZE' (fila 36) es el número clásico de usuarios por brazo. Si la fila 37 dice NO, no existen suficientes usuarios para ese cambio esperado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. 'Qué hacer' (fila 39) te lo dice en una línea.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Para cambiar la métrica: escribe su nombre en la fila 14 y pon en la fila 20 cuántos usuarios de cada tier la cumplen al mes hoy.</t>
@@ -876,7 +891,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -1257,15 +1272,15 @@
         <v>49</v>
       </c>
       <c r="B31" s="19" t="n">
-        <f aca="false">IF(OR(B26&lt;=0,B29=0),0,NORMSDIST((ABS(B30-B25)-$B$10*SQRT(B42*(1-B42)*(1/B41+1/B40)))/SQRT(B25*(1-B25)/B41+B30*(1-B30)/B40)))</f>
+        <f aca="false">IF(OR(B26&lt;=0,B29=0),0,NORMSDIST((ABS(B30-B25)-$B$10*SQRT(B44*(1-B44)*(1/B43+1/B42)))/SQRT(B25*(1-B25)/B43+B30*(1-B30)/B42)))</f>
         <v>0.833642091009647</v>
       </c>
       <c r="C31" s="19" t="n">
-        <f aca="false">IF(OR(C26&lt;=0,C29=0),0,NORMSDIST((ABS(C30-C25)-$B$10*SQRT(C42*(1-C42)*(1/C41+1/C40)))/SQRT(C25*(1-C25)/C41+C30*(1-C30)/C40)))</f>
+        <f aca="false">IF(OR(C26&lt;=0,C29=0),0,NORMSDIST((ABS(C30-C25)-$B$10*SQRT(C44*(1-C44)*(1/C43+1/C42)))/SQRT(C25*(1-C25)/C43+C30*(1-C30)/C42)))</f>
         <v>0.379325029852179</v>
       </c>
       <c r="D31" s="19" t="n">
-        <f aca="false">IF(OR(D26&lt;=0,D29=0),0,NORMSDIST((ABS(D30-D25)-$B$10*SQRT(D42*(1-D42)*(1/D41+1/D40)))/SQRT(D25*(1-D25)/D41+D30*(1-D30)/D40)))</f>
+        <f aca="false">IF(OR(D26&lt;=0,D29=0),0,NORMSDIST((ABS(D30-D25)-$B$10*SQRT(D44*(1-D44)*(1/D43+1/D42)))/SQRT(D25*(1-D25)/D43+D30*(1-D30)/D42)))</f>
         <v>0.996923501492287</v>
       </c>
       <c r="E31" s="7" t="s">
@@ -1294,15 +1309,15 @@
         <v>52</v>
       </c>
       <c r="B33" s="17" t="n">
-        <f aca="false">IF(B26&lt;=0,"n/a",B47/B25)</f>
+        <f aca="false">IF(B26&lt;=0,"n/a",B49/B25)</f>
         <v>0.28611986853037</v>
       </c>
       <c r="C33" s="17" t="n">
-        <f aca="false">IF(C26&lt;=0,"n/a",C47/C25)</f>
+        <f aca="false">IF(C26&lt;=0,"n/a",C49/C25)</f>
         <v>0.260730906417824</v>
       </c>
       <c r="D33" s="17" t="n">
-        <f aca="false">IF(D26&lt;=0,"n/a",D47/D25)</f>
+        <f aca="false">IF(D26&lt;=0,"n/a",D49/D25)</f>
         <v>0.0951582685017244</v>
       </c>
       <c r="E33" s="7" t="s">
@@ -1349,287 +1364,269 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
         <v>58</v>
       </c>
       <c r="B36" s="22" t="n">
-        <f aca="false">IF(COUNT(F50:F57)=0,"No llega ni con todo el pool",MIN(F50:F57))</f>
-        <v>250000</v>
-      </c>
-      <c r="C36" s="22" t="str">
-        <f aca="false">IF(COUNT(G50:G57)=0,"No llega ni con todo el pool",MIN(G50:G57))</f>
-        <v>No llega ni con todo el pool</v>
+        <f aca="false">IF(B29=0,"n/a",ROUNDUP(((($B$10*SQRT(2*((B25+B30)/2)*(1-(B25+B30)/2))+$B$11*SQRT(B25*(1-B25)+B30*(1-B30)))^2)/(B30-B25)^2)/(1-$B$8),0))</f>
+        <v>257227</v>
+      </c>
+      <c r="C36" s="22" t="n">
+        <f aca="false">IF(C29=0,"n/a",ROUNDUP(((($B$10*SQRT(2*((C25+C30)/2)*(1-(C25+C30)/2))+$B$11*SQRT(C25*(1-C25)+C30*(1-C30)))^2)/(C30-C25)^2)/(1-$B$8),0))</f>
+        <v>960306</v>
       </c>
       <c r="D36" s="22" t="n">
-        <f aca="false">IF(COUNT(H50:H57)=0,"No llega ni con todo el pool",MIN(H50:H57))</f>
-        <v>500000</v>
+        <f aca="false">IF(D29=0,"n/a",ROUNDUP(((($B$10*SQRT(2*((D25+D30)/2)*(1-(D25+D30)/2))+$B$11*SQRT(D25*(1-D25)+D30*(1-D30)))^2)/(D30-D25)^2)/(1-$B$8),0))</f>
+        <v>827073</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
         <v>60</v>
       </c>
       <c r="B37" s="20" t="str">
-        <f aca="false">IF(B26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(B32="SÍ","Corre con "&amp;TEXT(B21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(B36),"Sube tratamiento a "&amp;TEXT(B36,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
+        <f aca="false">IF(ISNUMBER(B36),IF(2*B36&lt;=B19,"SÍ, cabe","NO: necesitas "&amp;TEXT(2*B36,"#,##0")&amp;" y tienes "&amp;TEXT(B19,"#,##0")),"n/a")</f>
+        <v>SÍ, cabe</v>
+      </c>
+      <c r="C37" s="20" t="str">
+        <f aca="false">IF(ISNUMBER(C36),IF(2*C36&lt;=C19,"SÍ, cabe","NO: necesitas "&amp;TEXT(2*C36,"#,##0")&amp;" y tienes "&amp;TEXT(C19,"#,##0")),"n/a")</f>
+        <v>NO: necesitas 1,920,612 y tienes 668,384</v>
+      </c>
+      <c r="D37" s="20" t="str">
+        <f aca="false">IF(ISNUMBER(D36),IF(2*D36&lt;=D19,"SÍ, cabe","NO: necesitas "&amp;TEXT(2*D36,"#,##0")&amp;" y tienes "&amp;TEXT(D19,"#,##0")),"n/a")</f>
+        <v>SÍ, cabe</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="22" t="n">
+        <f aca="false">IF(COUNT(F52:F59)=0,"No llega ni con todo el pool",MIN(F52:F59))</f>
+        <v>250000</v>
+      </c>
+      <c r="C38" s="22" t="str">
+        <f aca="false">IF(COUNT(G52:G59)=0,"No llega ni con todo el pool",MIN(G52:G59))</f>
+        <v>No llega ni con todo el pool</v>
+      </c>
+      <c r="D38" s="22" t="n">
+        <f aca="false">IF(COUNT(H52:H59)=0,"No llega ni con todo el pool",MIN(H52:H59))</f>
+        <v>500000</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="20" t="str">
+        <f aca="false">IF(B26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(B32="SÍ","Corre con "&amp;TEXT(B21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(B38),"Sube tratamiento a "&amp;TEXT(B38,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
         <v>Corre con 281,000 en tratamiento.</v>
       </c>
-      <c r="C37" s="20" t="str">
-        <f aca="false">IF(C26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(C32="SÍ","Corre con "&amp;TEXT(C21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(C36),"Sube tratamiento a "&amp;TEXT(C36,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
+      <c r="C39" s="20" t="str">
+        <f aca="false">IF(C26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(C32="SÍ","Corre con "&amp;TEXT(C21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(C38),"Sube tratamiento a "&amp;TEXT(C38,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
         <v>No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.</v>
       </c>
-      <c r="D37" s="20" t="str">
-        <f aca="false">IF(D26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(D32="SÍ","Corre con "&amp;TEXT(D21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(D36),"Sube tratamiento a "&amp;TEXT(D36,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
+      <c r="D39" s="20" t="str">
+        <f aca="false">IF(D26&lt;0,"Tratamiento mayor al pool. Bájalo.",IF(D32="SÍ","Corre con "&amp;TEXT(D21,"#,##0")&amp;" en tratamiento.",IF(ISNUMBER(D38),"Sube tratamiento a "&amp;TEXT(D38,"#,##0")&amp;".","No se puede medir en 1 mes con este cambio esperado. Cambia la métrica por una más frecuente o espera un cambio mayor.")))</f>
         <v>Corre con 2,327,000 en tratamiento.</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="B39" s="24" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C39" s="24" t="s">
+      <c r="C41" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="D39" s="24" t="s">
+      <c r="D41" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="E39" s="24"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B40" s="16" t="n">
+      <c r="E41" s="24"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B42" s="16" t="n">
         <f aca="false">B21*(1-$B$8)</f>
         <v>266950</v>
       </c>
-      <c r="C40" s="16" t="n">
+      <c r="C42" s="16" t="n">
         <f aca="false">C21*(1-$B$8)</f>
         <v>317482.4</v>
       </c>
-      <c r="D40" s="16" t="n">
+      <c r="D42" s="16" t="n">
         <f aca="false">D21*(1-$B$8)</f>
         <v>2210650</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B41" s="16" t="n">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43" s="16" t="n">
         <f aca="false">MAX(B26,1)*(1-$B$8)</f>
         <v>267101.05</v>
       </c>
-      <c r="C41" s="16" t="n">
+      <c r="C43" s="16" t="n">
         <f aca="false">MAX(C26,1)*(1-$B$8)</f>
         <v>317482.4</v>
       </c>
-      <c r="D41" s="16" t="n">
+      <c r="D43" s="16" t="n">
         <f aca="false">MAX(D26,1)*(1-$B$8)</f>
         <v>2211034.75</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B42" s="25" t="n">
-        <f aca="false">(B41*B25+B40*B30)/(B41+B40)</f>
-        <v>0.000943025801852056</v>
-      </c>
-      <c r="C42" s="25" t="n">
-        <f aca="false">(C41*C25+C40*C30)/(C41+C40)</f>
-        <v>0.000882987923110069</v>
-      </c>
-      <c r="D42" s="25" t="n">
-        <f aca="false">(D41*D25+D40*D30)/(D41+D40)</f>
-        <v>0.000759178655404867</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B43" s="25" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(B25*(1-B25)*(1/B41+1/B40))</f>
-        <v>0.000219475070481767</v>
-      </c>
-      <c r="C43" s="25" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(C25*(1-C25)*(1/C41+1/C40))</f>
-        <v>0.000201443715395474</v>
-      </c>
-      <c r="D43" s="25" t="n">
-        <f aca="false">($B$10+$B$11)*SQRT(D25*(1-D25)*(1/D41+1/D40))</f>
-        <v>7.63064502860877E-005</v>
-      </c>
-    </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B44" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B43))/(B41+B40))*(1-((B41*B25+B40*(B25+B43))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B43)*(1-B25-B43)/B40)</f>
-        <v>0.00023368413016945</v>
+        <f aca="false">(B43*B25+B42*B30)/(B43+B42)</f>
+        <v>0.000943025801852056</v>
       </c>
       <c r="C44" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C43))/(C41+C40))*(1-((C41*C25+C40*(C25+C43))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C43)*(1-C25-C43)/C40)</f>
-        <v>0.000213426519316081</v>
+        <f aca="false">(C43*C25+C42*C30)/(C43+C42)</f>
+        <v>0.000882987923110069</v>
       </c>
       <c r="D44" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D43))/(D41+D40))*(1-((D41*D25+D40*(D25+D43))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D43)*(1-D25-D43)/D40)</f>
-        <v>7.80583639702972E-005</v>
+        <f aca="false">(D43*D25+D42*D30)/(D43+D42)</f>
+        <v>0.000759178655404867</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B45" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B44))/(B41+B40))*(1-((B41*B25+B40*(B25+B44))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B44)*(1-B25-B44)/B40)</f>
-        <v>0.00023457424210403</v>
+        <f aca="false">($B$10+$B$11)*SQRT(B25*(1-B25)*(1/B43+1/B42))</f>
+        <v>0.000219475070481767</v>
       </c>
       <c r="C45" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C44))/(C41+C40))*(1-((C41*C25+C40*(C25+C44))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C44)*(1-C25-C44)/C40)</f>
-        <v>0.000214118085343449</v>
+        <f aca="false">($B$10+$B$11)*SQRT(C25*(1-C25)*(1/C43+1/C42))</f>
+        <v>0.000201443715395474</v>
       </c>
       <c r="D45" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D44))/(D41+D40))*(1-((D41*D25+D40*(D25+D44))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D44)*(1-D25-D44)/D40)</f>
-        <v>7.80981225045379E-005</v>
+        <f aca="false">($B$10+$B$11)*SQRT(D25*(1-D25)*(1/D43+1/D42))</f>
+        <v>7.63064502860877E-005</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B46" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B45))/(B41+B40))*(1-((B41*B25+B40*(B25+B45))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B45)*(1-B25-B45)/B40)</f>
-        <v>0.00023462988930975</v>
+        <f aca="false">$B$10*SQRT(((B43*B25+B42*(B25+B45))/(B43+B42))*(1-((B43*B25+B42*(B25+B45))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B25*(1-B25)/B43+(B25+B45)*(1-B25-B45)/B42)</f>
+        <v>0.00023368413016945</v>
       </c>
       <c r="C46" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C45))/(C41+C40))*(1-((C41*C25+C40*(C25+C45))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C45)*(1-C25-C45)/C40)</f>
-        <v>0.00021415792934427</v>
+        <f aca="false">$B$10*SQRT(((C43*C25+C42*(C25+C45))/(C43+C42))*(1-((C43*C25+C42*(C25+C45))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C25*(1-C25)/C43+(C25+C45)*(1-C25-C45)/C42)</f>
+        <v>0.000213426519316081</v>
       </c>
       <c r="D46" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D45))/(D41+D40))*(1-((D41*D25+D40*(D25+D45))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D45)*(1-D25-D45)/D40)</f>
-        <v>7.80990245625121E-005</v>
+        <f aca="false">$B$10*SQRT(((D43*D25+D42*(D25+D45))/(D43+D42))*(1-((D43*D25+D42*(D25+D45))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D25*(1-D25)/D43+(D25+D45)*(1-D25-D45)/D42)</f>
+        <v>7.80583639702972E-005</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B47" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((B41*B25+B40*(B25+B46))/(B41+B40))*(1-((B41*B25+B40*(B25+B46))/(B41+B40)))*(1/B41+1/B40))+$B$11*SQRT(B25*(1-B25)/B41+(B25+B46)*(1-B25-B46)/B40)</f>
+        <f aca="false">$B$10*SQRT(((B43*B25+B42*(B25+B46))/(B43+B42))*(1-((B43*B25+B42*(B25+B46))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B25*(1-B25)/B43+(B25+B46)*(1-B25-B46)/B42)</f>
+        <v>0.00023457424210403</v>
+      </c>
+      <c r="C47" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((C43*C25+C42*(C25+C46))/(C43+C42))*(1-((C43*C25+C42*(C25+C46))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C25*(1-C25)/C43+(C25+C46)*(1-C25-C46)/C42)</f>
+        <v>0.000214118085343449</v>
+      </c>
+      <c r="D47" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((D43*D25+D42*(D25+D46))/(D43+D42))*(1-((D43*D25+D42*(D25+D46))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D25*(1-D25)/D43+(D25+D46)*(1-D25-D46)/D42)</f>
+        <v>7.80981225045379E-005</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B48" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((B43*B25+B42*(B25+B47))/(B43+B42))*(1-((B43*B25+B42*(B25+B47))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B25*(1-B25)/B43+(B25+B47)*(1-B25-B47)/B42)</f>
+        <v>0.00023462988930975</v>
+      </c>
+      <c r="C48" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((C43*C25+C42*(C25+C47))/(C43+C42))*(1-((C43*C25+C42*(C25+C47))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C25*(1-C25)/C43+(C25+C47)*(1-C25-C47)/C42)</f>
+        <v>0.00021415792934427</v>
+      </c>
+      <c r="D48" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((D43*D25+D42*(D25+D47))/(D43+D42))*(1-((D43*D25+D42*(D25+D47))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D25*(1-D25)/D43+(D25+D47)*(1-D25-D47)/D42)</f>
+        <v>7.80990245625121E-005</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B49" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((B43*B25+B42*(B25+B48))/(B43+B42))*(1-((B43*B25+B42*(B25+B48))/(B43+B42)))*(1/B43+1/B42))+$B$11*SQRT(B25*(1-B25)/B43+(B25+B48)*(1-B25-B48)/B42)</f>
         <v>0.000234633367770507</v>
       </c>
-      <c r="C47" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((C41*C25+C40*(C25+C46))/(C41+C40))*(1-((C41*C25+C40*(C25+C46))/(C41+C40)))*(1/C41+1/C40))+$B$11*SQRT(C25*(1-C25)/C41+(C25+C46)*(1-C25-C46)/C40)</f>
+      <c r="C49" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((C43*C25+C42*(C25+C48))/(C43+C42))*(1-((C43*C25+C42*(C25+C48))/(C43+C42)))*(1/C43+1/C42))+$B$11*SQRT(C25*(1-C25)/C43+(C25+C48)*(1-C25-C48)/C42)</f>
         <v>0.00021416022469626</v>
       </c>
-      <c r="D47" s="25" t="n">
-        <f aca="false">$B$10*SQRT(((D41*D25+D40*(D25+D46))/(D41+D40))*(1-((D41*D25+D40*(D25+D46))/(D41+D40)))*(1/D41+1/D40))+$B$11*SQRT(D25*(1-D25)/D41+(D25+D46)*(1-D25-D46)/D40)</f>
+      <c r="D49" s="25" t="n">
+        <f aca="false">$B$10*SQRT(((D43*D25+D42*(D25+D48))/(D43+D42))*(1-((D43*D25+D42*(D25+D48))/(D43+D42)))*(1/D43+1/D42))+$B$11*SQRT(D25*(1-D25)/D43+(D25+D48)*(1-D25-D48)/D42)</f>
         <v>7.80990450286529E-005</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="23" t="s">
-        <v>70</v>
-      </c>
-      <c r="B49" s="24" t="s">
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B51" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C49" s="24" t="s">
+      <c r="C51" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="D49" s="24" t="s">
+      <c r="D51" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="E49" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="26" t="n">
-        <v>10000</v>
-      </c>
-      <c r="B50" s="17" t="n">
-        <f aca="false">IF(OR($A50&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A50)*(1-$B$8))*B$25+($A50*(1-$B$8))*B$30)/(((B$19-$A50)*(1-$B$8))+($A50*(1-$B$8))))*(1-((((B$19-$A50)*(1-$B$8))*B$25+($A50*(1-$B$8))*B$30)/(((B$19-$A50)*(1-$B$8))+($A50*(1-$B$8)))))*(1/((B$19-$A50)*(1-$B$8))+1/($A50*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A50)*(1-$B$8))+B$30*(1-B$30)/($A50*(1-$B$8)))))</f>
-        <v>0.159233528632258</v>
-      </c>
-      <c r="C50" s="17" t="n">
-        <f aca="false">IF(OR($A50&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A50)*(1-$B$8))*C$25+($A50*(1-$B$8))*C$30)/(((C$19-$A50)*(1-$B$8))+($A50*(1-$B$8))))*(1-((((C$19-$A50)*(1-$B$8))*C$25+($A50*(1-$B$8))*C$30)/(((C$19-$A50)*(1-$B$8))+($A50*(1-$B$8)))))*(1/((C$19-$A50)*(1-$B$8))+1/($A50*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A50)*(1-$B$8))+C$30*(1-C$30)/($A50*(1-$B$8)))))</f>
-        <v>0.0744729646625192</v>
-      </c>
-      <c r="D50" s="17" t="n">
-        <f aca="false">IF(OR($A50&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A50)*(1-$B$8))*D$25+($A50*(1-$B$8))*D$30)/(((D$19-$A50)*(1-$B$8))+($A50*(1-$B$8))))*(1-((((D$19-$A50)*(1-$B$8))*D$25+($A50*(1-$B$8))*D$30)/(((D$19-$A50)*(1-$B$8))+($A50*(1-$B$8)))))*(1/((D$19-$A50)*(1-$B$8))+1/($A50*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A50)*(1-$B$8))+D$30*(1-D$30)/($A50*(1-$B$8)))))</f>
-        <v>0.0473490763527856</v>
-      </c>
-      <c r="F50" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B50),B50&gt;=$B$6),$A50,"")</f>
-        <v/>
-      </c>
-      <c r="G50" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C50),C50&gt;=$B$6),$A50,"")</f>
-        <v/>
-      </c>
-      <c r="H50" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D50),D50&gt;=$B$6),$A50,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="26" t="n">
-        <v>25000</v>
-      </c>
-      <c r="B51" s="17" t="n">
-        <f aca="false">IF(OR($A51&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A51)*(1-$B$8))*B$25+($A51*(1-$B$8))*B$30)/(((B$19-$A51)*(1-$B$8))+($A51*(1-$B$8))))*(1-((((B$19-$A51)*(1-$B$8))*B$25+($A51*(1-$B$8))*B$30)/(((B$19-$A51)*(1-$B$8))+($A51*(1-$B$8)))))*(1/((B$19-$A51)*(1-$B$8))+1/($A51*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A51)*(1-$B$8))+B$30*(1-B$30)/($A51*(1-$B$8)))))</f>
-        <v>0.274910152696791</v>
-      </c>
-      <c r="C51" s="17" t="n">
-        <f aca="false">IF(OR($A51&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A51)*(1-$B$8))*C$25+($A51*(1-$B$8))*C$30)/(((C$19-$A51)*(1-$B$8))+($A51*(1-$B$8))))*(1-((((C$19-$A51)*(1-$B$8))*C$25+($A51*(1-$B$8))*C$30)/(((C$19-$A51)*(1-$B$8))+($A51*(1-$B$8)))))*(1/((C$19-$A51)*(1-$B$8))+1/($A51*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A51)*(1-$B$8))+C$30*(1-C$30)/($A51*(1-$B$8)))))</f>
-        <v>0.109445307468781</v>
-      </c>
-      <c r="D51" s="17" t="n">
-        <f aca="false">IF(OR($A51&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A51)*(1-$B$8))*D$25+($A51*(1-$B$8))*D$30)/(((D$19-$A51)*(1-$B$8))+($A51*(1-$B$8))))*(1-((((D$19-$A51)*(1-$B$8))*D$25+($A51*(1-$B$8))*D$30)/(((D$19-$A51)*(1-$B$8))+($A51*(1-$B$8)))))*(1/((D$19-$A51)*(1-$B$8))+1/($A51*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A51)*(1-$B$8))+D$30*(1-D$30)/($A51*(1-$B$8)))))</f>
-        <v>0.0796253915860124</v>
-      </c>
-      <c r="F51" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B51),B51&gt;=$B$6),$A51,"")</f>
-        <v/>
-      </c>
-      <c r="G51" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C51),C51&gt;=$B$6),$A51,"")</f>
-        <v/>
-      </c>
-      <c r="H51" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D51),D51&gt;=$B$6),$A51,"")</f>
-        <v/>
+      <c r="E51" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="26" t="n">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="B52" s="17" t="n">
         <f aca="false">IF(OR($A52&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A52)*(1-$B$8))*B$25+($A52*(1-$B$8))*B$30)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((B$19-$A52)*(1-$B$8))*B$25+($A52*(1-$B$8))*B$30)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((B$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A52)*(1-$B$8))+B$30*(1-B$30)/($A52*(1-$B$8)))))</f>
-        <v>0.430336919216376</v>
+        <v>0.159233528632258</v>
       </c>
       <c r="C52" s="17" t="n">
         <f aca="false">IF(OR($A52&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A52)*(1-$B$8))*C$25+($A52*(1-$B$8))*C$30)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((C$19-$A52)*(1-$B$8))*C$25+($A52*(1-$B$8))*C$30)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((C$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A52)*(1-$B$8))+C$30*(1-C$30)/($A52*(1-$B$8)))))</f>
-        <v>0.158142581595719</v>
+        <v>0.0744729646625192</v>
       </c>
       <c r="D52" s="17" t="n">
         <f aca="false">IF(OR($A52&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A52)*(1-$B$8))*D$25+($A52*(1-$B$8))*D$30)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((D$19-$A52)*(1-$B$8))*D$25+($A52*(1-$B$8))*D$30)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((D$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A52)*(1-$B$8))+D$30*(1-D$30)/($A52*(1-$B$8)))))</f>
-        <v>0.133014193269905</v>
+        <v>0.0473490763527856</v>
       </c>
       <c r="F52" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(B52),B52&gt;=$B$6),$A52,"")</f>
@@ -1646,19 +1643,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="26" t="n">
-        <v>100000</v>
+        <v>25000</v>
       </c>
       <c r="B53" s="17" t="n">
         <f aca="false">IF(OR($A53&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A53)*(1-$B$8))*B$25+($A53*(1-$B$8))*B$30)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((B$19-$A53)*(1-$B$8))*B$25+($A53*(1-$B$8))*B$30)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((B$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A53)*(1-$B$8))+B$30*(1-B$30)/($A53*(1-$B$8)))))</f>
-        <v>0.636690055383955</v>
+        <v>0.274910152696791</v>
       </c>
       <c r="C53" s="17" t="n">
         <f aca="false">IF(OR($A53&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A53)*(1-$B$8))*C$25+($A53*(1-$B$8))*C$30)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((C$19-$A53)*(1-$B$8))*C$25+($A53*(1-$B$8))*C$30)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((C$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A53)*(1-$B$8))+C$30*(1-C$30)/($A53*(1-$B$8)))))</f>
-        <v>0.237238824135504</v>
+        <v>0.109445307468781</v>
       </c>
       <c r="D53" s="17" t="n">
         <f aca="false">IF(OR($A53&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A53)*(1-$B$8))*D$25+($A53*(1-$B$8))*D$30)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((D$19-$A53)*(1-$B$8))*D$25+($A53*(1-$B$8))*D$30)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((D$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A53)*(1-$B$8))+D$30*(1-D$30)/($A53*(1-$B$8)))))</f>
-        <v>0.242152249674039</v>
+        <v>0.0796253915860124</v>
       </c>
       <c r="F53" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(B53),B53&gt;=$B$6),$A53,"")</f>
@@ -1675,23 +1672,23 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="26" t="n">
-        <v>250000</v>
+        <v>50000</v>
       </c>
       <c r="B54" s="17" t="n">
         <f aca="false">IF(OR($A54&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A54)*(1-$B$8))*B$25+($A54*(1-$B$8))*B$30)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((B$19-$A54)*(1-$B$8))*B$25+($A54*(1-$B$8))*B$30)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((B$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A54)*(1-$B$8))+B$30*(1-B$30)/($A54*(1-$B$8)))))</f>
-        <v>0.830962778781712</v>
+        <v>0.430336919216376</v>
       </c>
       <c r="C54" s="17" t="n">
         <f aca="false">IF(OR($A54&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A54)*(1-$B$8))*C$25+($A54*(1-$B$8))*C$30)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((C$19-$A54)*(1-$B$8))*C$25+($A54*(1-$B$8))*C$30)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((C$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A54)*(1-$B$8))+C$30*(1-C$30)/($A54*(1-$B$8)))))</f>
-        <v>0.36681549520206</v>
+        <v>0.158142581595719</v>
       </c>
       <c r="D54" s="17" t="n">
         <f aca="false">IF(OR($A54&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A54)*(1-$B$8))*D$25+($A54*(1-$B$8))*D$30)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((D$19-$A54)*(1-$B$8))*D$25+($A54*(1-$B$8))*D$30)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((D$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A54)*(1-$B$8))+D$30*(1-D$30)/($A54*(1-$B$8)))))</f>
-        <v>0.536974464177551</v>
-      </c>
-      <c r="F54" s="27" t="n">
+        <v>0.133014193269905</v>
+      </c>
+      <c r="F54" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(B54),B54&gt;=$B$6),$A54,"")</f>
-        <v>250000</v>
+        <v/>
       </c>
       <c r="G54" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(C54),C54&gt;=$B$6),$A54,"")</f>
@@ -1704,19 +1701,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="26" t="n">
-        <v>500000</v>
+        <v>100000</v>
       </c>
       <c r="B55" s="17" t="n">
         <f aca="false">IF(OR($A55&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A55)*(1-$B$8))*B$25+($A55*(1-$B$8))*B$30)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((B$19-$A55)*(1-$B$8))*B$25+($A55*(1-$B$8))*B$30)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((B$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A55)*(1-$B$8))+B$30*(1-B$30)/($A55*(1-$B$8)))))</f>
-        <v>0.408153831705151</v>
+        <v>0.636690055383955</v>
       </c>
       <c r="C55" s="17" t="n">
         <f aca="false">IF(OR($A55&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A55)*(1-$B$8))*C$25+($A55*(1-$B$8))*C$30)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((C$19-$A55)*(1-$B$8))*C$25+($A55*(1-$B$8))*C$30)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((C$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A55)*(1-$B$8))+C$30*(1-C$30)/($A55*(1-$B$8)))))</f>
-        <v>0.28483495767885</v>
+        <v>0.237238824135504</v>
       </c>
       <c r="D55" s="17" t="n">
         <f aca="false">IF(OR($A55&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A55)*(1-$B$8))*D$25+($A55*(1-$B$8))*D$30)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((D$19-$A55)*(1-$B$8))*D$25+($A55*(1-$B$8))*D$30)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((D$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A55)*(1-$B$8))+D$30*(1-D$30)/($A55*(1-$B$8)))))</f>
-        <v>0.820893449627511</v>
+        <v>0.242152249674039</v>
       </c>
       <c r="F55" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(B55),B55&gt;=$B$6),$A55,"")</f>
@@ -1726,55 +1723,55 @@
         <f aca="false">IF(AND(ISNUMBER(C55),C55&gt;=$B$6),$A55,"")</f>
         <v/>
       </c>
-      <c r="H55" s="27" t="n">
+      <c r="H55" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(D55),D55&gt;=$B$6),$A55,"")</f>
-        <v>500000</v>
+        <v/>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="26" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="B56" s="17" t="str">
+        <v>250000</v>
+      </c>
+      <c r="B56" s="17" t="n">
         <f aca="false">IF(OR($A56&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A56)*(1-$B$8))*B$25+($A56*(1-$B$8))*B$30)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((B$19-$A56)*(1-$B$8))*B$25+($A56*(1-$B$8))*B$30)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((B$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A56)*(1-$B$8))+B$30*(1-B$30)/($A56*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="C56" s="17" t="str">
+        <v>0.830962778781712</v>
+      </c>
+      <c r="C56" s="17" t="n">
         <f aca="false">IF(OR($A56&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A56)*(1-$B$8))*C$25+($A56*(1-$B$8))*C$30)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((C$19-$A56)*(1-$B$8))*C$25+($A56*(1-$B$8))*C$30)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((C$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A56)*(1-$B$8))+C$30*(1-C$30)/($A56*(1-$B$8)))))</f>
-        <v/>
+        <v>0.36681549520206</v>
       </c>
       <c r="D56" s="17" t="n">
         <f aca="false">IF(OR($A56&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A56)*(1-$B$8))*D$25+($A56*(1-$B$8))*D$30)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((D$19-$A56)*(1-$B$8))*D$25+($A56*(1-$B$8))*D$30)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((D$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A56)*(1-$B$8))+D$30*(1-D$30)/($A56*(1-$B$8)))))</f>
-        <v>0.971283737774168</v>
-      </c>
-      <c r="F56" s="27" t="str">
+        <v>0.536974464177551</v>
+      </c>
+      <c r="F56" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(B56),B56&gt;=$B$6),$A56,"")</f>
-        <v/>
+        <v>250000</v>
       </c>
       <c r="G56" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(C56),C56&gt;=$B$6),$A56,"")</f>
         <v/>
       </c>
-      <c r="H56" s="27" t="n">
+      <c r="H56" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(D56),D56&gt;=$B$6),$A56,"")</f>
-        <v>1000000</v>
+        <v/>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="26" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="B57" s="17" t="str">
+        <v>500000</v>
+      </c>
+      <c r="B57" s="17" t="n">
         <f aca="false">IF(OR($A57&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A57)*(1-$B$8))*B$25+($A57*(1-$B$8))*B$30)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((B$19-$A57)*(1-$B$8))*B$25+($A57*(1-$B$8))*B$30)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((B$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A57)*(1-$B$8))+B$30*(1-B$30)/($A57*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="C57" s="17" t="str">
+        <v>0.408153831705151</v>
+      </c>
+      <c r="C57" s="17" t="n">
         <f aca="false">IF(OR($A57&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A57)*(1-$B$8))*C$25+($A57*(1-$B$8))*C$30)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((C$19-$A57)*(1-$B$8))*C$25+($A57*(1-$B$8))*C$30)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((C$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A57)*(1-$B$8))+C$30*(1-C$30)/($A57*(1-$B$8)))))</f>
-        <v/>
+        <v>0.28483495767885</v>
       </c>
       <c r="D57" s="17" t="n">
         <f aca="false">IF(OR($A57&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A57)*(1-$B$8))*D$25+($A57*(1-$B$8))*D$30)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((D$19-$A57)*(1-$B$8))*D$25+($A57*(1-$B$8))*D$30)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((D$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A57)*(1-$B$8))+D$30*(1-D$30)/($A57*(1-$B$8)))))</f>
-        <v>0.996502733288146</v>
+        <v>0.820893449627511</v>
       </c>
       <c r="F57" s="27" t="str">
         <f aca="false">IF(AND(ISNUMBER(B57),B57&gt;=$B$6),$A57,"")</f>
@@ -1786,31 +1783,89 @@
       </c>
       <c r="H57" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(D57),D57&gt;=$B$6),$A57,"")</f>
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="B58" s="17" t="str">
+        <f aca="false">IF(OR($A58&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A58)*(1-$B$8))*B$25+($A58*(1-$B$8))*B$30)/(((B$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((B$19-$A58)*(1-$B$8))*B$25+($A58*(1-$B$8))*B$30)/(((B$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((B$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A58)*(1-$B$8))+B$30*(1-B$30)/($A58*(1-$B$8)))))</f>
+        <v/>
+      </c>
+      <c r="C58" s="17" t="str">
+        <f aca="false">IF(OR($A58&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A58)*(1-$B$8))*C$25+($A58*(1-$B$8))*C$30)/(((C$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((C$19-$A58)*(1-$B$8))*C$25+($A58*(1-$B$8))*C$30)/(((C$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((C$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A58)*(1-$B$8))+C$30*(1-C$30)/($A58*(1-$B$8)))))</f>
+        <v/>
+      </c>
+      <c r="D58" s="17" t="n">
+        <f aca="false">IF(OR($A58&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A58)*(1-$B$8))*D$25+($A58*(1-$B$8))*D$30)/(((D$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((D$19-$A58)*(1-$B$8))*D$25+($A58*(1-$B$8))*D$30)/(((D$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((D$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A58)*(1-$B$8))+D$30*(1-D$30)/($A58*(1-$B$8)))))</f>
+        <v>0.971283737774168</v>
+      </c>
+      <c r="F58" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B58),B58&gt;=$B$6),$A58,"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C58),C58&gt;=$B$6),$A58,"")</f>
+        <v/>
+      </c>
+      <c r="H58" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D58),D58&gt;=$B$6),$A58,"")</f>
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="26" t="n">
         <v>2000000</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="B59" s="28"/>
-      <c r="C59" s="28"/>
-      <c r="D59" s="28"/>
-      <c r="E59" s="28"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="28"/>
-      <c r="B60" s="28"/>
-      <c r="C60" s="28"/>
-      <c r="D60" s="28"/>
-      <c r="E60" s="28"/>
+      <c r="B59" s="17" t="str">
+        <f aca="false">IF(OR($A59&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A59)*(1-$B$8))*B$25+($A59*(1-$B$8))*B$30)/(((B$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((B$19-$A59)*(1-$B$8))*B$25+($A59*(1-$B$8))*B$30)/(((B$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((B$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A59)*(1-$B$8))+B$30*(1-B$30)/($A59*(1-$B$8)))))</f>
+        <v/>
+      </c>
+      <c r="C59" s="17" t="str">
+        <f aca="false">IF(OR($A59&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A59)*(1-$B$8))*C$25+($A59*(1-$B$8))*C$30)/(((C$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((C$19-$A59)*(1-$B$8))*C$25+($A59*(1-$B$8))*C$30)/(((C$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((C$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A59)*(1-$B$8))+C$30*(1-C$30)/($A59*(1-$B$8)))))</f>
+        <v/>
+      </c>
+      <c r="D59" s="17" t="n">
+        <f aca="false">IF(OR($A59&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A59)*(1-$B$8))*D$25+($A59*(1-$B$8))*D$30)/(((D$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((D$19-$A59)*(1-$B$8))*D$25+($A59*(1-$B$8))*D$30)/(((D$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((D$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A59)*(1-$B$8))+D$30*(1-D$30)/($A59*(1-$B$8)))))</f>
+        <v>0.996502733288146</v>
+      </c>
+      <c r="F59" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B59),B59&gt;=$B$6),$A59,"")</f>
+        <v/>
+      </c>
+      <c r="G59" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C59),C59&gt;=$B$6),$A59,"")</f>
+        <v/>
+      </c>
+      <c r="H59" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D59),D59&gt;=$B$6),$A59,"")</f>
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="B61" s="28"/>
+      <c r="C61" s="28"/>
+      <c r="D61" s="28"/>
+      <c r="E61" s="28"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="28"/>
+      <c r="B62" s="28"/>
+      <c r="C62" s="28"/>
+      <c r="D62" s="28"/>
+      <c r="E62" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="A59:E60"/>
+    <mergeCell ref="A61:E62"/>
   </mergeCells>
-  <conditionalFormatting sqref="B50:D57">
+  <conditionalFormatting sqref="B52:D59">
     <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$B$6</formula>
     </cfRule>
@@ -1823,8 +1878,16 @@
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B37:D37">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>LEFT(B37,2)="SÍ"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>LEFT(B37,2)="NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B26:D26">
-    <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+    <cfRule type="cellIs" priority="7" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1843,7 +1906,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -1851,45 +1914,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="29" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="29" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="29" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29"/>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
-        <v>81</v>
+      <c r="A9" s="29" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="29"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="29" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calculator v7: power table as pool percentages so minimum works for any pool size
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ygiEd3g3fKiFCARJZcKLp
</commit_message>
<xml_diff>
--- a/calculadora-sample-size.xlsx
+++ b/calculadora-sample-size.xlsx
@@ -212,7 +212,7 @@
     <t xml:space="preserve">Mínimo de usuarios en tratamiento para llegar al poder</t>
   </si>
   <si>
-    <t xml:space="preserve">Sale de la tabla de abajo. Pon ese número (o más) en 'Usuarios en TRATAMIENTO'.</t>
+    <t xml:space="preserve">Sale de la tabla de abajo (en % del pool). Pon ese número o más en 'Usuarios en TRATAMIENTO'. Si dice que no llega, revisa SAMPLE SIZE: si cabe, usa la mitad del pool.</t>
   </si>
   <si>
     <t xml:space="preserve">Qué hacer</t>
@@ -245,10 +245,10 @@
     <t xml:space="preserve">Iteración 4 = mínimo detectable (pp)</t>
   </si>
   <si>
-    <t xml:space="preserve">PODER SEGÚN USUARIOS EN TRATAMIENTO (control = resto del pool)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usa esta tabla para escoger cuántos usuarios meter</t>
+    <t xml:space="preserve">PODER SEGÚN % DEL POOL EN TRATAMIENTO (control = resto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poder si metes ese % del pool de cada tier. 50% es el máximo útil.</t>
   </si>
   <si>
     <t xml:space="preserve">auxiliar</t>
@@ -288,7 +288,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
@@ -299,6 +299,7 @@
     <numFmt numFmtId="171" formatCode="0.000%"/>
     <numFmt numFmtId="172" formatCode="\$#,##0;[RED]&quot;-$&quot;#,##0"/>
     <numFmt numFmtId="173" formatCode="0.00000"/>
+    <numFmt numFmtId="174" formatCode="0%&quot; del pool&quot;"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -567,7 +568,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -891,7 +892,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -1409,16 +1410,16 @@
         <v>62</v>
       </c>
       <c r="B38" s="22" t="n">
-        <f aca="false">IF(COUNT(F52:F59)=0,"No llega ni con todo el pool",MIN(F52:F59))</f>
-        <v>250000</v>
+        <f aca="false">IF(COUNT(F52:F58)=0,"No llega ni con todo el pool",MIN(F52:F58))</f>
+        <v>224864</v>
       </c>
       <c r="C38" s="22" t="str">
-        <f aca="false">IF(COUNT(G52:G59)=0,"No llega ni con todo el pool",MIN(G52:G59))</f>
+        <f aca="false">IF(COUNT(G52:G58)=0,"No llega ni con todo el pool",MIN(G52:G58))</f>
         <v>No llega ni con todo el pool</v>
       </c>
       <c r="D38" s="22" t="n">
-        <f aca="false">IF(COUNT(H52:H59)=0,"No llega ni con todo el pool",MIN(H52:H59))</f>
-        <v>500000</v>
+        <f aca="false">IF(COUNT(H52:H58)=0,"No llega ni con todo el pool",MIN(H52:H58))</f>
+        <v>698161</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>63</v>
@@ -1614,258 +1615,229 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="26" t="n">
-        <v>10000</v>
+        <v>0.05</v>
       </c>
       <c r="B52" s="17" t="n">
-        <f aca="false">IF(OR($A52&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A52)*(1-$B$8))*B$25+($A52*(1-$B$8))*B$30)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((B$19-$A52)*(1-$B$8))*B$25+($A52*(1-$B$8))*B$30)/(((B$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((B$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A52)*(1-$B$8))+B$30*(1-B$30)/($A52*(1-$B$8)))))</f>
-        <v>0.159233528632258</v>
+        <f aca="false">IF(B$29=0,"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT((((B$19*(1-$A52)*(1-$B$8))*B$25+(B$19*$A52*(1-$B$8))*B$30)/((B$19*(1-$A52)*(1-$B$8))+(B$19*$A52*(1-$B$8))))*(1-(((B$19*(1-$A52)*(1-$B$8))*B$25+(B$19*$A52*(1-$B$8))*B$30)/((B$19*(1-$A52)*(1-$B$8))+(B$19*$A52*(1-$B$8)))))*(1/(B$19*(1-$A52)*(1-$B$8))+1/(B$19*$A52*(1-$B$8)))))/SQRT(B$25*(1-B$25)/(B$19*(1-$A52)*(1-$B$8))+B$30*(1-B$30)/(B$19*$A52*(1-$B$8)))))</f>
+        <v>0.296524476018358</v>
       </c>
       <c r="C52" s="17" t="n">
-        <f aca="false">IF(OR($A52&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A52)*(1-$B$8))*C$25+($A52*(1-$B$8))*C$30)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((C$19-$A52)*(1-$B$8))*C$25+($A52*(1-$B$8))*C$30)/(((C$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((C$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A52)*(1-$B$8))+C$30*(1-C$30)/($A52*(1-$B$8)))))</f>
-        <v>0.0744729646625192</v>
+        <f aca="false">IF(C$29=0,"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT((((C$19*(1-$A52)*(1-$B$8))*C$25+(C$19*$A52*(1-$B$8))*C$30)/((C$19*(1-$A52)*(1-$B$8))+(C$19*$A52*(1-$B$8))))*(1-(((C$19*(1-$A52)*(1-$B$8))*C$25+(C$19*$A52*(1-$B$8))*C$30)/((C$19*(1-$A52)*(1-$B$8))+(C$19*$A52*(1-$B$8)))))*(1/(C$19*(1-$A52)*(1-$B$8))+1/(C$19*$A52*(1-$B$8)))))/SQRT(C$25*(1-C$25)/(C$19*(1-$A52)*(1-$B$8))+C$30*(1-C$30)/(C$19*$A52*(1-$B$8)))))</f>
+        <v>0.126765130489271</v>
       </c>
       <c r="D52" s="17" t="n">
-        <f aca="false">IF(OR($A52&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A52)*(1-$B$8))*D$25+($A52*(1-$B$8))*D$30)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8))))*(1-((((D$19-$A52)*(1-$B$8))*D$25+($A52*(1-$B$8))*D$30)/(((D$19-$A52)*(1-$B$8))+($A52*(1-$B$8)))))*(1/((D$19-$A52)*(1-$B$8))+1/($A52*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A52)*(1-$B$8))+D$30*(1-D$30)/($A52*(1-$B$8)))))</f>
-        <v>0.0473490763527856</v>
+        <f aca="false">IF(D$29=0,"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT((((D$19*(1-$A52)*(1-$B$8))*D$25+(D$19*$A52*(1-$B$8))*D$30)/((D$19*(1-$A52)*(1-$B$8))+(D$19*$A52*(1-$B$8))))*(1-(((D$19*(1-$A52)*(1-$B$8))*D$25+(D$19*$A52*(1-$B$8))*D$30)/((D$19*(1-$A52)*(1-$B$8))+(D$19*$A52*(1-$B$8)))))*(1/(D$19*(1-$A52)*(1-$B$8))+1/(D$19*$A52*(1-$B$8)))))/SQRT(D$25*(1-D$25)/(D$19*(1-$A52)*(1-$B$8))+D$30*(1-D$30)/(D$19*$A52*(1-$B$8)))))</f>
+        <v>0.50757784417896</v>
       </c>
       <c r="F52" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B52),B52&gt;=$B$6),$A52,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(B52),B52&gt;=$B$6),ROUND(B$19*$A52,0),"")</f>
         <v/>
       </c>
       <c r="G52" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C52),C52&gt;=$B$6),$A52,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(C52),C52&gt;=$B$6),ROUND(C$19*$A52,0),"")</f>
         <v/>
       </c>
       <c r="H52" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D52),D52&gt;=$B$6),$A52,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(D52),D52&gt;=$B$6),ROUND(D$19*$A52,0),"")</f>
         <v/>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="26" t="n">
-        <v>25000</v>
+        <v>0.1</v>
       </c>
       <c r="B53" s="17" t="n">
-        <f aca="false">IF(OR($A53&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A53)*(1-$B$8))*B$25+($A53*(1-$B$8))*B$30)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((B$19-$A53)*(1-$B$8))*B$25+($A53*(1-$B$8))*B$30)/(((B$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((B$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A53)*(1-$B$8))+B$30*(1-B$30)/($A53*(1-$B$8)))))</f>
-        <v>0.274910152696791</v>
+        <f aca="false">IF(B$29=0,"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT((((B$19*(1-$A53)*(1-$B$8))*B$25+(B$19*$A53*(1-$B$8))*B$30)/((B$19*(1-$A53)*(1-$B$8))+(B$19*$A53*(1-$B$8))))*(1-(((B$19*(1-$A53)*(1-$B$8))*B$25+(B$19*$A53*(1-$B$8))*B$30)/((B$19*(1-$A53)*(1-$B$8))+(B$19*$A53*(1-$B$8)))))*(1/(B$19*(1-$A53)*(1-$B$8))+1/(B$19*$A53*(1-$B$8)))))/SQRT(B$25*(1-B$25)/(B$19*(1-$A53)*(1-$B$8))+B$30*(1-B$30)/(B$19*$A53*(1-$B$8)))))</f>
+        <v>0.462915743014895</v>
       </c>
       <c r="C53" s="17" t="n">
-        <f aca="false">IF(OR($A53&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A53)*(1-$B$8))*C$25+($A53*(1-$B$8))*C$30)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((C$19-$A53)*(1-$B$8))*C$25+($A53*(1-$B$8))*C$30)/(((C$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((C$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A53)*(1-$B$8))+C$30*(1-C$30)/($A53*(1-$B$8)))))</f>
-        <v>0.109445307468781</v>
+        <f aca="false">IF(C$29=0,"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT((((C$19*(1-$A53)*(1-$B$8))*C$25+(C$19*$A53*(1-$B$8))*C$30)/((C$19*(1-$A53)*(1-$B$8))+(C$19*$A53*(1-$B$8))))*(1-(((C$19*(1-$A53)*(1-$B$8))*C$25+(C$19*$A53*(1-$B$8))*C$30)/((C$19*(1-$A53)*(1-$B$8))+(C$19*$A53*(1-$B$8)))))*(1/(C$19*(1-$A53)*(1-$B$8))+1/(C$19*$A53*(1-$B$8)))))/SQRT(C$25*(1-C$25)/(C$19*(1-$A53)*(1-$B$8))+C$30*(1-C$30)/(C$19*$A53*(1-$B$8)))))</f>
+        <v>0.18714453759629</v>
       </c>
       <c r="D53" s="17" t="n">
-        <f aca="false">IF(OR($A53&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A53)*(1-$B$8))*D$25+($A53*(1-$B$8))*D$30)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8))))*(1-((((D$19-$A53)*(1-$B$8))*D$25+($A53*(1-$B$8))*D$30)/(((D$19-$A53)*(1-$B$8))+($A53*(1-$B$8)))))*(1/((D$19-$A53)*(1-$B$8))+1/($A53*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A53)*(1-$B$8))+D$30*(1-D$30)/($A53*(1-$B$8)))))</f>
-        <v>0.0796253915860124</v>
+        <f aca="false">IF(D$29=0,"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT((((D$19*(1-$A53)*(1-$B$8))*D$25+(D$19*$A53*(1-$B$8))*D$30)/((D$19*(1-$A53)*(1-$B$8))+(D$19*$A53*(1-$B$8))))*(1-(((D$19*(1-$A53)*(1-$B$8))*D$25+(D$19*$A53*(1-$B$8))*D$30)/((D$19*(1-$A53)*(1-$B$8))+(D$19*$A53*(1-$B$8)))))*(1/(D$19*(1-$A53)*(1-$B$8))+1/(D$19*$A53*(1-$B$8)))))/SQRT(D$25*(1-D$25)/(D$19*(1-$A53)*(1-$B$8))+D$30*(1-D$30)/(D$19*$A53*(1-$B$8)))))</f>
+        <v>0.79513392381669</v>
       </c>
       <c r="F53" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B53),B53&gt;=$B$6),$A53,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(B53),B53&gt;=$B$6),ROUND(B$19*$A53,0),"")</f>
         <v/>
       </c>
       <c r="G53" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C53),C53&gt;=$B$6),$A53,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(C53),C53&gt;=$B$6),ROUND(C$19*$A53,0),"")</f>
         <v/>
       </c>
       <c r="H53" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D53),D53&gt;=$B$6),$A53,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(D53),D53&gt;=$B$6),ROUND(D$19*$A53,0),"")</f>
         <v/>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="26" t="n">
-        <v>50000</v>
+        <v>0.15</v>
       </c>
       <c r="B54" s="17" t="n">
-        <f aca="false">IF(OR($A54&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A54)*(1-$B$8))*B$25+($A54*(1-$B$8))*B$30)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((B$19-$A54)*(1-$B$8))*B$25+($A54*(1-$B$8))*B$30)/(((B$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((B$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A54)*(1-$B$8))+B$30*(1-B$30)/($A54*(1-$B$8)))))</f>
-        <v>0.430336919216376</v>
+        <f aca="false">IF(B$29=0,"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT((((B$19*(1-$A54)*(1-$B$8))*B$25+(B$19*$A54*(1-$B$8))*B$30)/((B$19*(1-$A54)*(1-$B$8))+(B$19*$A54*(1-$B$8))))*(1-(((B$19*(1-$A54)*(1-$B$8))*B$25+(B$19*$A54*(1-$B$8))*B$30)/((B$19*(1-$A54)*(1-$B$8))+(B$19*$A54*(1-$B$8)))))*(1/(B$19*(1-$A54)*(1-$B$8))+1/(B$19*$A54*(1-$B$8)))))/SQRT(B$25*(1-B$25)/(B$19*(1-$A54)*(1-$B$8))+B$30*(1-B$30)/(B$19*$A54*(1-$B$8)))))</f>
+        <v>0.584526275265234</v>
       </c>
       <c r="C54" s="17" t="n">
-        <f aca="false">IF(OR($A54&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A54)*(1-$B$8))*C$25+($A54*(1-$B$8))*C$30)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((C$19-$A54)*(1-$B$8))*C$25+($A54*(1-$B$8))*C$30)/(((C$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((C$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A54)*(1-$B$8))+C$30*(1-C$30)/($A54*(1-$B$8)))))</f>
-        <v>0.158142581595719</v>
+        <f aca="false">IF(C$29=0,"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT((((C$19*(1-$A54)*(1-$B$8))*C$25+(C$19*$A54*(1-$B$8))*C$30)/((C$19*(1-$A54)*(1-$B$8))+(C$19*$A54*(1-$B$8))))*(1-(((C$19*(1-$A54)*(1-$B$8))*C$25+(C$19*$A54*(1-$B$8))*C$30)/((C$19*(1-$A54)*(1-$B$8))+(C$19*$A54*(1-$B$8)))))*(1/(C$19*(1-$A54)*(1-$B$8))+1/(C$19*$A54*(1-$B$8)))))/SQRT(C$25*(1-C$25)/(C$19*(1-$A54)*(1-$B$8))+C$30*(1-C$30)/(C$19*$A54*(1-$B$8)))))</f>
+        <v>0.237594090132639</v>
       </c>
       <c r="D54" s="17" t="n">
-        <f aca="false">IF(OR($A54&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A54)*(1-$B$8))*D$25+($A54*(1-$B$8))*D$30)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8))))*(1-((((D$19-$A54)*(1-$B$8))*D$25+($A54*(1-$B$8))*D$30)/(((D$19-$A54)*(1-$B$8))+($A54*(1-$B$8)))))*(1/((D$19-$A54)*(1-$B$8))+1/($A54*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A54)*(1-$B$8))+D$30*(1-D$30)/($A54*(1-$B$8)))))</f>
-        <v>0.133014193269905</v>
+        <f aca="false">IF(D$29=0,"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT((((D$19*(1-$A54)*(1-$B$8))*D$25+(D$19*$A54*(1-$B$8))*D$30)/((D$19*(1-$A54)*(1-$B$8))+(D$19*$A54*(1-$B$8))))*(1-(((D$19*(1-$A54)*(1-$B$8))*D$25+(D$19*$A54*(1-$B$8))*D$30)/((D$19*(1-$A54)*(1-$B$8))+(D$19*$A54*(1-$B$8)))))*(1/(D$19*(1-$A54)*(1-$B$8))+1/(D$19*$A54*(1-$B$8)))))/SQRT(D$25*(1-D$25)/(D$19*(1-$A54)*(1-$B$8))+D$30*(1-D$30)/(D$19*$A54*(1-$B$8)))))</f>
+        <v>0.916369149506601</v>
       </c>
       <c r="F54" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B54),B54&gt;=$B$6),$A54,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(B54),B54&gt;=$B$6),ROUND(B$19*$A54,0),"")</f>
         <v/>
       </c>
       <c r="G54" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C54),C54&gt;=$B$6),$A54,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(C54),C54&gt;=$B$6),ROUND(C$19*$A54,0),"")</f>
         <v/>
       </c>
-      <c r="H54" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D54),D54&gt;=$B$6),$A54,"")</f>
-        <v/>
+      <c r="H54" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D54),D54&gt;=$B$6),ROUND(D$19*$A54,0),"")</f>
+        <v>698161</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="26" t="n">
-        <v>100000</v>
+        <v>0.2</v>
       </c>
       <c r="B55" s="17" t="n">
-        <f aca="false">IF(OR($A55&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A55)*(1-$B$8))*B$25+($A55*(1-$B$8))*B$30)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((B$19-$A55)*(1-$B$8))*B$25+($A55*(1-$B$8))*B$30)/(((B$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((B$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A55)*(1-$B$8))+B$30*(1-B$30)/($A55*(1-$B$8)))))</f>
-        <v>0.636690055383955</v>
+        <f aca="false">IF(B$29=0,"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT((((B$19*(1-$A55)*(1-$B$8))*B$25+(B$19*$A55*(1-$B$8))*B$30)/((B$19*(1-$A55)*(1-$B$8))+(B$19*$A55*(1-$B$8))))*(1-(((B$19*(1-$A55)*(1-$B$8))*B$25+(B$19*$A55*(1-$B$8))*B$30)/((B$19*(1-$A55)*(1-$B$8))+(B$19*$A55*(1-$B$8)))))*(1/(B$19*(1-$A55)*(1-$B$8))+1/(B$19*$A55*(1-$B$8)))))/SQRT(B$25*(1-B$25)/(B$19*(1-$A55)*(1-$B$8))+B$30*(1-B$30)/(B$19*$A55*(1-$B$8)))))</f>
+        <v>0.671503950505927</v>
       </c>
       <c r="C55" s="17" t="n">
-        <f aca="false">IF(OR($A55&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A55)*(1-$B$8))*C$25+($A55*(1-$B$8))*C$30)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((C$19-$A55)*(1-$B$8))*C$25+($A55*(1-$B$8))*C$30)/(((C$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((C$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A55)*(1-$B$8))+C$30*(1-C$30)/($A55*(1-$B$8)))))</f>
-        <v>0.237238824135504</v>
+        <f aca="false">IF(C$29=0,"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT((((C$19*(1-$A55)*(1-$B$8))*C$25+(C$19*$A55*(1-$B$8))*C$30)/((C$19*(1-$A55)*(1-$B$8))+(C$19*$A55*(1-$B$8))))*(1-(((C$19*(1-$A55)*(1-$B$8))*C$25+(C$19*$A55*(1-$B$8))*C$30)/((C$19*(1-$A55)*(1-$B$8))+(C$19*$A55*(1-$B$8)))))*(1/(C$19*(1-$A55)*(1-$B$8))+1/(C$19*$A55*(1-$B$8)))))/SQRT(C$25*(1-C$25)/(C$19*(1-$A55)*(1-$B$8))+C$30*(1-C$30)/(C$19*$A55*(1-$B$8)))))</f>
+        <v>0.279516639181519</v>
       </c>
       <c r="D55" s="17" t="n">
-        <f aca="false">IF(OR($A55&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A55)*(1-$B$8))*D$25+($A55*(1-$B$8))*D$30)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8))))*(1-((((D$19-$A55)*(1-$B$8))*D$25+($A55*(1-$B$8))*D$30)/(((D$19-$A55)*(1-$B$8))+($A55*(1-$B$8)))))*(1/((D$19-$A55)*(1-$B$8))+1/($A55*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A55)*(1-$B$8))+D$30*(1-D$30)/($A55*(1-$B$8)))))</f>
-        <v>0.242152249674039</v>
+        <f aca="false">IF(D$29=0,"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT((((D$19*(1-$A55)*(1-$B$8))*D$25+(D$19*$A55*(1-$B$8))*D$30)/((D$19*(1-$A55)*(1-$B$8))+(D$19*$A55*(1-$B$8))))*(1-(((D$19*(1-$A55)*(1-$B$8))*D$25+(D$19*$A55*(1-$B$8))*D$30)/((D$19*(1-$A55)*(1-$B$8))+(D$19*$A55*(1-$B$8)))))*(1/(D$19*(1-$A55)*(1-$B$8))+1/(D$19*$A55*(1-$B$8)))))/SQRT(D$25*(1-D$25)/(D$19*(1-$A55)*(1-$B$8))+D$30*(1-D$30)/(D$19*$A55*(1-$B$8)))))</f>
+        <v>0.963813145360621</v>
       </c>
       <c r="F55" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B55),B55&gt;=$B$6),$A55,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(B55),B55&gt;=$B$6),ROUND(B$19*$A55,0),"")</f>
         <v/>
       </c>
       <c r="G55" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C55),C55&gt;=$B$6),$A55,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(C55),C55&gt;=$B$6),ROUND(C$19*$A55,0),"")</f>
         <v/>
       </c>
-      <c r="H55" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D55),D55&gt;=$B$6),$A55,"")</f>
-        <v/>
+      <c r="H55" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D55),D55&gt;=$B$6),ROUND(D$19*$A55,0),"")</f>
+        <v>930881</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="26" t="n">
-        <v>250000</v>
+        <v>0.3</v>
       </c>
       <c r="B56" s="17" t="n">
-        <f aca="false">IF(OR($A56&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A56)*(1-$B$8))*B$25+($A56*(1-$B$8))*B$30)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((B$19-$A56)*(1-$B$8))*B$25+($A56*(1-$B$8))*B$30)/(((B$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((B$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A56)*(1-$B$8))+B$30*(1-B$30)/($A56*(1-$B$8)))))</f>
-        <v>0.830962778781712</v>
+        <f aca="false">IF(B$29=0,"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT((((B$19*(1-$A56)*(1-$B$8))*B$25+(B$19*$A56*(1-$B$8))*B$30)/((B$19*(1-$A56)*(1-$B$8))+(B$19*$A56*(1-$B$8))))*(1-(((B$19*(1-$A56)*(1-$B$8))*B$25+(B$19*$A56*(1-$B$8))*B$30)/((B$19*(1-$A56)*(1-$B$8))+(B$19*$A56*(1-$B$8)))))*(1/(B$19*(1-$A56)*(1-$B$8))+1/(B$19*$A56*(1-$B$8)))))/SQRT(B$25*(1-B$25)/(B$19*(1-$A56)*(1-$B$8))+B$30*(1-B$30)/(B$19*$A56*(1-$B$8)))))</f>
+        <v>0.775309578120823</v>
       </c>
       <c r="C56" s="17" t="n">
-        <f aca="false">IF(OR($A56&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A56)*(1-$B$8))*C$25+($A56*(1-$B$8))*C$30)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((C$19-$A56)*(1-$B$8))*C$25+($A56*(1-$B$8))*C$30)/(((C$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((C$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A56)*(1-$B$8))+C$30*(1-C$30)/($A56*(1-$B$8)))))</f>
-        <v>0.36681549520206</v>
+        <f aca="false">IF(C$29=0,"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT((((C$19*(1-$A56)*(1-$B$8))*C$25+(C$19*$A56*(1-$B$8))*C$30)/((C$19*(1-$A56)*(1-$B$8))+(C$19*$A56*(1-$B$8))))*(1-(((C$19*(1-$A56)*(1-$B$8))*C$25+(C$19*$A56*(1-$B$8))*C$30)/((C$19*(1-$A56)*(1-$B$8))+(C$19*$A56*(1-$B$8)))))*(1/(C$19*(1-$A56)*(1-$B$8))+1/(C$19*$A56*(1-$B$8)))))/SQRT(C$25*(1-C$25)/(C$19*(1-$A56)*(1-$B$8))+C$30*(1-C$30)/(C$19*$A56*(1-$B$8)))))</f>
+        <v>0.340166736556853</v>
       </c>
       <c r="D56" s="17" t="n">
-        <f aca="false">IF(OR($A56&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A56)*(1-$B$8))*D$25+($A56*(1-$B$8))*D$30)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8))))*(1-((((D$19-$A56)*(1-$B$8))*D$25+($A56*(1-$B$8))*D$30)/(((D$19-$A56)*(1-$B$8))+($A56*(1-$B$8)))))*(1/((D$19-$A56)*(1-$B$8))+1/($A56*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A56)*(1-$B$8))+D$30*(1-D$30)/($A56*(1-$B$8)))))</f>
-        <v>0.536974464177551</v>
-      </c>
-      <c r="F56" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(B56),B56&gt;=$B$6),$A56,"")</f>
-        <v>250000</v>
+        <f aca="false">IF(D$29=0,"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT((((D$19*(1-$A56)*(1-$B$8))*D$25+(D$19*$A56*(1-$B$8))*D$30)/((D$19*(1-$A56)*(1-$B$8))+(D$19*$A56*(1-$B$8))))*(1-(((D$19*(1-$A56)*(1-$B$8))*D$25+(D$19*$A56*(1-$B$8))*D$30)/((D$19*(1-$A56)*(1-$B$8))+(D$19*$A56*(1-$B$8)))))*(1/(D$19*(1-$A56)*(1-$B$8))+1/(D$19*$A56*(1-$B$8)))))/SQRT(D$25*(1-D$25)/(D$19*(1-$A56)*(1-$B$8))+D$30*(1-D$30)/(D$19*$A56*(1-$B$8)))))</f>
+        <v>0.990716985648439</v>
+      </c>
+      <c r="F56" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B56),B56&gt;=$B$6),ROUND(B$19*$A56,0),"")</f>
+        <v/>
       </c>
       <c r="G56" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C56),C56&gt;=$B$6),$A56,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(C56),C56&gt;=$B$6),ROUND(C$19*$A56,0),"")</f>
         <v/>
       </c>
-      <c r="H56" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D56),D56&gt;=$B$6),$A56,"")</f>
-        <v/>
+      <c r="H56" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D56),D56&gt;=$B$6),ROUND(D$19*$A56,0),"")</f>
+        <v>1396322</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="26" t="n">
-        <v>500000</v>
+        <v>0.4</v>
       </c>
       <c r="B57" s="17" t="n">
-        <f aca="false">IF(OR($A57&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A57)*(1-$B$8))*B$25+($A57*(1-$B$8))*B$30)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((B$19-$A57)*(1-$B$8))*B$25+($A57*(1-$B$8))*B$30)/(((B$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((B$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A57)*(1-$B$8))+B$30*(1-B$30)/($A57*(1-$B$8)))))</f>
-        <v>0.408153831705151</v>
+        <f aca="false">IF(B$29=0,"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT((((B$19*(1-$A57)*(1-$B$8))*B$25+(B$19*$A57*(1-$B$8))*B$30)/((B$19*(1-$A57)*(1-$B$8))+(B$19*$A57*(1-$B$8))))*(1-(((B$19*(1-$A57)*(1-$B$8))*B$25+(B$19*$A57*(1-$B$8))*B$30)/((B$19*(1-$A57)*(1-$B$8))+(B$19*$A57*(1-$B$8)))))*(1/(B$19*(1-$A57)*(1-$B$8))+1/(B$19*$A57*(1-$B$8)))))/SQRT(B$25*(1-B$25)/(B$19*(1-$A57)*(1-$B$8))+B$30*(1-B$30)/(B$19*$A57*(1-$B$8)))))</f>
+        <v>0.822055367812686</v>
       </c>
       <c r="C57" s="17" t="n">
-        <f aca="false">IF(OR($A57&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A57)*(1-$B$8))*C$25+($A57*(1-$B$8))*C$30)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((C$19-$A57)*(1-$B$8))*C$25+($A57*(1-$B$8))*C$30)/(((C$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((C$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A57)*(1-$B$8))+C$30*(1-C$30)/($A57*(1-$B$8)))))</f>
-        <v>0.28483495767885</v>
+        <f aca="false">IF(C$29=0,"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT((((C$19*(1-$A57)*(1-$B$8))*C$25+(C$19*$A57*(1-$B$8))*C$30)/((C$19*(1-$A57)*(1-$B$8))+(C$19*$A57*(1-$B$8))))*(1-(((C$19*(1-$A57)*(1-$B$8))*C$25+(C$19*$A57*(1-$B$8))*C$30)/((C$19*(1-$A57)*(1-$B$8))+(C$19*$A57*(1-$B$8)))))*(1/(C$19*(1-$A57)*(1-$B$8))+1/(C$19*$A57*(1-$B$8)))))/SQRT(C$25*(1-C$25)/(C$19*(1-$A57)*(1-$B$8))+C$30*(1-C$30)/(C$19*$A57*(1-$B$8)))))</f>
+        <v>0.372711646488239</v>
       </c>
       <c r="D57" s="17" t="n">
-        <f aca="false">IF(OR($A57&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A57)*(1-$B$8))*D$25+($A57*(1-$B$8))*D$30)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8))))*(1-((((D$19-$A57)*(1-$B$8))*D$25+($A57*(1-$B$8))*D$30)/(((D$19-$A57)*(1-$B$8))+($A57*(1-$B$8)))))*(1/((D$19-$A57)*(1-$B$8))+1/($A57*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A57)*(1-$B$8))+D$30*(1-D$30)/($A57*(1-$B$8)))))</f>
-        <v>0.820893449627511</v>
-      </c>
-      <c r="F57" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B57),B57&gt;=$B$6),$A57,"")</f>
+        <f aca="false">IF(D$29=0,"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT((((D$19*(1-$A57)*(1-$B$8))*D$25+(D$19*$A57*(1-$B$8))*D$30)/((D$19*(1-$A57)*(1-$B$8))+(D$19*$A57*(1-$B$8))))*(1-(((D$19*(1-$A57)*(1-$B$8))*D$25+(D$19*$A57*(1-$B$8))*D$30)/((D$19*(1-$A57)*(1-$B$8))+(D$19*$A57*(1-$B$8)))))*(1/(D$19*(1-$A57)*(1-$B$8))+1/(D$19*$A57*(1-$B$8)))))/SQRT(D$25*(1-D$25)/(D$19*(1-$A57)*(1-$B$8))+D$30*(1-D$30)/(D$19*$A57*(1-$B$8)))))</f>
+        <v>0.995979079431428</v>
+      </c>
+      <c r="F57" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(B57),B57&gt;=$B$6),ROUND(B$19*$A57,0),"")</f>
+        <v>224864</v>
+      </c>
+      <c r="G57" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C57),C57&gt;=$B$6),ROUND(C$19*$A57,0),"")</f>
         <v/>
       </c>
-      <c r="G57" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C57),C57&gt;=$B$6),$A57,"")</f>
-        <v/>
-      </c>
       <c r="H57" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(D57),D57&gt;=$B$6),$A57,"")</f>
-        <v>500000</v>
+        <f aca="false">IF(AND(ISNUMBER(D57),D57&gt;=$B$6),ROUND(D$19*$A57,0),"")</f>
+        <v>1861762</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="26" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="B58" s="17" t="str">
-        <f aca="false">IF(OR($A58&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A58)*(1-$B$8))*B$25+($A58*(1-$B$8))*B$30)/(((B$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((B$19-$A58)*(1-$B$8))*B$25+($A58*(1-$B$8))*B$30)/(((B$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((B$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A58)*(1-$B$8))+B$30*(1-B$30)/($A58*(1-$B$8)))))</f>
+        <v>0.5</v>
+      </c>
+      <c r="B58" s="17" t="n">
+        <f aca="false">IF(B$29=0,"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT((((B$19*(1-$A58)*(1-$B$8))*B$25+(B$19*$A58*(1-$B$8))*B$30)/((B$19*(1-$A58)*(1-$B$8))+(B$19*$A58*(1-$B$8))))*(1-(((B$19*(1-$A58)*(1-$B$8))*B$25+(B$19*$A58*(1-$B$8))*B$30)/((B$19*(1-$A58)*(1-$B$8))+(B$19*$A58*(1-$B$8)))))*(1/(B$19*(1-$A58)*(1-$B$8))+1/(B$19*$A58*(1-$B$8)))))/SQRT(B$25*(1-B$25)/(B$19*(1-$A58)*(1-$B$8))+B$30*(1-B$30)/(B$19*$A58*(1-$B$8)))))</f>
+        <v>0.833637561177275</v>
+      </c>
+      <c r="C58" s="17" t="n">
+        <f aca="false">IF(C$29=0,"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT((((C$19*(1-$A58)*(1-$B$8))*C$25+(C$19*$A58*(1-$B$8))*C$30)/((C$19*(1-$A58)*(1-$B$8))+(C$19*$A58*(1-$B$8))))*(1-(((C$19*(1-$A58)*(1-$B$8))*C$25+(C$19*$A58*(1-$B$8))*C$30)/((C$19*(1-$A58)*(1-$B$8))+(C$19*$A58*(1-$B$8)))))*(1/(C$19*(1-$A58)*(1-$B$8))+1/(C$19*$A58*(1-$B$8)))))/SQRT(C$25*(1-C$25)/(C$19*(1-$A58)*(1-$B$8))+C$30*(1-C$30)/(C$19*$A58*(1-$B$8)))))</f>
+        <v>0.379325029852179</v>
+      </c>
+      <c r="D58" s="17" t="n">
+        <f aca="false">IF(D$29=0,"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT((((D$19*(1-$A58)*(1-$B$8))*D$25+(D$19*$A58*(1-$B$8))*D$30)/((D$19*(1-$A58)*(1-$B$8))+(D$19*$A58*(1-$B$8))))*(1-(((D$19*(1-$A58)*(1-$B$8))*D$25+(D$19*$A58*(1-$B$8))*D$30)/((D$19*(1-$A58)*(1-$B$8))+(D$19*$A58*(1-$B$8)))))*(1/(D$19*(1-$A58)*(1-$B$8))+1/(D$19*$A58*(1-$B$8)))))/SQRT(D$25*(1-D$25)/(D$19*(1-$A58)*(1-$B$8))+D$30*(1-D$30)/(D$19*$A58*(1-$B$8)))))</f>
+        <v>0.996923475940705</v>
+      </c>
+      <c r="F58" s="27" t="n">
+        <f aca="false">IF(AND(ISNUMBER(B58),B58&gt;=$B$6),ROUND(B$19*$A58,0),"")</f>
+        <v>281080</v>
+      </c>
+      <c r="G58" s="27" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C58),C58&gt;=$B$6),ROUND(C$19*$A58,0),"")</f>
         <v/>
       </c>
-      <c r="C58" s="17" t="str">
-        <f aca="false">IF(OR($A58&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A58)*(1-$B$8))*C$25+($A58*(1-$B$8))*C$30)/(((C$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((C$19-$A58)*(1-$B$8))*C$25+($A58*(1-$B$8))*C$30)/(((C$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((C$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A58)*(1-$B$8))+C$30*(1-C$30)/($A58*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="D58" s="17" t="n">
-        <f aca="false">IF(OR($A58&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A58)*(1-$B$8))*D$25+($A58*(1-$B$8))*D$30)/(((D$19-$A58)*(1-$B$8))+($A58*(1-$B$8))))*(1-((((D$19-$A58)*(1-$B$8))*D$25+($A58*(1-$B$8))*D$30)/(((D$19-$A58)*(1-$B$8))+($A58*(1-$B$8)))))*(1/((D$19-$A58)*(1-$B$8))+1/($A58*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A58)*(1-$B$8))+D$30*(1-D$30)/($A58*(1-$B$8)))))</f>
-        <v>0.971283737774168</v>
-      </c>
-      <c r="F58" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B58),B58&gt;=$B$6),$A58,"")</f>
-        <v/>
-      </c>
-      <c r="G58" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C58),C58&gt;=$B$6),$A58,"")</f>
-        <v/>
-      </c>
       <c r="H58" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(D58),D58&gt;=$B$6),$A58,"")</f>
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="26" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="B59" s="17" t="str">
-        <f aca="false">IF(OR($A59&gt;=B$19,B$29=0),"",NORMSDIST((ABS(B$30-B$25)-$B$10*SQRT(((((B$19-$A59)*(1-$B$8))*B$25+($A59*(1-$B$8))*B$30)/(((B$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((B$19-$A59)*(1-$B$8))*B$25+($A59*(1-$B$8))*B$30)/(((B$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((B$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(B$25*(1-B$25)/((B$19-$A59)*(1-$B$8))+B$30*(1-B$30)/($A59*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="C59" s="17" t="str">
-        <f aca="false">IF(OR($A59&gt;=C$19,C$29=0),"",NORMSDIST((ABS(C$30-C$25)-$B$10*SQRT(((((C$19-$A59)*(1-$B$8))*C$25+($A59*(1-$B$8))*C$30)/(((C$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((C$19-$A59)*(1-$B$8))*C$25+($A59*(1-$B$8))*C$30)/(((C$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((C$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(C$25*(1-C$25)/((C$19-$A59)*(1-$B$8))+C$30*(1-C$30)/($A59*(1-$B$8)))))</f>
-        <v/>
-      </c>
-      <c r="D59" s="17" t="n">
-        <f aca="false">IF(OR($A59&gt;=D$19,D$29=0),"",NORMSDIST((ABS(D$30-D$25)-$B$10*SQRT(((((D$19-$A59)*(1-$B$8))*D$25+($A59*(1-$B$8))*D$30)/(((D$19-$A59)*(1-$B$8))+($A59*(1-$B$8))))*(1-((((D$19-$A59)*(1-$B$8))*D$25+($A59*(1-$B$8))*D$30)/(((D$19-$A59)*(1-$B$8))+($A59*(1-$B$8)))))*(1/((D$19-$A59)*(1-$B$8))+1/($A59*(1-$B$8)))))/SQRT(D$25*(1-D$25)/((D$19-$A59)*(1-$B$8))+D$30*(1-D$30)/($A59*(1-$B$8)))))</f>
-        <v>0.996502733288146</v>
-      </c>
-      <c r="F59" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(B59),B59&gt;=$B$6),$A59,"")</f>
-        <v/>
-      </c>
-      <c r="G59" s="27" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C59),C59&gt;=$B$6),$A59,"")</f>
-        <v/>
-      </c>
-      <c r="H59" s="27" t="n">
-        <f aca="false">IF(AND(ISNUMBER(D59),D59&gt;=$B$6),$A59,"")</f>
-        <v>2000000</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="28" t="s">
+        <f aca="false">IF(AND(ISNUMBER(D58),D58&gt;=$B$6),ROUND(D$19*$A58,0),"")</f>
+        <v>2327203</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="28" t="s">
         <v>77</v>
       </c>
+      <c r="B60" s="28"/>
+      <c r="C60" s="28"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="28"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="28"/>
       <c r="B61" s="28"/>
       <c r="C61" s="28"/>
       <c r="D61" s="28"/>
       <c r="E61" s="28"/>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="28"/>
-      <c r="B62" s="28"/>
-      <c r="C62" s="28"/>
-      <c r="D62" s="28"/>
-      <c r="E62" s="28"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="A61:E62"/>
+    <mergeCell ref="A60:E61"/>
   </mergeCells>
-  <conditionalFormatting sqref="B52:D59">
+  <conditionalFormatting sqref="B52:D58">
     <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$B$6</formula>
     </cfRule>
@@ -1879,11 +1851,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37:D37">
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>LEFT(B37,2)="SÍ"</formula>
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"SÍ, cabe"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>LEFT(B37,2)="NO"</formula>
+    <cfRule type="cellIs" priority="6" operator="notEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>"SÍ, cabe"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:D26">

</xml_diff>